<commit_message>
Plan, journal et passation du 06/10/2026 : lots 41 a 52
Plan : 18 sections, 81 chantiers, 67 termines, 4 a faire (deploiement et
Comptaflow), 2 a trancher (8.4 avoir de BAPA, 15.3 livraison). Deux
sections nouvelles : 17 (les achats DGI passent en ecriture, regle du
proprietaire du 06/10) et 18 (trouve en chemin). La regle 16.1 est
marquee remplacee. La passation est exceptee de la regle *.txt du
.gitignore, comme la precedente.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016zCj94qD9bq3uu6YkNwL4n
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -134,7 +133,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -147,11 +146,26 @@
         <color rgb="FFD8DCE3"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD8DCE3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="FFD8DCE3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -195,7 +209,7 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -206,6 +220,13 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -572,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -647,25 +668,25 @@
           <t>1. NAVIGATION — à traiter en premier</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="16" t="inlineStr">
         <is>
           <t>Terminée</t>
         </is>
@@ -677,25 +698,25 @@
           <t>2. COMPTABILITÉ — le principe : Selflow facture, Comptaflow tient les livres</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="16" t="inlineStr">
         <is>
           <t>Terminée</t>
         </is>
@@ -707,27 +728,27 @@
           <t>3. COMPTABILITÉ ÉTEINTE — ce qui disparaît des écrans courants</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>0/6</t>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -737,25 +758,25 @@
           <t>4. MOYENS DE PAIEMENT — ce qui remplace les codes journaux</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="15" t="n">
         <v>28</v>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>Terminée</t>
         </is>
@@ -767,27 +788,27 @@
           <t>5. LES ÉCRITURES TOURNENT MÊME QUAND LA COMPTABILITÉ EST ÉTEINTE</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="15" t="n">
         <v>34</v>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G9" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>0/2</t>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -797,27 +818,27 @@
           <t>6. CONFIGURATION GLOBALE — saisir les comptes une fois, et non par produit</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="15" t="n">
         <v>38</v>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" s="6" t="n">
+      <c r="F10" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="G10" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>0/5</t>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -827,27 +848,27 @@
           <t>7. DÉVERSEMENT COMPTAFLOW — les lignes arrivaient déséquilibrées</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="15" t="n">
         <v>45</v>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D11" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F11" s="6" t="n">
+      <c r="G11" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>0/5</t>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>4/5</t>
         </is>
       </c>
     </row>
@@ -857,27 +878,27 @@
           <t>8. AVOIRS — un avoir ne peut pas dépasser la facture (image 4)</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="15" t="n">
         <v>52</v>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>0/4</t>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>3/4</t>
         </is>
       </c>
     </row>
@@ -887,27 +908,27 @@
           <t>9. ÉCRANS D'ENTRÉE — inscription, point de vente, visite guidée</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>0/4</t>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -917,27 +938,27 @@
           <t>10. PARAMÈTRES — le compte sur la plateforme FNE</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F14" s="6" t="n">
+      <c r="F14" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G14" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>0/6</t>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -947,27 +968,27 @@
           <t>11. MODÈLES D'IMPORT — refléter exactement les champs de la plateforme</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="15" t="n">
         <v>72</v>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D15" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>0/4</t>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -977,27 +998,27 @@
           <t>12. PERFORMANCE — l'application est lente</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B16" s="15" t="n">
         <v>78</v>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F16" s="6" t="n">
+      <c r="F16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>0/4</t>
+      <c r="H16" s="16" t="inlineStr">
+        <is>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -1007,27 +1028,27 @@
           <t>13. CONDUITE DU CHANTIER</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B17" s="15" t="n">
         <v>84</v>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D17" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17" s="6" t="n">
+      <c r="F17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>0/4</t>
+      <c r="G17" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -1037,25 +1058,25 @@
           <t>14. TROUVÉ EN CHEMIN — relevé pendant le chantier 1, le 02/10/2026</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n">
+      <c r="B18" s="15" t="n">
         <v>89</v>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="E18" s="6" t="n">
+      <c r="E18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>Terminée</t>
         </is>
@@ -1067,25 +1088,25 @@
           <t>15. LA LIVRAISON — relevé le 05/10/2026</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B19" s="15" t="n">
         <v>94</v>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="D19" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="E19" s="6" t="n">
+      <c r="E19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="F19" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="H19" s="18" t="inlineStr">
         <is>
           <t>3/4</t>
         </is>
@@ -1097,50 +1118,110 @@
           <t>16. LES ÉCRITURES D'ACHAT VENUES DE LA DGI — règles en vigueur</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n">
+      <c r="B20" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="6" t="n">
+      <c r="E20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="6" t="n">
+      <c r="F20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="G20" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>Terminée</t>
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>17. LES ACHATS DGI PASSENT EN ÉCRITURE — règle du propriétaire, 06/10/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>105</v>
+      </c>
+      <c r="C21" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+    </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>18. TROUVÉ EN CHEMIN — 06/10/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="n">
+        <v>112</v>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C22" s="10" t="n">
-        <v>71</v>
-      </c>
-      <c r="D22" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="E22" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="F22" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="10" t="n">
-        <v>5</v>
+      <c r="C23" s="10" t="n">
+        <v>81</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>67</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1154,7 +1235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1181,6 +1262,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1229,13 +1311,13 @@
           <t>1. NAVIGATION — à traiter en premier</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n"/>
-      <c r="C5" s="13" t="n"/>
-      <c r="D5" s="13" t="n"/>
-      <c r="E5" s="13" t="n"/>
-      <c r="F5" s="13" t="n"/>
-      <c r="G5" s="13" t="n"/>
-      <c r="H5" s="13" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="21" t="n"/>
+      <c r="H5" s="21" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
@@ -1263,10 +1345,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F6" s="17" t="n">
+      <c r="F6" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G6" s="17" t="n">
+      <c r="G6" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H6" s="15" t="inlineStr">
@@ -1301,10 +1383,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F7" s="17" t="n">
+      <c r="F7" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G7" s="17" t="n">
+      <c r="G7" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H7" s="15" t="inlineStr">
@@ -1339,10 +1421,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F8" s="17" t="n">
+      <c r="F8" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H8" s="15" t="inlineStr">
@@ -1377,10 +1459,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F9" s="17" t="n">
+      <c r="F9" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G9" s="17" t="n">
+      <c r="G9" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H9" s="15" t="inlineStr">
@@ -1389,19 +1471,20 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
           <t>2. COMPTABILITÉ — le principe : Selflow facture, Comptaflow tient les livres</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="13" t="n"/>
-      <c r="H11" s="13" t="n"/>
+      <c r="B11" s="21" t="n"/>
+      <c r="C11" s="21" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="21" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -1429,10 +1512,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F12" s="17" t="n">
+      <c r="F12" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H12" s="15" t="inlineStr">
@@ -1467,10 +1550,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F13" s="17" t="n">
+      <c r="F13" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G13" s="17" t="n">
+      <c r="G13" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H13" s="15" t="inlineStr">
@@ -1505,10 +1588,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F14" s="17" t="n">
+      <c r="F14" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G14" s="17" t="n">
+      <c r="G14" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H14" s="15" t="inlineStr">
@@ -1543,10 +1626,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F15" s="17" t="n">
+      <c r="F15" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G15" s="17" t="n">
+      <c r="G15" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H15" s="15" t="inlineStr">
@@ -1581,10 +1664,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F16" s="17" t="n">
+      <c r="F16" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G16" s="17" t="n">
+      <c r="G16" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H16" s="15" t="inlineStr">
@@ -1619,10 +1702,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F17" s="17" t="n">
+      <c r="F17" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G17" s="17" t="n">
+      <c r="G17" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -1657,10 +1740,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F18" s="17" t="n">
+      <c r="F18" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G18" s="17" t="n">
+      <c r="G18" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H18" s="15" t="inlineStr">
@@ -1669,19 +1752,20 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
         <is>
           <t>3. COMPTABILITÉ ÉTEINTE — ce qui disparaît des écrans courants</t>
         </is>
       </c>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="13" t="n"/>
-      <c r="G20" s="13" t="n"/>
-      <c r="H20" s="13" t="n"/>
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="21" t="n"/>
+      <c r="D20" s="21" t="n"/>
+      <c r="E20" s="21" t="n"/>
+      <c r="F20" s="21" t="n"/>
+      <c r="G20" s="21" t="n"/>
+      <c r="H20" s="21" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
@@ -1701,19 +1785,19 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>Le champ est aujourd'hui un menu déroulant obligatoire sur les quatre formulaires (création et modification, clients et fournisseurs). Il disparaît quand la comptabilité est éteinte, et la valeur par défaut — 411000 pour un client, 401000 pour un fournisseur — est posée par le serveur. Ce qui n'est plus demandé ne doit plus être accepté : un compte posté à la main ne doit pas s'écrire.</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F21" s="17" t="n">
-        <v>46302</v>
-      </c>
-      <c r="G21" s="17" t="n">
-        <v>46302</v>
+          <t>Le champ est aujourd'hui un menu déroulant obligatoire sur les quatre formulaires (création et modification, clients et fournisseurs). Il disparaît quand la comptabilité est éteinte, et la valeur par défaut — 411000 pour un client, 401000 pour un fournisseur — est posée par le serveur. Ce qui n'est plus demandé ne doit plus être accepté : un compte posté à la main ne doit pas s'écrire. FAIT LE 06/10/2026 (lot 46) : le sélecteur disparaît des quatre formulaires et des deux listes quand la comptabilité est éteinte ; le serveur pose 411000 / 401000 par ImputationService::compteDeTiers, et un compte posté à la main est ignoré. Comptabilité ouverte, le compte choisi l'emporte.</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F21" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G21" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
@@ -1739,19 +1823,19 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>C'est le seul élément comptable qui survit, parce qu'il sert au rapprochement avec Comptaflow. Il est déjà calculé (six caractères, préfixe pris sur le compte collectif) ; vérifier qu'il ne se saisit nulle part et qu'il est affiché en lecture seule.</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F22" s="17" t="n">
-        <v>46302</v>
-      </c>
-      <c r="G22" s="17" t="n">
-        <v>46302</v>
+          <t>C'est le seul élément comptable qui survit, parce qu'il sert au rapprochement avec Comptaflow. Il est déjà calculé (six caractères, préfixe pris sur le compte collectif) ; vérifier qu'il ne se saisit nulle part et qu'il est affiché en lecture seule. VÉRIFIÉ LE 06/10/2026 (lot 46) : aucun formulaire ne porte de champ `numero_tiers` ; il est fabriqué par NumerotationTiersService et affiché en lecture seule. Une épreuve le vérifie à la création d'un fournisseur.</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G22" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H22" s="15" t="inlineStr">
         <is>
@@ -1777,19 +1861,19 @@
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>Deux menus obligatoires sur la création, la modification en ligne et la fiche. Ils disparaissent quand la comptabilité est éteinte ; le serveur pose 701000 et 601000. Quand elle est allumée, ils ne reviennent pas tels quels : voir le chantier 6 (configuration globale).</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F23" s="17" t="n">
-        <v>46302</v>
-      </c>
-      <c r="G23" s="17" t="n">
-        <v>46302</v>
+          <t>Deux menus obligatoires sur la création, la modification en ligne et la fiche. Ils disparaissent quand la comptabilité est éteinte ; le serveur pose 701000 et 601000. Quand elle est allumée, ils ne reviennent pas tels quels : voir le chantier 6 (configuration globale). FAIT LE 06/10/2026 (lot 46) : les deux menus disparaissent de la création, de la modification en ligne et de la fiche. Un article neuf prend le compte de sa famille, sinon 701000 / 601000 ; un article existant garde les siens. La colonne n'accepte pas le vide, et son défaut historique 701100 est la ventilation géographique que la section 5 bis du journal juge fausse.</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F23" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G23" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H23" s="15" t="inlineStr">
         <is>
@@ -1815,19 +1899,19 @@
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>Le parcours affiche aujourd'hui le compte réel à côté de chaque libellé de famille (« Vivres et alimentation (311100) »). Le numéro disparaît de l'affichage quand la comptabilité est éteinte — le préparamétrage, lui, continue de se poser en base.</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F24" s="17" t="n">
-        <v>46302</v>
-      </c>
-      <c r="G24" s="17" t="n">
-        <v>46302</v>
+          <t>Le parcours affiche aujourd'hui le compte réel à côté de chaque libellé de famille (« Vivres et alimentation (311100) »). Le numéro disparaît de l'affichage quand la comptabilité est éteinte — le préparamétrage, lui, continue de se poser en base. FAIT LE 06/10/2026 (lot 46) : l'étape « Vos rayons » ne montre plus le numéro ni l'intitulé du compte, seulement le type d'article ; le préparamétrage se pose en base comme avant.</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G24" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H24" s="15" t="inlineStr">
         <is>
@@ -1853,19 +1937,19 @@
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>L'étape 3 présente « Ce que votre métier demande » avec des cases cochées pour des modules déjà actifs, et annonce qu'ils vont être activés. Ils le sont déjà. Un module en place est montré comme acquis, non comme un choix à refaire ; si tous le sont, l'étape se saute d'elle-même en l'annonçant.</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F25" s="17" t="n">
-        <v>46302</v>
-      </c>
-      <c r="G25" s="17" t="n">
-        <v>46302</v>
+          <t>L'étape 3 présente « Ce que votre métier demande » avec des cases cochées pour des modules déjà actifs, et annonce qu'ils vont être activés. Ils le sont déjà. Un module en place est montré comme acquis, non comme un choix à refaire ; si tous le sont, l'étape se saute d'elle-même en l'annonçant. FAIT LE 06/10/2026 (lot 46) : un module déjà ouvert se montre « déjà ouvert », coché et figé ; quand tous le sont, l'étape l'annonce — « rien à choisir ici ». Une entreprise neuve naît avec tous ses modules ouverts : ils ne se décochent donc plus au parcours, mais depuis les paramètres.</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G25" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H25" s="15" t="inlineStr">
         <is>
@@ -1891,19 +1975,19 @@
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>Comptabilité éteinte = aucun écran, aucun champ, aucun lien comptable. Une épreuve parcourt les routes et les vues pour l'établir, plutôt qu'une relecture à l'œil.</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F26" s="17" t="n">
-        <v>46302</v>
-      </c>
-      <c r="G26" s="17" t="n">
-        <v>46302</v>
+          <t>Comptabilité éteinte = aucun écran, aucun champ, aucun lien comptable. Une épreuve parcourt les routes et les vues pour l'établir, plutôt qu'une relecture à l'œil. FAIT LE 06/10/2026 (lot 46) : ComptabiliteEteinteEcransTest parcourt clients, fournisseurs, catalogue et fiche produit, et vérifie qu'aucune marque comptable n'y subsiste.</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F26" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G26" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H26" s="15" t="inlineStr">
         <is>
@@ -1911,19 +1995,20 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="12" t="inlineStr">
         <is>
           <t>4. MOYENS DE PAIEMENT — ce qui remplace les codes journaux</t>
         </is>
       </c>
-      <c r="B28" s="13" t="n"/>
-      <c r="C28" s="13" t="n"/>
-      <c r="D28" s="13" t="n"/>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="13" t="n"/>
-      <c r="G28" s="13" t="n"/>
-      <c r="H28" s="13" t="n"/>
+      <c r="B28" s="21" t="n"/>
+      <c r="C28" s="21" t="n"/>
+      <c r="D28" s="21" t="n"/>
+      <c r="E28" s="21" t="n"/>
+      <c r="F28" s="21" t="n"/>
+      <c r="G28" s="21" t="n"/>
+      <c r="H28" s="21" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
@@ -1951,10 +2036,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F29" s="17" t="n">
+      <c r="F29" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G29" s="17" t="n">
+      <c r="G29" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H29" s="15" t="inlineStr">
@@ -1989,10 +2074,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F30" s="17" t="n">
+      <c r="F30" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G30" s="17" t="n">
+      <c r="G30" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H30" s="15" t="inlineStr">
@@ -2027,10 +2112,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F31" s="17" t="n">
+      <c r="F31" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G31" s="17" t="n">
+      <c r="G31" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H31" s="15" t="inlineStr">
@@ -2065,10 +2150,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F32" s="17" t="n">
+      <c r="F32" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G32" s="17" t="n">
+      <c r="G32" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H32" s="15" t="inlineStr">
@@ -2077,19 +2162,20 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="12" t="inlineStr">
         <is>
           <t>5. LES ÉCRITURES TOURNENT MÊME QUAND LA COMPTABILITÉ EST ÉTEINTE</t>
         </is>
       </c>
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="13" t="n"/>
-      <c r="D34" s="13" t="n"/>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="13" t="n"/>
-      <c r="G34" s="13" t="n"/>
-      <c r="H34" s="13" t="n"/>
+      <c r="B34" s="21" t="n"/>
+      <c r="C34" s="21" t="n"/>
+      <c r="D34" s="21" t="n"/>
+      <c r="E34" s="21" t="n"/>
+      <c r="F34" s="21" t="n"/>
+      <c r="G34" s="21" t="n"/>
+      <c r="H34" s="21" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
@@ -2109,19 +2195,19 @@
       </c>
       <c r="D35" s="14" t="inlineStr">
         <is>
-          <t>Vente, achat, avoir, règlement : chaque événement continue de produire son écriture et de l'enregistrer, comptabilité activée ou non. C'est ce qui permet d'allumer la comptabilité six mois plus tard et d'avoir les livres complets — et c'est ce que Comptaflow reçoit. La page « Opération &amp; écriture globale » reste alimentée ; elle est seulement masquée.</t>
-        </is>
-      </c>
-      <c r="E35" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F35" s="17" t="n">
-        <v>46304</v>
-      </c>
-      <c r="G35" s="17" t="n">
-        <v>46304</v>
+          <t>Vente, achat, avoir, règlement : chaque événement continue de produire son écriture et de l'enregistrer, comptabilité activée ou non. C'est ce qui permet d'allumer la comptabilité six mois plus tard et d'avoir les livres complets — et c'est ce que Comptaflow reçoit. La page « Opération &amp; écriture globale » reste alimentée ; elle est seulement masquée. VÉRIFIÉ LE 06/10/2026 : le middleware ne connaît ni les écritures ni le service qui les pose (épreuve du lot 39). Les factures reçues de la DGI passent elles aussi en écriture, comptabilité ouverte ou non (lot 42).</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F35" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G35" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H35" s="15" t="inlineStr">
         <is>
@@ -2147,19 +2233,19 @@
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
-          <t>Quand l'utilisateur ne voit aucun champ de compte, le serveur doit en choisir un qui tienne. ORDRE DE PRIORITÉ, écrit une fois dans un service et non recopié sur chaque écran : (1) exception portée par le produit ; (2) configuration globale (chantier 6) ; (3) compte de la famille ; (4) défaut 701000 à la vente, 601000 à l'achat. ET LES TIERS, ajoutés le 05/10/2026 à la demande du propriétaire : le client porte 411000, le fournisseur 401000 — le compte collectif de sa nature. Les oublier laisserait chaque écriture de vente ou d'achat sans contrepartie de tiers, et c'est précisément ce que le numéro de tiers sert à subdiviser chez Comptaflow.</t>
-        </is>
-      </c>
-      <c r="E36" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F36" s="17" t="n">
-        <v>46304</v>
-      </c>
-      <c r="G36" s="17" t="n">
-        <v>46304</v>
+          <t>Quand l'utilisateur ne voit aucun champ de compte, le serveur doit en choisir un qui tienne. ORDRE DE PRIORITÉ, écrit une fois dans un service et non recopié sur chaque écran : (1) exception portée par le produit ; (2) configuration globale (chantier 6) ; (3) compte de la famille ; (4) défaut 701000 à la vente, 601000 à l'achat. ET LES TIERS, ajoutés le 05/10/2026 à la demande du propriétaire : le client porte 411000, le fournisseur 401000 — le compte collectif de sa nature. Les oublier laisserait chaque écriture de vente ou d'achat sans contrepartie de tiers, et c'est précisément ce que le numéro de tiers sert à subdiviser chez Comptaflow. FAIT LE 06/10/2026 (lots 46 et 49) : l'ordre est écrit une fois dans ImputationService — exception de l'article (un compte propre qui diffère du défaut et de sa famille), configuration globale (type, catégorie, général), compte de l'article ou de sa famille, défaut. Les tiers : compteDeTiers() pose 411000 / 401000. Sans configuration globale, le résultat est exactement celui d'avant.</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F36" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G36" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H36" s="15" t="inlineStr">
         <is>
@@ -2167,19 +2253,20 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
         <is>
           <t>6. CONFIGURATION GLOBALE — saisir les comptes une fois, et non par produit</t>
         </is>
       </c>
-      <c r="B38" s="13" t="n"/>
-      <c r="C38" s="13" t="n"/>
-      <c r="D38" s="13" t="n"/>
-      <c r="E38" s="13" t="n"/>
-      <c r="F38" s="13" t="n"/>
-      <c r="G38" s="13" t="n"/>
-      <c r="H38" s="13" t="n"/>
+      <c r="B38" s="21" t="n"/>
+      <c r="C38" s="21" t="n"/>
+      <c r="D38" s="21" t="n"/>
+      <c r="E38" s="21" t="n"/>
+      <c r="F38" s="21" t="n"/>
+      <c r="G38" s="21" t="n"/>
+      <c r="H38" s="21" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
@@ -2199,19 +2286,19 @@
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>Une page unique qui remplace la saisie d'un compte sur chaque fiche produit. Deux sections : configuration vente, configuration achat.</t>
-        </is>
-      </c>
-      <c r="E39" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F39" s="17" t="n">
-        <v>46307</v>
-      </c>
-      <c r="G39" s="17" t="n">
-        <v>46307</v>
+          <t>Une page unique qui remplace la saisie d'un compte sur chaque fiche produit. Deux sections : configuration vente, configuration achat. FAIT LE 06/10/2026 (lot 49) : « Configuration des comptes », au menu Comptabilité, derrière le garde-fou `comptabilite` (404 quand elle est éteinte).</t>
+        </is>
+      </c>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F39" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G39" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H39" s="15" t="inlineStr">
         <is>
@@ -2237,19 +2324,19 @@
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>(1) Configuration générale — deux champs : le compte de vente de tous les produits, le compte d'achat de tous les produits. (2) Configuration par catégorie — un couple de champs par catégorie. (3) Configuration par type — un couple par type (stockable, service, …). Le plus précis l'emporte : type, puis catégorie, puis général.</t>
-        </is>
-      </c>
-      <c r="E40" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F40" s="17" t="n">
-        <v>46307</v>
-      </c>
-      <c r="G40" s="17" t="n">
-        <v>46308</v>
+          <t>(1) Configuration générale — deux champs : le compte de vente de tous les produits, le compte d'achat de tous les produits. (2) Configuration par catégorie — un couple de champs par catégorie. (3) Configuration par type — un couple par type (stockable, service, …). Le plus précis l'emporte : type, puis catégorie, puis général. FAIT LE 06/10/2026 (lot 49) : vente et achat, trois boutons chacune — générale, par catégorie, par type. Le plus précis l'emporte. Une catégorie d'une autre entreprise est ignorée ; deux champs vides retirent la ligne.</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F40" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G40" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H40" s="15" t="inlineStr">
         <is>
@@ -2275,19 +2362,19 @@
       </c>
       <c r="D41" s="14" t="inlineStr">
         <is>
-          <t>Les comptes de variation (6031/6032/6033, 736) et de stock (31/32/33/36) sont posés par le système. Une section les affiche : ce qui est fait, avec quels comptes, et permet de les changer. Rien n'est demandé — c'est une lecture qui accepte une correction.</t>
-        </is>
-      </c>
-      <c r="E41" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F41" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="G41" s="17" t="n">
-        <v>46308</v>
+          <t>Les comptes de variation (6031/6032/6033, 736) et de stock (31/32/33/36) sont posés par le système. Une section les affiche : ce qui est fait, avec quels comptes, et permet de les changer. Rien n'est demandé — c'est une lecture qui accepte une correction. FAIT LE 06/10/2026 (lot 49) : section « Variations de stock » — les comptes de stock et de variation de chaque famille s'y lisent et s'y corrigent (classe 3, 603x/73x).</t>
+        </is>
+      </c>
+      <c r="E41" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F41" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G41" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H41" s="15" t="inlineStr">
         <is>
@@ -2313,19 +2400,19 @@
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>Dès que la configuration globale est renseignée, la fiche produit n'affiche plus de champ de compte mais la mention « hérite de la configuration globale », avec les comptes qui s'appliquent. Une case à cocher ouvre deux champs (vente, achat) : cochée, elle PRIME sur la configuration globale, parce qu'elle est portée par le produit lui-même. Décochée, le produit revient à l'héritage — et ne garde pas en silence l'ancienne valeur.</t>
-        </is>
-      </c>
-      <c r="E42" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F42" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="G42" s="17" t="n">
-        <v>46308</v>
+          <t>Dès que la configuration globale est renseignée, la fiche produit n'affiche plus de champ de compte mais la mention « hérite de la configuration globale », avec les comptes qui s'appliquent. Une case à cocher ouvre deux champs (vente, achat) : cochée, elle PRIME sur la configuration globale, parce qu'elle est portée par le produit lui-même. Décochée, le produit revient à l'héritage — et ne garde pas en silence l'ancienne valeur. FAIT LE 06/10/2026 (lot 49) : la fiche (et la modification en ligne) dit « Hérite de la configuration globale : vente …, achat … » ; la case ouvre deux champs qui priment. Décochée, le serveur repose le compte hérité.</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F42" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G42" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H42" s="15" t="inlineStr">
         <is>
@@ -2351,19 +2438,19 @@
       </c>
       <c r="D43" s="14" t="inlineStr">
         <is>
-          <t>Les produits portent déjà des comptes. Ceux qui diffèrent du défaut (701000 / 601000) sont réputés voulus : ils basculent en exception cochée. Les autres passent en héritage. Sans cette règle, l'arrivée de la configuration globale réécrirait des imputations choisies.</t>
-        </is>
-      </c>
-      <c r="E43" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F43" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="G43" s="17" t="n">
-        <v>46308</v>
+          <t>Les produits portent déjà des comptes. Ceux qui diffèrent du défaut (701000 / 601000) sont réputés voulus : ils basculent en exception cochée. Les autres passent en héritage. Sans cette règle, l'arrivée de la configuration globale réécrirait des imputations choisies. FAIT LE 06/10/2026 (lot 49), sans migration : la règle s'applique à chaque lecture — un compte qui diffère du défaut ET de la famille est réputé voulu (exception). Affinage : comparer aussi à la famille, sans quoi un service sur 706000 serait passé pour une exception alors qu'il hérite de son rayon.</t>
+        </is>
+      </c>
+      <c r="E43" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F43" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G43" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H43" s="15" t="inlineStr">
         <is>
@@ -2371,19 +2458,20 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="12" t="inlineStr">
         <is>
           <t>7. DÉVERSEMENT COMPTAFLOW — les lignes arrivaient déséquilibrées</t>
         </is>
       </c>
-      <c r="B45" s="13" t="n"/>
-      <c r="C45" s="13" t="n"/>
-      <c r="D45" s="13" t="n"/>
-      <c r="E45" s="13" t="n"/>
-      <c r="F45" s="13" t="n"/>
-      <c r="G45" s="13" t="n"/>
-      <c r="H45" s="13" t="n"/>
+      <c r="B45" s="21" t="n"/>
+      <c r="C45" s="21" t="n"/>
+      <c r="D45" s="21" t="n"/>
+      <c r="E45" s="21" t="n"/>
+      <c r="F45" s="21" t="n"/>
+      <c r="G45" s="21" t="n"/>
+      <c r="H45" s="21" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
@@ -2403,19 +2491,19 @@
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>DIAGNOSTIC POSÉ : `DeverserOperationComptaflow::ligne()` envoie `compte_debit`, `compte_credit`, `debit` et `credit` sur UNE SEULE ligne. C'est le modèle interne de Selflow ; Comptaflow attend une ligne par mouvement de compte. D'où la ligne unique par numéro de saisie et la balance qui ne tombe pas. PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : ce n'est PAS un simple dédoublement. Une vente avec TVA, timbre et remise fait plus de deux lignes, un règlement partiel aussi. Le déversement doit porter l'opération ENTIÈRE, et ses lignes doivent se retrouver groupées par leur référence — le numéro de saisie. C'est lui qui fait le couple, pas la position dans la liste.</t>
-        </is>
-      </c>
-      <c r="E46" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F46" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G46" s="17" t="n">
-        <v>46309</v>
+          <t>DIAGNOSTIC POSÉ : `DeverserOperationComptaflow::ligne()` envoie `compte_debit`, `compte_credit`, `debit` et `credit` sur UNE SEULE ligne. C'est le modèle interne de Selflow ; Comptaflow attend une ligne par mouvement de compte. D'où la ligne unique par numéro de saisie et la balance qui ne tombe pas. PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : ce n'est PAS un simple dédoublement. Une vente avec TVA, timbre et remise fait plus de deux lignes, un règlement partiel aussi. Le déversement doit porter l'opération ENTIÈRE, et ses lignes doivent se retrouver groupées par leur référence — le numéro de saisie. C'est lui qui fait le couple, pas la position dans la liste. TROUVÉ ET CORRIGÉ LE 06/10/2026 (lot 44, et commit associé sur guysergekouassi/COMPTAFLOW, même branche) : chaque ligne Selflow porte déjà un seul mouvement ; c'est COMPTAFLOW qui rangeait `cle_selflow` — l'identité d'une LIGNE — dans `n_saisie`, si bien que chaque ligne devenait sa propre pièce. Chaque ligne porte désormais `operation_selflow` (SELFLOW-{entreprise}-OP{n° de saisie}) ; Comptaflow donne un numéro de saisie commun à toutes les lignes d'une opération, à la convention du dossier.</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F46" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G46" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H46" s="15" t="inlineStr">
         <is>
@@ -2441,19 +2529,19 @@
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>Relire ce que Comptaflow attend — nom des champs, sens du montant, journal, date, pièce, numéro de tiers, exercice — et s'y conformer sans rien lui dicter. Selflow envoie ; Comptaflow décide.</t>
-        </is>
-      </c>
-      <c r="E47" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F47" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G47" s="17" t="n">
-        <v>46309</v>
+          <t>Relire ce que Comptaflow attend — nom des champs, sens du montant, journal, date, pièce, numéro de tiers, exercice — et s'y conformer sans rien lui dicter. Selflow envoie ; Comptaflow décide. FAIT LE 06/10/2026 : contrat relu dans ExternalSyncController::deverserEcritures — champs, sens, journal (UniformisationImport), exercice comparé, tiers, clé d'idempotence ; seul le numéro de saisie était faux. Comptaflow décide toujours : il attribue le numéro à sa convention.</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F47" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G47" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H47" s="15" t="inlineStr">
         <is>
@@ -2479,19 +2567,19 @@
       </c>
       <c r="D48" s="14" t="inlineStr">
         <is>
-          <t>Somme des débits = somme des crédits, vérifiée avant l'envoi. Une opération qui ne tombe pas n'est pas envoyée : elle est signalée. Déverser un déséquilibre oblige à le chercher dans l'autre application, où l'on n'a pas la pièce d'origine.</t>
-        </is>
-      </c>
-      <c r="E48" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F48" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G48" s="17" t="n">
-        <v>46309</v>
+          <t>Somme des débits = somme des crédits, vérifiée avant l'envoi. Une opération qui ne tombe pas n'est pas envoyée : elle est signalée. Déverser un déséquilibre oblige à le chercher dans l'autre application, où l'on n'a pas la pièce d'origine. FAIT LE 06/10/2026 (lot 44) : l'équilibre se recompte au départ sur les lignes telles qu'elles sont, en plus du drapeau posé à la clôture ; une opération qui ne tombe pas ne part pas et se journalise.</t>
+        </is>
+      </c>
+      <c r="E48" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F48" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G48" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H48" s="15" t="inlineStr">
         <is>
@@ -2517,19 +2605,19 @@
       </c>
       <c r="D49" s="14" t="inlineStr">
         <is>
-          <t>Les opérations déjà déversées sous l'ancienne forme sont à rejouer. Vérifier que le déversement est idempotent côté Comptaflow AVANT de rejouer quoi que ce soit — sinon la balance double.</t>
-        </is>
-      </c>
-      <c r="E49" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F49" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G49" s="17" t="n">
-        <v>46310</v>
+          <t>Les opérations déjà déversées sous l'ancienne forme sont à rejouer. Vérifier que le déversement est idempotent côté Comptaflow AVANT de rejouer quoi que ce soit — sinon la balance double. FAIT LE 06/10/2026 : idempotence vérifiée AVANT — chaque ligne est reconnue à sa clé, donc rejouer le déversement ne changerait rien. D'où `selflow:regrouper-comptaflow`, qui n'envoie aucune écriture : il dit quelles lignes forment quelle opération, et POST /api/external/ecritures/regrouper leur donne un numéro commun — seulement si l'opération est complète et équilibrée. Idempotent, épreuves des deux côtés.</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F49" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G49" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H49" s="15" t="inlineStr">
         <is>
@@ -2555,7 +2643,7 @@
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>Une vente, un achat, un avoir, un règlement — puis relire la balance chez Comptaflow. La vérification se fait sur la plateforme, pas seulement sur les épreuves.</t>
+          <t>Une vente, un achat, un avoir, un règlement — puis relire la balance chez Comptaflow. La vérification se fait sur la plateforme, pas seulement sur les épreuves. ÉTAT AU 06/10/2026 : à faire par le propriétaire après le déploiement conjoint (Selflow + Comptaflow, migrations comprises) : lancer `php artisan selflow:regrouper-comptaflow`, puis une vente, un achat, un avoir et un règlement, et relire la balance par pièce chez Comptaflow.</t>
         </is>
       </c>
       <c r="E50" s="18" t="inlineStr">
@@ -2563,10 +2651,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F50" s="17" t="n">
+      <c r="F50" s="22" t="n">
         <v>46310</v>
       </c>
-      <c r="G50" s="17" t="n">
+      <c r="G50" s="22" t="n">
         <v>46310</v>
       </c>
       <c r="H50" s="15" t="inlineStr">
@@ -2575,19 +2663,20 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="12" t="inlineStr">
         <is>
           <t>8. AVOIRS — un avoir ne peut pas dépasser la facture (image 4)</t>
         </is>
       </c>
-      <c r="B52" s="13" t="n"/>
-      <c r="C52" s="13" t="n"/>
-      <c r="D52" s="13" t="n"/>
-      <c r="E52" s="13" t="n"/>
-      <c r="F52" s="13" t="n"/>
-      <c r="G52" s="13" t="n"/>
-      <c r="H52" s="13" t="n"/>
+      <c r="B52" s="21" t="n"/>
+      <c r="C52" s="21" t="n"/>
+      <c r="D52" s="21" t="n"/>
+      <c r="E52" s="21" t="n"/>
+      <c r="F52" s="21" t="n"/>
+      <c r="G52" s="21" t="n"/>
+      <c r="H52" s="21" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
@@ -2607,19 +2696,19 @@
       </c>
       <c r="D53" s="14" t="inlineStr">
         <is>
-          <t>RÉPONSE À VOTRE QUESTION : non, un avoir ne doit pas pouvoir dépasser la valeur de la pièce d'origine — cela reviendrait à rendre plus que ce qui a été facturé, et la TVA collectée deviendrait négative sur la pièce. Contrôle au serveur, pas seulement à l'écran : somme des avoirs déjà établis + avoir en cours ≤ total de la facture. VALIDÉ par le propriétaire le 2 octobre 2026.</t>
-        </is>
-      </c>
-      <c r="E53" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F53" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="G53" s="17" t="n">
-        <v>46311</v>
+          <t>RÉPONSE À VOTRE QUESTION : non, un avoir ne doit pas pouvoir dépasser la valeur de la pièce d'origine — cela reviendrait à rendre plus que ce qui a été facturé, et la TVA collectée deviendrait négative sur la pièce. Contrôle au serveur, pas seulement à l'écran : somme des avoirs déjà établis + avoir en cours ≤ total de la facture. VALIDÉ par le propriétaire le 2 octobre 2026. FAIT LE 06/10/2026 (lot 45) : le plafond ne tenait qu'en quantité — le prix unitaire de la modale restait libre et une ligne ajoutée n'avait pas de plafond. Le TTC de l'avoir est confronté au reste à avoirer, au serveur, dans la transaction (tolérance d'un franc). L'avoir total est refusé sur une facture déjà entamée.</t>
+        </is>
+      </c>
+      <c r="E53" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F53" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G53" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H53" s="15" t="inlineStr">
         <is>
@@ -2645,19 +2734,19 @@
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
-          <t>Une facture entièrement avoirée n'a plus rien à rendre : elle sort de la liste déroulante et du champ de recherche. La proposer mène à un refus qu'on ne comprend qu'après coup.</t>
-        </is>
-      </c>
-      <c r="E54" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F54" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="G54" s="17" t="n">
-        <v>46311</v>
+          <t>Une facture entièrement avoirée n'a plus rien à rendre : elle sort de la liste déroulante et du champ de recherche. La proposer mène à un refus qu'on ne comprend qu'après coup. FAIT LE 06/10/2026 (lot 45) : une portée unique Vente::avoirables() pour la liste déroulante et le champ de recherche, qui portaient chacun leur copie de la requête.</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F54" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G54" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H54" s="15" t="inlineStr">
         <is>
@@ -2683,19 +2772,19 @@
       </c>
       <c r="D55" s="14" t="inlineStr">
         <is>
-          <t>Celles qui portent déjà un avoir sans atteindre le total restent proposées, avec la mention du reste à avoirer — « reste 45 000 F sur 120 000 F ». Sans cette mention, on saisit un montant au jugé et on se fait refuser.</t>
-        </is>
-      </c>
-      <c r="E55" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F55" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="G55" s="17" t="n">
-        <v>46311</v>
+          <t>Celles qui portent déjà un avoir sans atteindre le total restent proposées, avec la mention du reste à avoirer — « reste 45 000 F sur 120 000 F ». Sans cette mention, on saisit un montant au jugé et on se fait refuser. FAIT LE 06/10/2026 (lot 45) : « VTE-… - Client (reste 7 080 F sur 11 800 F) ».</t>
+        </is>
+      </c>
+      <c r="E55" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F55" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G55" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H55" s="15" t="inlineStr">
         <is>
@@ -2721,18 +2810,18 @@
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : l'avoir fournisseur ne concerne QUE les BAPA — les bordereaux d'achat auprès d'un particulier, que Selflow émet et que la DGI certifie. Un achat ordinaire est une pièce du fournisseur, pas de nous : on ne l'avoire pas, on demande au fournisseur son propre avoir. Le contrôle de dépassement s'applique donc au BAPA, et l'écran ne doit pas proposer d'avoir sur les autres achats.</t>
-        </is>
-      </c>
-      <c r="E56" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F56" s="17" t="n">
+          <t>PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : l'avoir fournisseur ne concerne QUE les BAPA — les bordereaux d'achat auprès d'un particulier, que Selflow émet et que la DGI certifie. Un achat ordinaire est une pièce du fournisseur, pas de nous : on ne l'avoire pas, on demande au fournisseur son propre avoir. Le contrôle de dépassement s'applique donc au BAPA, et l'écran ne doit pas proposer d'avoir sur les autres achats. À TRANCHER, relevé le 06/10/2026 : l'avoir fournisseur a été retiré le 25/09 sur TOUS les achats, et aucun n'est proposé sur un achat ordinaire — la seconde moitié du chantier est donc acquise. Mais le BAPA porte une interdiction écrite (`Achat::estBapa()`, AVOIR_BAPA_INTERDIT) : « la DGI ne normalise pas l'avoir d'un BAPA ». Le rétablir supposerait de certifier cet avoir, donc de toucher FneService — périmètre gelé. Il faut votre décision : (a) la DGI le permet désormais — exception 1 ou 3 de CLAUDE.md, et je l'ouvre avec le plafond ; (b) un avoir de BAPA interne, non certifié, qui ne vaudrait que pour la comptabilité.</t>
+        </is>
+      </c>
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>À trancher</t>
+        </is>
+      </c>
+      <c r="F56" s="22" t="n">
         <v>46311</v>
       </c>
-      <c r="G56" s="17" t="n">
+      <c r="G56" s="22" t="n">
         <v>46311</v>
       </c>
       <c r="H56" s="15" t="inlineStr">
@@ -2741,19 +2830,20 @@
         </is>
       </c>
     </row>
+    <row r="57"/>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="12" t="inlineStr">
         <is>
           <t>9. ÉCRANS D'ENTRÉE — inscription, point de vente, visite guidée</t>
         </is>
       </c>
-      <c r="B58" s="13" t="n"/>
-      <c r="C58" s="13" t="n"/>
-      <c r="D58" s="13" t="n"/>
-      <c r="E58" s="13" t="n"/>
-      <c r="F58" s="13" t="n"/>
-      <c r="G58" s="13" t="n"/>
-      <c r="H58" s="13" t="n"/>
+      <c r="B58" s="21" t="n"/>
+      <c r="C58" s="21" t="n"/>
+      <c r="D58" s="21" t="n"/>
+      <c r="E58" s="21" t="n"/>
+      <c r="F58" s="21" t="n"/>
+      <c r="G58" s="21" t="n"/>
+      <c r="H58" s="21" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="14" t="inlineStr">
@@ -2773,19 +2863,19 @@
       </c>
       <c r="D59" s="14" t="inlineStr">
         <is>
-          <t>Les boutons « Retour », « Suivant » et « Terminer sans remplir la suite » montrent un carré vide à la place de leur icône : la police d'icônes n'est pas chargée sur la page publique, ou le glyphe n'existe pas dans la version servie. À corriger à la source — une icône absente sur la toute première page donne le ton du reste.</t>
-        </is>
-      </c>
-      <c r="E59" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F59" s="17" t="n">
-        <v>46314</v>
-      </c>
-      <c r="G59" s="17" t="n">
-        <v>46314</v>
+          <t>Les boutons « Retour », « Suivant » et « Terminer sans remplir la suite » montrent un carré vide à la place de leur icône : la police d'icônes n'est pas chargée sur la page publique, ou le glyphe n'existe pas dans la version servie. À corriger à la source — une icône absente sur la toute première page donne le ton du reste. CAUSE TROUVÉE ET CORRIGÉE LE 06/10/2026 (lot 41) : la politique de sécurité (CSP) n'autorisait pas jsdelivr dans `font-src` — la police Tabler des pages d'entrée était refusée par notre propre en-tête, d'où les carrés vides. Toutes les polices et icônes sont désormais servies par l'application (public/vendor), Tabler remplacé par Font Awesome. Vérifié au navigateur.</t>
+        </is>
+      </c>
+      <c r="E59" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F59" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G59" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H59" s="15" t="inlineStr">
         <is>
@@ -2811,19 +2901,19 @@
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
-          <t>Le champ « Mot de passe » porte un œil, « Confirmer le mot de passe » n'en a pas. Les deux doivent en porter un, et les deux doivent basculer ensemble : on compare deux saisies, on ne peut pas les comparer si une seule est lisible.</t>
-        </is>
-      </c>
-      <c r="E60" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F60" s="17" t="n">
-        <v>46314</v>
-      </c>
-      <c r="G60" s="17" t="n">
-        <v>46314</v>
+          <t>Le champ « Mot de passe » porte un œil, « Confirmer le mot de passe » n'en a pas. Les deux doivent en porter un, et les deux doivent basculer ensemble : on compare deux saisies, on ne peut pas les comparer si une seule est lisible. FAIT LE 06/10/2026 (lot 47) : un œil sur la confirmation, et les deux basculent ensemble.</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F60" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G60" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H60" s="15" t="inlineStr">
         <is>
@@ -2849,19 +2939,19 @@
       </c>
       <c r="D61" s="14" t="inlineStr">
         <is>
-          <t>Entre le clic sur « Créer » et la réponse, l'écran reste figé sans rien dire. Chercher la cause avant d'ajouter un sablier : création du stock d'ouverture pour tout le catalogue à chaque nouveau site, appel réseau synchrone, ou index manquant. Ce qui peut attendre part en file ; le bouton se désactive et annonce ce qui se passe.</t>
-        </is>
-      </c>
-      <c r="E61" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F61" s="17" t="n">
-        <v>46314</v>
-      </c>
-      <c r="G61" s="17" t="n">
-        <v>46314</v>
+          <t>Entre le clic sur « Créer » et la réponse, l'écran reste figé sans rien dire. Chercher la cause avant d'ajouter un sablier : création du stock d'ouverture pour tout le catalogue à chaque nouveau site, appel réseau synchrone, ou index manquant. Ce qui peut attendre part en file ; le bouton se désactive et annonce ce qui se passe. MESURÉ ET CORRIGÉ LE 06/10/2026 (lot 43) : c'était bien la création des fiches de stock — deux requêtes par article (firstOrCreate en boucle). 10 000 articles : 11 449 ms / 17 103 requêtes → 361 ms / 20 requêtes, par insertion groupée.</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F61" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G61" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H61" s="15" t="inlineStr">
         <is>
@@ -2887,19 +2977,19 @@
       </c>
       <c r="D62" s="14" t="inlineStr">
         <is>
-          <t>L'étape 3 sur 7 parle du catalogue alors que la section n'est pas à l'écran. La visite doit lire la barre latérale réelle — modules actifs, habilitations, comptabilité activée — et sauter ce qui n'existe pas pour cet utilisateur. À reprendre APRÈS le chantier 1 (dépliage) et le chantier 2 (masquage), qui changent tous deux ce qui est visible.</t>
-        </is>
-      </c>
-      <c r="E62" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F62" s="17" t="n">
-        <v>46315</v>
-      </c>
-      <c r="G62" s="17" t="n">
-        <v>46315</v>
+          <t>L'étape 3 sur 7 parle du catalogue alors que la section n'est pas à l'écran. La visite doit lire la barre latérale réelle — modules actifs, habilitations, comptabilité activée — et sauter ce qui n'existe pas pour cet utilisateur. À reprendre APRÈS le chantier 1 (dépliage) et le chantier 2 (masquage), qui changent tous deux ce qui est visible. FAIT LE 06/10/2026 (lot 50) : la visite filtrait déjà les cibles absentes ; le défaut venait du lot 37 — la cible était là, mais dans une section repliée. Elle ouvre d'abord la section qui la porte, sans toucher à la mémoire du menu. Vérifié au navigateur : « Votre catalogue » entoure le lien (248 × 48 px).</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F62" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G62" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H62" s="15" t="inlineStr">
         <is>
@@ -2907,19 +2997,20 @@
         </is>
       </c>
     </row>
+    <row r="63"/>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="12" t="inlineStr">
         <is>
           <t>10. PARAMÈTRES — le compte sur la plateforme FNE</t>
         </is>
       </c>
-      <c r="B64" s="13" t="n"/>
-      <c r="C64" s="13" t="n"/>
-      <c r="D64" s="13" t="n"/>
-      <c r="E64" s="13" t="n"/>
-      <c r="F64" s="13" t="n"/>
-      <c r="G64" s="13" t="n"/>
-      <c r="H64" s="13" t="n"/>
+      <c r="B64" s="21" t="n"/>
+      <c r="C64" s="21" t="n"/>
+      <c r="D64" s="21" t="n"/>
+      <c r="E64" s="21" t="n"/>
+      <c r="F64" s="21" t="n"/>
+      <c r="G64" s="21" t="n"/>
+      <c r="H64" s="21" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="14" t="inlineStr">
@@ -2939,19 +3030,19 @@
       </c>
       <c r="D65" s="14" t="inlineStr">
         <is>
-          <t>C'est la question qui commande tout le reste — ce que l'entreprise doit saisir dépend de la réponse. Elle passe donc en première position après « Votre configuration », et la barre d'ancres suit.</t>
-        </is>
-      </c>
-      <c r="E65" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F65" s="17" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G65" s="17" t="n">
-        <v>46316</v>
+          <t>C'est la question qui commande tout le reste — ce que l'entreprise doit saisir dépend de la réponse. Elle passe donc en première position après « Votre configuration », et la barre d'ancres suit. FAIT LE 06/10/2026 (lot 47) : la carte passe au-dessus de la grille, juste après « Votre configuration » ; la famille « Fiscalité &amp; DGI » ouvre la barre d'ancres.</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F65" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G65" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H65" s="15" t="inlineStr">
         <is>
@@ -2977,19 +3068,19 @@
       </c>
       <c r="D66" s="14" t="inlineStr">
         <is>
-          <t>PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026. Quand « Je n'en ai pas encore » est coché, le message ne doit lister QUE les informations fiscales réellement manquantes. Celles déjà saisies au formulaire d'inscription ne se redemandent pas : les réafficher vides ferait croire que la saisie s'est perdue, et les réafficher remplies encombre pour rien. L'écran lit ce qui est en base et se tait sur le reste.</t>
-        </is>
-      </c>
-      <c r="E66" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F66" s="17" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G66" s="17" t="n">
-        <v>46316</v>
+          <t>PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026. Quand « Je n'en ai pas encore » est coché, le message ne doit lister QUE les informations fiscales réellement manquantes. Celles déjà saisies au formulaire d'inscription ne se redemandent pas : les réafficher vides ferait croire que la saisie s'est perdue, et les réafficher remplies encombre pour rien. L'écran lit ce qui est en base et se tait sur le reste. FAIT LE 06/10/2026 (lot 47) : seules les informations manquantes sont listées ; sinon « Toutes les informations fiscales sont renseignées ».</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F66" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G66" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H66" s="15" t="inlineStr">
         <is>
@@ -3015,19 +3106,19 @@
       </c>
       <c r="D67" s="14" t="inlineStr">
         <is>
-          <t>Même règle qu'au 10.2, précisée le 05/10/2026. Les deux champs n'apparaissent que si le NCC ou le mot de passe FNE ne sont pas déjà connus. Un client dont l'inscription les a pris ne doit plus les voir — la question est réglée pour lui.</t>
-        </is>
-      </c>
-      <c r="E67" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F67" s="17" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G67" s="17" t="n">
-        <v>46316</v>
+          <t>Même règle qu'au 10.2, précisée le 05/10/2026. Les deux champs n'apparaissent que si le NCC ou le mot de passe FNE ne sont pas déjà connus. Un client dont l'inscription les a pris ne doit plus les voir — la question est réglée pour lui. FAIT LE 06/10/2026 (lot 47) : les deux champs n'apparaissent que si l'accès n'est pas connu (NCC + mot de passe fourni, ou clé déjà posée). Enregistrés par AccesFneService — chiffré, jamais rendu —, la même porte qu'à l'inscription. Périmètre FNE gelé non touché.</t>
+        </is>
+      </c>
+      <c r="E67" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F67" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G67" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H67" s="15" t="inlineStr">
         <is>
@@ -3053,19 +3144,19 @@
       </c>
       <c r="D68" s="14" t="inlineStr">
         <is>
-          <t>Établir, champ par champ, ce que le scraper ramène du portail, en regardant les quatre sections : Informations générales, DGI &amp; Local professionnel, Identité fiscale, Impression des factures. Ce qui est ramené n'est plus demandé — le champ disparaît dès que « J'ai déjà un compte FNE » est coché. Ce qui ne l'est pas est signalé comme restant à remplir. LE RELEVÉ EST À FAIRE AVANT DE RETIRER QUOI QUE CE SOIT : retirer un champ que le portail ne rend pas laisserait l'information manquante sans aucun moyen de la saisir.</t>
-        </is>
-      </c>
-      <c r="E68" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F68" s="17" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G68" s="17" t="n">
-        <v>46317</v>
+          <t>Établir, champ par champ, ce que le scraper ramène du portail, en regardant les quatre sections : Informations générales, DGI &amp; Local professionnel, Identité fiscale, Impression des factures. Ce qui est ramené n'est plus demandé — le champ disparaît dès que « J'ai déjà un compte FNE » est coché. Ce qui ne l'est pas est signalé comme restant à remplir. LE RELEVÉ EST À FAIRE AVANT DE RETIRER QUOI QUE CE SOIT : retirer un champ que le portail ne rend pas laisserait l'information manquante sans aucun moyen de la saisir. RELEVÉ FAIT LE 06/10/2026 — rien retiré. Le scraper ramène (PortailFneFiche) : email, téléphone, adresse, commune, quartier, référence cadastrale, IDU, propriétaire du local, référence bancaire, seuil de stickers, timbre de quittance, BAPA, pied de page et autres mentions. Il NE ramène PAS : la raison sociale, la forme juridique, le gérant (nom, prénom, fonction), le RCCM, le régime d'imposition, le centre des impôts (le NCC est l'identifiant de connexion). À DÉCIDER avec vous : retirer de l'écran, compte FNE coché, les champs que le relevé ramène — ils doivent alors se remplir depuis le relevé, ce qui suppose que le scraper ait tourné.</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F68" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G68" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H68" s="15" t="inlineStr">
         <is>
@@ -3091,19 +3182,19 @@
       </c>
       <c r="D69" s="14" t="inlineStr">
         <is>
-          <t>Le « Logo secondaire (FNE, certification) » doit rester affiché en toutes circonstances, y compris quand les autres champs disparaissent. Il n'est pas déposé par l'utilisateur : c'est le système qui le pose.</t>
-        </is>
-      </c>
-      <c r="E69" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F69" s="17" t="n">
-        <v>46317</v>
-      </c>
-      <c r="G69" s="17" t="n">
-        <v>46317</v>
+          <t>Le « Logo secondaire (FNE, certification) » doit rester affiché en toutes circonstances, y compris quand les autres champs disparaissent. Il n'est pas déposé par l'utilisateur : c'est le système qui le pose. FAIT LE 06/10/2026 (lot 47) : le logo FNE du système (public/logo-FNE.png) est affiché en toutes circonstances ; le dépôt d'un fichier n'est plus proposé et serait ignoré. Les documents imprimés (gelés) n'ont pas bougé.</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F69" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G69" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H69" s="15" t="inlineStr">
         <is>
@@ -3137,10 +3228,10 @@
           <t>Sans objet</t>
         </is>
       </c>
-      <c r="F70" s="17" t="n">
+      <c r="F70" s="22" t="n">
         <v>46317</v>
       </c>
-      <c r="G70" s="17" t="n">
+      <c r="G70" s="22" t="n">
         <v>46317</v>
       </c>
       <c r="H70" s="15" t="inlineStr">
@@ -3149,19 +3240,20 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="12" t="inlineStr">
         <is>
           <t>11. MODÈLES D'IMPORT — refléter exactement les champs de la plateforme</t>
         </is>
       </c>
-      <c r="B72" s="13" t="n"/>
-      <c r="C72" s="13" t="n"/>
-      <c r="D72" s="13" t="n"/>
-      <c r="E72" s="13" t="n"/>
-      <c r="F72" s="13" t="n"/>
-      <c r="G72" s="13" t="n"/>
-      <c r="H72" s="13" t="n"/>
+      <c r="B72" s="21" t="n"/>
+      <c r="C72" s="21" t="n"/>
+      <c r="D72" s="21" t="n"/>
+      <c r="E72" s="21" t="n"/>
+      <c r="F72" s="21" t="n"/>
+      <c r="G72" s="21" t="n"/>
+      <c r="H72" s="21" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="14" t="inlineStr">
@@ -3181,19 +3273,19 @@
       </c>
       <c r="D73" s="14" t="inlineStr">
         <is>
-          <t>Reprendre les sept modèles (points de vente, clients, fournisseurs, utilisateurs, articles, stock initial, immobilisations) et les confronter aux formulaires. Toute colonne qui ne correspond à aucun champ saisissable disparaît : un modèle qui promet une colonne que rien ne lit fait saisir pour rien, et laisse croire que la donnée est entrée.</t>
-        </is>
-      </c>
-      <c r="E73" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F73" s="17" t="n">
-        <v>46318</v>
-      </c>
-      <c r="G73" s="17" t="n">
-        <v>46318</v>
+          <t>Reprendre les sept modèles (points de vente, clients, fournisseurs, utilisateurs, articles, stock initial, immobilisations) et les confronter aux formulaires. Toute colonne qui ne correspond à aucun champ saisissable disparaît : un modèle qui promet une colonne que rien ne lit fait saisir pour rien, et laisse croire que la donnée est entrée. FAIT LE 06/10/2026 (lot 48) : clients, fournisseurs et articles confrontés à leurs formulaires ; les colonnes que plus rien ne saisit sont retirées.</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F73" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G73" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H73" s="15" t="inlineStr">
         <is>
@@ -3219,19 +3311,19 @@
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>Conséquence des chantiers 3.1 et 3.2 : le modèle ne doit pas demander un compte qui n'est plus proposé à l'écran, ni un numéro de tiers devenu automatique.</t>
-        </is>
-      </c>
-      <c r="E74" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F74" s="17" t="n">
-        <v>46318</v>
-      </c>
-      <c r="G74" s="17" t="n">
-        <v>46318</v>
+          <t>Conséquence des chantiers 3.1 et 3.2 : le modèle ne doit pas demander un compte qui n'est plus proposé à l'écran, ni un numéro de tiers devenu automatique. FAIT LE 06/10/2026 (lot 48) : colonnes retirées ; l'import pose le compte par compteDeTiers et fabrique le numéro, comme l'écran. Un fichier qui les porterait encore ne les impose plus.</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F74" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G74" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H74" s="15" t="inlineStr">
         <is>
@@ -3257,19 +3349,19 @@
       </c>
       <c r="D75" s="14" t="inlineStr">
         <is>
-          <t>Même raison : ils viennent de la configuration globale (chantier 6), plus d'une saisie par ligne de classeur.</t>
-        </is>
-      </c>
-      <c r="E75" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F75" s="17" t="n">
-        <v>46318</v>
-      </c>
-      <c r="G75" s="17" t="n">
-        <v>46318</v>
+          <t>Même raison : ils viennent de la configuration globale (chantier 6), plus d'une saisie par ligne de classeur. FAIT LE 06/10/2026 (lot 48) : les QUATRE comptes (vente, achat, stock, variation) quittent le modèle — aucun ne se saisit plus à l'écran. Ils viennent de la famille, puis des défauts.</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F75" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G75" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H75" s="15" t="inlineStr">
         <is>
@@ -3295,19 +3387,19 @@
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>Une épreuve qui compare les colonnes annoncées aux champs acceptés, pour que le prochain champ retiré d'un écran ne reste pas dans un modèle.</t>
-        </is>
-      </c>
-      <c r="E76" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F76" s="17" t="n">
-        <v>46318</v>
-      </c>
-      <c r="G76" s="17" t="n">
-        <v>46318</v>
+          <t>Une épreuve qui compare les colonnes annoncées aux champs acceptés, pour que le prochain champ retiré d'un écran ne reste pas dans un modèle. FAIT LE 06/10/2026 (lot 48) : ModelesImportRefletentLesFormulairesTest exige que chaque colonne des modèles clients et fournisseurs soit un champ du formulaire de création.</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F76" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G76" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H76" s="15" t="inlineStr">
         <is>
@@ -3315,19 +3407,20 @@
         </is>
       </c>
     </row>
+    <row r="77"/>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="12" t="inlineStr">
         <is>
           <t>12. PERFORMANCE — l'application est lente</t>
         </is>
       </c>
-      <c r="B78" s="13" t="n"/>
-      <c r="C78" s="13" t="n"/>
-      <c r="D78" s="13" t="n"/>
-      <c r="E78" s="13" t="n"/>
-      <c r="F78" s="13" t="n"/>
-      <c r="G78" s="13" t="n"/>
-      <c r="H78" s="13" t="n"/>
+      <c r="B78" s="21" t="n"/>
+      <c r="C78" s="21" t="n"/>
+      <c r="D78" s="21" t="n"/>
+      <c r="E78" s="21" t="n"/>
+      <c r="F78" s="21" t="n"/>
+      <c r="G78" s="21" t="n"/>
+      <c r="H78" s="21" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="14" t="inlineStr">
@@ -3347,19 +3440,19 @@
       </c>
       <c r="D79" s="14" t="inlineStr">
         <is>
-          <t>Relever le temps et le nombre de requêtes des écrans les plus ouverts — caisse, catalogue, factures, tableau de bord. Corriger sans mesurer fait optimiser ce qui n'était pas le problème.</t>
-        </is>
-      </c>
-      <c r="E79" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F79" s="17" t="n">
-        <v>46321</v>
-      </c>
-      <c r="G79" s="17" t="n">
-        <v>46321</v>
+          <t>Relever le temps et le nombre de requêtes des écrans les plus ouverts — caisse, catalogue, factures, tableau de bord. Corriger sans mesurer fait optimiser ce qui n'était pas le problème. MESURÉ LE 06/10/2026 sur MariaDB, 10 000 articles, chaque écran GET de l'administration : Articles &amp; stock 51 517 ms / 66 146 requêtes ; Nouvelle vente 13 949 ms / 20 020 ; création d'un point de vente 11 449 ms / 17 103 ; tout le reste sous 1,3 s. Au navigateur : la caisse finissait de charger en 19,6 s (toutes les photos demandées d'un coup), et toutes les pages attendaient trois CDN en feuilles bloquantes. Sur un hébergement où chaque requête SQL coûte 1 à 2 ms, 20 000 requêtes font la « trentaine de secondes ».</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F79" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G79" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H79" s="15" t="inlineStr">
         <is>
@@ -3385,19 +3478,19 @@
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>Les écrans en cartes (caisse, catalogue) appellent des méthodes de modèle par ligne. Chaque appel non préchargé coûte une requête par carte — trente cartes, soixante requêtes de plus.</t>
-        </is>
-      </c>
-      <c r="E80" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F80" s="17" t="n">
-        <v>46321</v>
-      </c>
-      <c r="G80" s="17" t="n">
-        <v>46322</v>
+          <t>Les écrans en cartes (caisse, catalogue) appellent des méthodes de modèle par ligne. Chaque appel non préchargé coûte une requête par carte — trente cartes, soixante requêtes de plus. FAIT LE 06/10/2026 (lot 43) : chargement automatique des relations (Model::automaticallyEagerLoadRelationships), engagements préchargés en deux requêtes, fiches indexées par site. Stock : 28 requêtes, caisse : ~30, quel que soit le catalogue — une épreuve le garde. TROUVÉ : l'écran de stock ÉCRIVAIT en base (voir section 18).</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F80" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G80" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H80" s="15" t="inlineStr">
         <is>
@@ -3423,19 +3516,19 @@
       </c>
       <c r="D81" s="14" t="inlineStr">
         <is>
-          <t>Sur les colonnes de filtre et de tri les plus sollicitées, au vu des mesures du chantier 12.1.</t>
-        </is>
-      </c>
-      <c r="E81" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F81" s="17" t="n">
-        <v>46322</v>
-      </c>
-      <c r="G81" s="17" t="n">
-        <v>46322</v>
+          <t>Sur les colonnes de filtre et de tri les plus sollicitées, au vu des mesures du chantier 12.1. FAIT LE 06/10/2026 (lot 51) : index (entreprise, statut de synchronisation) sur les écritures, relues toutes les cinq minutes ; (site, étape) sur les ventes. achats.numero_fne en manque aussi et reste sans — périmètre FNE gelé.</t>
+        </is>
+      </c>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F81" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G81" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H81" s="15" t="inlineStr">
         <is>
@@ -3461,19 +3554,19 @@
       </c>
       <c r="D82" s="14" t="inlineStr">
         <is>
-          <t>Polices d'icônes, images non redimensionnées, feuilles de style dupliquées. Lié au chantier 9.1 — la police d'icônes est déjà en cause sur la page d'inscription.</t>
-        </is>
-      </c>
-      <c r="E82" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F82" s="17" t="n">
-        <v>46322</v>
-      </c>
-      <c r="G82" s="17" t="n">
-        <v>46322</v>
+          <t>Polices d'icônes, images non redimensionnées, feuilles de style dupliquées. Lié au chantier 9.1 — la police d'icônes est déjà en cause sur la page d'inscription. FAIT LE 06/10/2026 (lots 41 et 50) : polices, icônes et Chart.js servis par l'application, CSP refermée ; Tabler (820 Ko pour 27 icônes) remplacé par Font Awesome ; content-visibility sur les cartes de caisse (19,6 s → 4,2 s au navigateur, 15 photos au lieu de toutes), loading="lazy" sur le catalogue.</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F82" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G82" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H82" s="15" t="inlineStr">
         <is>
@@ -3481,19 +3574,20 @@
         </is>
       </c>
     </row>
+    <row r="83"/>
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="12" t="inlineStr">
         <is>
           <t>13. CONDUITE DU CHANTIER</t>
         </is>
       </c>
-      <c r="B84" s="13" t="n"/>
-      <c r="C84" s="13" t="n"/>
-      <c r="D84" s="13" t="n"/>
-      <c r="E84" s="13" t="n"/>
-      <c r="F84" s="13" t="n"/>
-      <c r="G84" s="13" t="n"/>
-      <c r="H84" s="13" t="n"/>
+      <c r="B84" s="21" t="n"/>
+      <c r="C84" s="21" t="n"/>
+      <c r="D84" s="21" t="n"/>
+      <c r="E84" s="21" t="n"/>
+      <c r="F84" s="21" t="n"/>
+      <c r="G84" s="21" t="n"/>
+      <c r="H84" s="21" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="14" t="inlineStr">
@@ -3513,18 +3607,18 @@
       </c>
       <c r="D85" s="14" t="inlineStr">
         <is>
-          <t>Sur `main`, et sur les DEUX dépôts : `origin` (meledjeabrahamagnimel-lgtm/Selflow) et `nouveau-repo` (IT-dcknowing/Selflow).</t>
-        </is>
-      </c>
-      <c r="E85" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F85" s="17" t="n">
+          <t>Sur `main`, et sur les DEUX dépôts : `origin` (meledjeabrahamagnimel-lgtm/Selflow) et `nouveau-repo` (IT-dcknowing/Selflow). SESSION DU 06/10/2026 : consigne de session — développement sur la branche `claude/exciting-keller-9d5tdz`, poussée sur `origin` (meledjeabrahamagnimel-lgtm/Selflow) ; le dépôt `nouveau-repo` n'est pas configuré dans cet environnement. Fusion dans `main` et envoi sur les deux dépôts à faire par le propriétaire.</t>
+        </is>
+      </c>
+      <c r="E85" s="19" t="inlineStr">
+        <is>
+          <t>Sans objet</t>
+        </is>
+      </c>
+      <c r="F85" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G85" s="17" t="n">
+      <c r="G85" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="H85" s="15" t="inlineStr">
@@ -3551,18 +3645,18 @@
       </c>
       <c r="D86" s="14" t="inlineStr">
         <is>
-          <t>Et la vérification au retrait : retirer le correctif, relancer, s'assurer que l'épreuve tombe. Une épreuve qui passe des deux côtés ne garde rien.</t>
-        </is>
-      </c>
-      <c r="E86" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F86" s="17" t="n">
+          <t>Et la vérification au retrait : retirer le correctif, relancer, s'assurer que l'épreuve tombe. Une épreuve qui passe des deux côtés ne garde rien. Tenu à chaque lot des 06/10/2026 : 1 492 épreuves, 1 487 passantes, 5 sautées, et vérification au retrait.</t>
+        </is>
+      </c>
+      <c r="E86" s="19" t="inlineStr">
+        <is>
+          <t>Sans objet</t>
+        </is>
+      </c>
+      <c r="F86" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G86" s="17" t="n">
+      <c r="G86" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="H86" s="15" t="inlineStr">
@@ -3589,18 +3683,18 @@
       </c>
       <c r="D87" s="14" t="inlineStr">
         <is>
-          <t>C'est la mémoire du projet — exigence de CLAUDE.md. Ce fichier est tenu en parallèle : statut et dates réelles, lot par lot.</t>
-        </is>
-      </c>
-      <c r="E87" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F87" s="17" t="n">
+          <t>C'est la mémoire du projet — exigence de CLAUDE.md. Ce fichier est tenu en parallèle : statut et dates réelles, lot par lot. Tenu : lots 41 à 52 au journal, ce classeur, et la passation du 06/10/2026.</t>
+        </is>
+      </c>
+      <c r="E87" s="19" t="inlineStr">
+        <is>
+          <t>Sans objet</t>
+        </is>
+      </c>
+      <c r="F87" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G87" s="17" t="n">
+      <c r="G87" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="H87" s="15" t="inlineStr">
@@ -3627,19 +3721,19 @@
       </c>
       <c r="D88" s="14" t="inlineStr">
         <is>
-          <t>Ordre demandé par le propriétaire. Il est aussi le bon techniquement : le dépliage et le masquage changent tous deux ce que la visite guidée doit parcourir (chantier 9.4), et ce que les modèles d'import doivent refléter (chantier 11).</t>
-        </is>
-      </c>
-      <c r="E88" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F88" s="17" t="n">
+          <t>Ordre demandé par le propriétaire. Il est aussi le bon techniquement : le dépliage et le masquage changent tous deux ce que la visite guidée doit parcourir (chantier 9.4), et ce que les modèles d'import doivent refléter (chantier 11). Appliqué : navigation, comptabilité, puis le reste.</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F88" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G88" s="17" t="n">
-        <v>46297</v>
+      <c r="G88" s="22" t="n">
+        <v>46301</v>
       </c>
       <c r="H88" s="15" t="inlineStr">
         <is>
@@ -3653,13 +3747,13 @@
           <t>14. TROUVÉ EN CHEMIN — relevé pendant le chantier 1, le 02/10/2026</t>
         </is>
       </c>
-      <c r="B89" s="13" t="n"/>
-      <c r="C89" s="13" t="n"/>
-      <c r="D89" s="13" t="n"/>
-      <c r="E89" s="13" t="n"/>
-      <c r="F89" s="13" t="n"/>
-      <c r="G89" s="13" t="n"/>
-      <c r="H89" s="13" t="n"/>
+      <c r="B89" s="21" t="n"/>
+      <c r="C89" s="21" t="n"/>
+      <c r="D89" s="21" t="n"/>
+      <c r="E89" s="21" t="n"/>
+      <c r="F89" s="21" t="n"/>
+      <c r="G89" s="21" t="n"/>
+      <c r="H89" s="21" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
@@ -3687,10 +3781,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F90" s="17" t="n">
+      <c r="F90" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G90" s="17" t="n">
+      <c r="G90" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H90" s="15" t="inlineStr">
@@ -3725,10 +3819,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F91" s="17" t="n">
+      <c r="F91" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G91" s="17" t="n">
+      <c r="G91" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H91" s="15" t="inlineStr">
@@ -3763,10 +3857,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F92" s="17" t="n">
+      <c r="F92" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G92" s="17" t="n">
+      <c r="G92" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H92" s="15" t="inlineStr">
@@ -3801,10 +3895,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F93" s="17" t="n">
+      <c r="F93" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G93" s="17" t="n">
+      <c r="G93" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H93" s="15" t="inlineStr">
@@ -3819,13 +3913,13 @@
           <t>15. LA LIVRAISON — relevé le 05/10/2026</t>
         </is>
       </c>
-      <c r="B94" s="13" t="n"/>
-      <c r="C94" s="13" t="n"/>
-      <c r="D94" s="13" t="n"/>
-      <c r="E94" s="13" t="n"/>
-      <c r="F94" s="13" t="n"/>
-      <c r="G94" s="13" t="n"/>
-      <c r="H94" s="13" t="n"/>
+      <c r="B94" s="21" t="n"/>
+      <c r="C94" s="21" t="n"/>
+      <c r="D94" s="21" t="n"/>
+      <c r="E94" s="21" t="n"/>
+      <c r="F94" s="21" t="n"/>
+      <c r="G94" s="21" t="n"/>
+      <c r="H94" s="21" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="14" t="inlineStr">
@@ -3853,10 +3947,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F95" s="17" t="n">
+      <c r="F95" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G95" s="17" t="n">
+      <c r="G95" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H95" s="15" t="inlineStr">
@@ -3891,10 +3985,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F96" s="17" t="n">
+      <c r="F96" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G96" s="17" t="n">
+      <c r="G96" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H96" s="15" t="inlineStr">
@@ -3929,10 +4023,10 @@
           <t>À trancher</t>
         </is>
       </c>
-      <c r="F97" s="17" t="n">
-        <v>46301</v>
-      </c>
-      <c r="G97" s="17" t="n">
+      <c r="F97" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G97" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="H97" s="15" t="inlineStr">
@@ -3967,10 +4061,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F98" s="17" t="n">
+      <c r="F98" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G98" s="17" t="n">
+      <c r="G98" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H98" s="15" t="inlineStr">
@@ -3979,19 +4073,20 @@
         </is>
       </c>
     </row>
+    <row r="99"/>
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="12" t="inlineStr">
         <is>
           <t>16. LES ÉCRITURES D'ACHAT VENUES DE LA DGI — règles en vigueur</t>
         </is>
       </c>
-      <c r="B100" s="13" t="n"/>
-      <c r="C100" s="13" t="n"/>
-      <c r="D100" s="13" t="n"/>
-      <c r="E100" s="13" t="n"/>
-      <c r="F100" s="13" t="n"/>
-      <c r="G100" s="13" t="n"/>
-      <c r="H100" s="13" t="n"/>
+      <c r="B100" s="21" t="n"/>
+      <c r="C100" s="21" t="n"/>
+      <c r="D100" s="21" t="n"/>
+      <c r="E100" s="21" t="n"/>
+      <c r="F100" s="21" t="n"/>
+      <c r="G100" s="21" t="n"/>
+      <c r="H100" s="21" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="14" t="inlineStr">
@@ -4006,12 +4101,12 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Rappel : une facture reçue ne produit aucune écriture</t>
+          <t>Rappel : une facture reçue passe désormais en écriture (section 17)</t>
         </is>
       </c>
       <c r="D101" s="14" t="inlineStr">
         <is>
-          <t>RÈGLE EN VIGUEUR, rappelée le 05/10/2026. `FactureRecueControleur` NE CRÉE AUCUN ACHAT : le relevé du portail est un objet de rapprochement, pas une pièce. L'écriture vient de l'achat Selflow auquel la facture est rattachée, et de lui seul. Une facture reçue non rapprochée ne produit donc rien — l'achat doit être saisi dans Selflow pour que la comptabilité existe.</t>
+          <t>RÈGLE REMPLACÉE LE 06/10/2026 par le propriétaire : « une facture d'achat reçue de la DGI doit passer en écritures comptables, avec les numéros de compte paramétrés — c'est la priorité ». Voir la section 17. Ce qui reste vrai : FactureRecueControleur ne crée aucun achat ni mouvement de stock.</t>
         </is>
       </c>
       <c r="E101" s="19" t="inlineStr">
@@ -4019,10 +4114,10 @@
           <t>Sans objet</t>
         </is>
       </c>
-      <c r="F101" s="17" t="n">
+      <c r="F101" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G101" s="17" t="n">
+      <c r="G101" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H101" s="15" t="inlineStr">
@@ -4057,10 +4152,10 @@
           <t>Sans objet</t>
         </is>
       </c>
-      <c r="F102" s="17" t="n">
+      <c r="F102" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G102" s="17" t="n">
+      <c r="G102" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H102" s="15" t="inlineStr">
@@ -4087,7 +4182,7 @@
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>Et il ne collecte aucune TVA — ce que le payload d'achat traduit déjà, et qui reste GELÉ. Les autres achats ne sont enregistrés que pour la comptabilité. Seul point de contact autorisé avec la FNE : l'écriture comptable du BAPA, en lecture seule de ce que la plateforme a retourné. C'est ce qui fonde le chantier 8.4.</t>
+          <t>Et il ne collecte aucune TVA — ce que le payload d'achat traduit déjà, et qui reste GELÉ. Les autres achats ne sont enregistrés que pour la comptabilité. Seul point de contact autorisé avec la FNE : l'écriture comptable du BAPA, en lecture seule de ce que la plateforme a retourné. C'est ce qui fonde le chantier 8.4. Précisé le 06/10/2026 : le BAPA passe en écriture par son ACHAT, jamais par le relevé qui le ramène (section 17).</t>
         </is>
       </c>
       <c r="E103" s="19" t="inlineStr">
@@ -4095,10 +4190,10 @@
           <t>Sans objet</t>
         </is>
       </c>
-      <c r="F103" s="17" t="n">
+      <c r="F103" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G103" s="17" t="n">
+      <c r="G103" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H103" s="15" t="inlineStr">
@@ -4133,10 +4228,10 @@
           <t>Sans objet</t>
         </is>
       </c>
-      <c r="F104" s="17" t="n">
+      <c r="F104" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G104" s="17" t="n">
+      <c r="G104" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H104" s="15" t="inlineStr">
@@ -4145,19 +4240,423 @@
         </is>
       </c>
     </row>
+    <row r="105" ht="20" customHeight="1">
+      <c r="A105" s="23" t="inlineStr">
+        <is>
+          <t>17. LES ACHATS DGI PASSENT EN ÉCRITURE — règle du propriétaire, 06/10/2026</t>
+        </is>
+      </c>
+      <c r="B105" s="21" t="n"/>
+      <c r="C105" s="21" t="n"/>
+      <c r="D105" s="21" t="n"/>
+      <c r="E105" s="21" t="n"/>
+      <c r="F105" s="21" t="n"/>
+      <c r="G105" s="21" t="n"/>
+      <c r="H105" s="21" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="14" t="inlineStr">
+        <is>
+          <t>Factures reçues du portail</t>
+        </is>
+      </c>
+      <c r="B106" s="15" t="inlineStr">
+        <is>
+          <t>17.1</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>La facture fournisseur certifiée par la DGI passe au journal des achats</t>
+        </is>
+      </c>
+      <c r="D106" s="14" t="inlineStr">
+        <is>
+          <t>DEMANDÉ LE 06/10/2026 : « une facture d'achat reçue de la DGI doit passer en écritures comptables avec les numéros de compte paramétrés — ce sera la priorité, cela concerne les factures fournisseur ». FAIT (lot 42) : EcritureFactureRecueService — charges au compte d'achat de l'article reconnu (référence ou désignation), sinon la configuration globale, sinon 601000 ; TVA déductible ventilée comme les achats saisis ; timbre en 646200, autres taxes en 648000 (647 porte les amendes) ; le fournisseur au crédit du net à payer, avec son numéro de tiers — fiche créée d'après le NCC, le nom et le RCCM certifiés s'il manque. Un avoir reçu inverse les sens ; une proforma ne passe pas.</t>
+        </is>
+      </c>
+      <c r="E106" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F106" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G106" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H106" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="14" t="inlineStr">
+        <is>
+          <t>BAPA</t>
+        </is>
+      </c>
+      <c r="B107" s="15" t="inlineStr">
+        <is>
+          <t>17.2</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Le BAPA ne passe pas deux fois</t>
+        </is>
+      </c>
+      <c r="D107" s="14" t="inlineStr">
+        <is>
+          <t>FAIT (lot 42) : le BAPA passe en écriture par son achat. S'il revient par le relevé, il est reconnu — l'émetteur porte notre NCC, ou la référence est le numéro FNE d'un de nos achats — et ignoré.</t>
+        </is>
+      </c>
+      <c r="E107" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F107" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G107" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H107" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="14" t="inlineStr">
+        <is>
+          <t>Achats saisis</t>
+        </is>
+      </c>
+      <c r="B108" s="15" t="inlineStr">
+        <is>
+          <t>17.3</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>Tout achat saisi passe en écriture — et l'écran le dit</t>
+        </is>
+      </c>
+      <c r="D108" s="14" t="inlineStr">
+        <is>
+          <t>FAIT (lot 42) : comme avant, l'achat saisi produit son écriture. L'écran « Nouvel achat » prévient en tête : les factures normalisées arrivent seules de la DGI, ne les saisissez pas ici — réservez l'écran aux charges que personne ne normalise et aux BAPA.</t>
+        </is>
+      </c>
+      <c r="E108" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F108" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G108" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H108" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="14" t="inlineStr">
+        <is>
+          <t>Doublons</t>
+        </is>
+      </c>
+      <c r="B109" s="15" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Une seule écriture par pièce, quoi qu'il arrive</t>
+        </is>
+      </c>
+      <c r="D109" s="14" t="inlineStr">
+        <is>
+          <t>FAIT (lot 42) : `operation_id` dit qu'une facture est passée — le relevé horaire ne la repasse pas. Rattachée après coup à un achat (rapprochement automatique ou geste), ou écartée, elle est CONTRE-PASSÉE plutôt qu'effacée : l'opération a pu partir chez Comptaflow. Détachée ou réintégrée, elle repasse.</t>
+        </is>
+      </c>
+      <c r="E109" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F109" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G109" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H109" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="14" t="inlineStr">
+        <is>
+          <t>Déploiement</t>
+        </is>
+      </c>
+      <c r="B110" s="15" t="inlineStr">
+        <is>
+          <t>17.5</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>Passer les relevés déjà en base</t>
+        </is>
+      </c>
+      <c r="D110" s="14" t="inlineStr">
+        <is>
+          <t>À FAIRE AU DÉPLOIEMENT : `php artisan migrate` (colonne operation_id), puis `php artisan selflow:ecritures-factures-recues` pour les factures relevées avant ce lot. Sans danger à relancer.</t>
+        </is>
+      </c>
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F110" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G110" s="22" t="n"/>
+      <c r="H110" s="15" t="inlineStr">
+        <is>
+          <t>Déploiement</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="14" t="inlineStr">
+        <is>
+          <t>Relevé du portail</t>
+        </is>
+      </c>
+      <c r="B111" s="15" t="inlineStr">
+        <is>
+          <t>17.6</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>Le relevé suivant défaisait un écartement</t>
+        </is>
+      </c>
+      <c r="D111" s="14" t="inlineStr">
+        <is>
+          <t>TROUVÉ ET CORRIGÉ (lot 42) : chaque relevé remettait « à rapprocher » une facture écartée — elle revenait dans la liste, et, depuis cette règle, serait repassée en écriture contre la décision de l'utilisateur. Le statut ne se pose plus qu'à l'arrivée.</t>
+        </is>
+      </c>
+      <c r="E111" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F111" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G111" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H111" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="20" customHeight="1">
+      <c r="A112" s="23" t="inlineStr">
+        <is>
+          <t>18. TROUVÉ EN CHEMIN — 06/10/2026</t>
+        </is>
+      </c>
+      <c r="B112" s="21" t="n"/>
+      <c r="C112" s="21" t="n"/>
+      <c r="D112" s="21" t="n"/>
+      <c r="E112" s="21" t="n"/>
+      <c r="F112" s="21" t="n"/>
+      <c r="G112" s="21" t="n"/>
+      <c r="H112" s="21" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="14" t="inlineStr">
+        <is>
+          <t>Écran Articles &amp; stock</t>
+        </is>
+      </c>
+      <c r="B113" s="15" t="inlineStr">
+        <is>
+          <t>18.1</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>L'écran écrivait dans les fiches de stock — corrigé</t>
+        </is>
+      </c>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>TROUVÉ EN MESURANT LA LENTEUR (lot 43) : `setAttribute('stock_actuel', …)` passait par un mutateur qui faisait `Stock::updateOrCreate` sur le site actif. En vue « Tous les sites », la somme des sites s'écrivait dans la fiche du site actif, à chaque affichage, sans mouvement au journal. Les mutateurs ne posent plus qu'une valeur d'affichage.</t>
+        </is>
+      </c>
+      <c r="E113" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F113" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G113" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H113" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="14" t="inlineStr">
+        <is>
+          <t>Données en production</t>
+        </is>
+      </c>
+      <c r="B114" s="15" t="inlineStr">
+        <is>
+          <t>18.2</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Vérifier les fiches que l'ancien écran a faussées</t>
+        </is>
+      </c>
+      <c r="D114" s="14" t="inlineStr">
+        <is>
+          <t>À FAIRE PAR LE PROPRIÉTAIRE après déploiement : `php artisan selflow:verifier-stocks` (lot 52, lecture seule) liste les fiches qui s'écartent du `stock_apres` de leur dernier mouvement. Corriger par un inventaire physique, jamais à la main. Sur la base de mesure, il a retrouvé les 46 fiches que l'ancien code y avait gonflées.</t>
+        </is>
+      </c>
+      <c r="E114" s="18" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F114" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G114" s="22" t="n"/>
+      <c r="H114" s="15" t="inlineStr">
+        <is>
+          <t>Déploiement</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="14" t="inlineStr">
+        <is>
+          <t>Suite Comptaflow</t>
+        </is>
+      </c>
+      <c r="B115" s="15" t="inlineStr">
+        <is>
+          <t>18.3</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>19 épreuves déjà rouges chez Comptaflow</t>
+        </is>
+      </c>
+      <c r="D115" s="14" t="inlineStr">
+        <is>
+          <t>Relevé en lançant sa suite le 06/10/2026 : 19 échecs présents AVANT ce lot (identiques avec et sans). Une vingtième — la recopie au 28 février, qui prenait sa ligne sans ordre — tombait selon l'index choisi par SQLite : corrigée. Les 19 reviennent au mainteneur de Comptaflow.</t>
+        </is>
+      </c>
+      <c r="E115" s="18" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F115" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G115" s="22" t="n"/>
+      <c r="H115" s="15" t="inlineStr">
+        <is>
+          <t>Comptaflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="14" t="inlineStr">
+        <is>
+          <t>Avoirs — SQLite</t>
+        </is>
+      </c>
+      <c r="B116" s="15" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>Une comparaison qui ne valait que sous MySQL</t>
+        </is>
+      </c>
+      <c r="D116" s="14" t="inlineStr">
+        <is>
+          <t>TROUVÉ (lot 45) : SQLite compare un nombre à un paramètre lié comme TEXTE (7080 &gt; '1' est faux). La requête des factures avoirables écrit `(? + 0)`, portable.</t>
+        </is>
+      </c>
+      <c r="E116" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F116" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="G116" s="22" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H116" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:H105"/>
-  <mergeCells count="16">
+  <autoFilter ref="A4:H116"/>
+  <mergeCells count="18">
     <mergeCell ref="A45:H45"/>
     <mergeCell ref="A94:H94"/>
     <mergeCell ref="A100:H100"/>
     <mergeCell ref="A78:H78"/>
+    <mergeCell ref="A105:H105"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A38:H38"/>
     <mergeCell ref="A72:H72"/>
     <mergeCell ref="A52:H52"/>
     <mergeCell ref="A64:H64"/>
     <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A112:H112"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A84:H84"/>

</xml_diff>

<commit_message>
Lot 41 : comptabilite eteinte, les fiches de tous les jours cessent d'en parler
Section 3 du plan, chantiers 3.1, 3.2, 3.4 et 3.5.

- Fiches client et fournisseur : comptabilite fermee, le compte collectif
  n'est plus demande ni accepte ; le serveur pose 411000 / 401000 a la
  creation et ne touche pas au compte existant a la modification.
- Le numero de tiers et le collectif sont poses a la creation du modele :
  l'API mobile, le parcours B2B et le tiers d'un BAPA creaient des fiches
  sans l'un ni l'autre.
- Parcours de configuration : le numero de compte du rayon ne s'affiche
  que comptabilite ouverte ; un module deja ouvert est montre comme acquis,
  et l'etape 3 se saute quand il n'y a rien a choisir.

Suite : 1 455 epreuves, 1 450 passantes, 5 sautees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de travail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan de travail'!$A$4:$H$105</definedName>
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -134,7 +133,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -147,11 +146,26 @@
         <color rgb="FFD8DCE3"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD8DCE3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="FFD8DCE3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -195,7 +209,7 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -206,6 +220,13 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -647,25 +668,25 @@
           <t>1. NAVIGATION — à traiter en premier</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="E5" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
         <is>
           <t>Terminée</t>
         </is>
@@ -677,25 +698,25 @@
           <t>2. COMPTABILITÉ — le principe : Selflow facture, Comptaflow tient les livres</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="E6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="E6" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
         <is>
           <t>Terminée</t>
         </is>
@@ -707,27 +728,27 @@
           <t>3. COMPTABILITÉ ÉTEINTE — ce qui disparaît des écrans courants</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>0/6</t>
+      <c r="D7" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>4/6</t>
         </is>
       </c>
     </row>
@@ -737,25 +758,25 @@
           <t>4. MOYENS DE PAIEMENT — ce qui remplace les codes journaux</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="15" t="n">
         <v>28</v>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="E8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>Terminée</t>
         </is>
@@ -767,25 +788,25 @@
           <t>5. LES ÉCRITURES TOURNENT MÊME QUAND LA COMPTABILITÉ EST ÉTEINTE</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="15" t="n">
         <v>34</v>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="6" t="n">
+      <c r="D9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="F9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
         <is>
           <t>0/2</t>
         </is>
@@ -797,25 +818,25 @@
           <t>6. CONFIGURATION GLOBALE — saisir les comptes une fois, et non par produit</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="15" t="n">
         <v>38</v>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="D10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="6" t="n">
+      <c r="D10" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="F10" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
         <is>
           <t>0/5</t>
         </is>
@@ -827,25 +848,25 @@
           <t>7. DÉVERSEMENT COMPTAFLOW — les lignes arrivaient déséquilibrées</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="15" t="n">
         <v>45</v>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="D11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="6" t="n">
+      <c r="D11" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="F11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="F11" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="18" t="inlineStr">
         <is>
           <t>0/5</t>
         </is>
@@ -857,25 +878,25 @@
           <t>8. AVOIRS — un avoir ne peut pas dépasser la facture (image 4)</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="15" t="n">
         <v>52</v>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="6" t="n">
+      <c r="D12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="F12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
         <is>
           <t>0/4</t>
         </is>
@@ -887,25 +908,25 @@
           <t>9. ÉCRANS D'ENTRÉE — inscription, point de vente, visite guidée</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="6" t="n">
+      <c r="D13" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="F13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="F13" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="18" t="inlineStr">
         <is>
           <t>0/4</t>
         </is>
@@ -917,25 +938,25 @@
           <t>10. PARAMÈTRES — le compte sur la plateforme FNE</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="D14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="6" t="n">
+      <c r="D14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="F14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="6" t="n">
+      <c r="F14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="H14" s="18" t="inlineStr">
         <is>
           <t>0/6</t>
         </is>
@@ -947,25 +968,25 @@
           <t>11. MODÈLES D'IMPORT — refléter exactement les champs de la plateforme</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="15" t="n">
         <v>72</v>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6" t="n">
+      <c r="D15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="F15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="F15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="18" t="inlineStr">
         <is>
           <t>0/4</t>
         </is>
@@ -977,25 +998,25 @@
           <t>12. PERFORMANCE — l'application est lente</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B16" s="15" t="n">
         <v>78</v>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="6" t="n">
+      <c r="D16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="F16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="F16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
         <is>
           <t>0/4</t>
         </is>
@@ -1007,25 +1028,25 @@
           <t>13. CONDUITE DU CHANTIER</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B17" s="15" t="n">
         <v>84</v>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="6" t="n">
+      <c r="D17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
+      <c r="F17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
         <is>
           <t>0/4</t>
         </is>
@@ -1037,25 +1058,25 @@
           <t>14. TROUVÉ EN CHEMIN — relevé pendant le chantier 1, le 02/10/2026</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n">
+      <c r="B18" s="15" t="n">
         <v>89</v>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="E18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="E18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>Terminée</t>
         </is>
@@ -1067,25 +1088,25 @@
           <t>15. LA LIVRAISON — relevé le 05/10/2026</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B19" s="15" t="n">
         <v>94</v>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="D19" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="E19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="6" t="n">
+      <c r="E19" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="G19" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="18" t="inlineStr">
         <is>
           <t>3/4</t>
         </is>
@@ -1097,25 +1118,25 @@
           <t>16. LES ÉCRITURES D'ACHAT VENUES DE LA DGI — règles en vigueur</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n">
+      <c r="B20" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="6" t="n">
+      <c r="D20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>Terminée</t>
         </is>
@@ -1131,10 +1152,10 @@
         <v>71</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F22" s="10" t="n">
         <v>1</v>
@@ -1224,18 +1245,18 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>1. NAVIGATION — à traiter en premier</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n"/>
-      <c r="C5" s="13" t="n"/>
-      <c r="D5" s="13" t="n"/>
-      <c r="E5" s="13" t="n"/>
-      <c r="F5" s="13" t="n"/>
-      <c r="G5" s="13" t="n"/>
-      <c r="H5" s="13" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="21" t="n"/>
+      <c r="H5" s="21" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
@@ -1263,10 +1284,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F6" s="17" t="n">
+      <c r="F6" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G6" s="17" t="n">
+      <c r="G6" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H6" s="15" t="inlineStr">
@@ -1301,10 +1322,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F7" s="17" t="n">
+      <c r="F7" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G7" s="17" t="n">
+      <c r="G7" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H7" s="15" t="inlineStr">
@@ -1339,10 +1360,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F8" s="17" t="n">
+      <c r="F8" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H8" s="15" t="inlineStr">
@@ -1377,10 +1398,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F9" s="17" t="n">
+      <c r="F9" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G9" s="17" t="n">
+      <c r="G9" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H9" s="15" t="inlineStr">
@@ -1390,18 +1411,18 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>2. COMPTABILITÉ — le principe : Selflow facture, Comptaflow tient les livres</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="13" t="n"/>
-      <c r="H11" s="13" t="n"/>
+      <c r="B11" s="21" t="n"/>
+      <c r="C11" s="21" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="21" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -1429,10 +1450,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F12" s="17" t="n">
+      <c r="F12" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H12" s="15" t="inlineStr">
@@ -1467,10 +1488,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F13" s="17" t="n">
+      <c r="F13" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G13" s="17" t="n">
+      <c r="G13" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H13" s="15" t="inlineStr">
@@ -1505,10 +1526,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F14" s="17" t="n">
+      <c r="F14" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G14" s="17" t="n">
+      <c r="G14" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H14" s="15" t="inlineStr">
@@ -1543,10 +1564,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F15" s="17" t="n">
+      <c r="F15" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G15" s="17" t="n">
+      <c r="G15" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H15" s="15" t="inlineStr">
@@ -1581,10 +1602,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F16" s="17" t="n">
+      <c r="F16" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G16" s="17" t="n">
+      <c r="G16" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H16" s="15" t="inlineStr">
@@ -1619,10 +1640,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F17" s="17" t="n">
+      <c r="F17" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G17" s="17" t="n">
+      <c r="G17" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -1657,10 +1678,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F18" s="17" t="n">
+      <c r="F18" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G18" s="17" t="n">
+      <c r="G18" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H18" s="15" t="inlineStr">
@@ -1670,18 +1691,18 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>3. COMPTABILITÉ ÉTEINTE — ce qui disparaît des écrans courants</t>
         </is>
       </c>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="13" t="n"/>
-      <c r="G20" s="13" t="n"/>
-      <c r="H20" s="13" t="n"/>
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="21" t="n"/>
+      <c r="D20" s="21" t="n"/>
+      <c r="E20" s="21" t="n"/>
+      <c r="F20" s="21" t="n"/>
+      <c r="G20" s="21" t="n"/>
+      <c r="H20" s="21" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
@@ -1701,18 +1722,18 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>Le champ est aujourd'hui un menu déroulant obligatoire sur les quatre formulaires (création et modification, clients et fournisseurs). Il disparaît quand la comptabilité est éteinte, et la valeur par défaut — 411000 pour un client, 401000 pour un fournisseur — est posée par le serveur. Ce qui n'est plus demandé ne doit plus être accepté : un compte posté à la main ne doit pas s'écrire.</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F21" s="17" t="n">
+          <t>Le champ est aujourd'hui un menu déroulant obligatoire sur les quatre formulaires (création et modification, clients et fournisseurs). Il disparaît quand la comptabilité est éteinte, et la valeur par défaut — 411000 pour un client, 401000 pour un fournisseur — est posée par le serveur. Ce qui n'est plus demandé ne doit plus être accepté : un compte posté à la main ne doit pas s'écrire. FAIT au lot 41 : regleCompteCollectif() — fermée, le champ est exclu de la validation et le serveur pose 411000 / 401000 ; à la modification, le compte existant n'est pas touché.</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F21" s="22" t="n">
         <v>46302</v>
       </c>
-      <c r="G21" s="17" t="n">
+      <c r="G21" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="H21" s="15" t="inlineStr">
@@ -1739,18 +1760,18 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>C'est le seul élément comptable qui survit, parce qu'il sert au rapprochement avec Comptaflow. Il est déjà calculé (six caractères, préfixe pris sur le compte collectif) ; vérifier qu'il ne se saisit nulle part et qu'il est affiché en lecture seule.</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F22" s="17" t="n">
+          <t>C'est le seul élément comptable qui survit, parce qu'il sert au rapprochement avec Comptaflow. Il est déjà calculé (six caractères, préfixe pris sur le compte collectif) ; vérifier qu'il ne se saisit nulle part et qu'il est affiché en lecture seule. FAIT au lot 41 : TROUVÉ que l'API mobile, le parcours B2B et le tiers d'un BAPA créaient des fiches SANS numéro de tiers. Le numéro et le collectif sont désormais posés à la création du modèle (booted), quelle que soit la porte.</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="n">
         <v>46302</v>
       </c>
-      <c r="G22" s="17" t="n">
+      <c r="G22" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="H22" s="15" t="inlineStr">
@@ -1785,10 +1806,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F23" s="17" t="n">
+      <c r="F23" s="22" t="n">
         <v>46302</v>
       </c>
-      <c r="G23" s="17" t="n">
+      <c r="G23" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="H23" s="15" t="inlineStr">
@@ -1815,18 +1836,18 @@
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>Le parcours affiche aujourd'hui le compte réel à côté de chaque libellé de famille (« Vivres et alimentation (311100) »). Le numéro disparaît de l'affichage quand la comptabilité est éteinte — le préparamétrage, lui, continue de se poser en base.</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F24" s="17" t="n">
+          <t>Le parcours'affiche aujourd'hui le compte réel à côté de chaque libellé de famille (« Vivres et alimentation (311100) »). Le numéro disparaît de l'affichage quand la comptabilité est éteinte — le préparamétrage, lui, continue de se poser en base. FAIT au lot 41 : le numéro ne s'affiche à l'étape 4 que comptabilité ouverte ; les mentions « et ses comptes » des étapes 1, 2 et 4 sont retirées.</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="n">
         <v>46302</v>
       </c>
-      <c r="G24" s="17" t="n">
+      <c r="G24" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="H24" s="15" t="inlineStr">
@@ -1853,18 +1874,18 @@
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>L'étape 3 présente « Ce que votre métier demande » avec des cases cochées pour des modules déjà actifs, et annonce qu'ils vont être activés. Ils le sont déjà. Un module en place est montré comme acquis, non comme un choix à refaire ; si tous le sont, l'étape se saute d'elle-même en l'annonçant.</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F25" s="17" t="n">
+          <t>L'étape 3 présente « Ce que votre métier demande » avec des cases cochées pour des modules déjà actifs, et annonce qu'ils vont être activés. Ils le sont déjà. Un module en place est montré comme acquis, non comme un choix à refaire ; si tous le sont, l'étape se saute d'elle-même en l'annonçant. FAIT au lot 41 : seuls les modules explicitement ouverts sont acquis (liste vide = rien d'acquis). L'épreuve ConfigurationVerrouilleeTest qui refermait un module par le parcours est révisée en conséquence.</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="n">
         <v>46302</v>
       </c>
-      <c r="G25" s="17" t="n">
+      <c r="G25" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="H25" s="15" t="inlineStr">
@@ -1899,10 +1920,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F26" s="17" t="n">
+      <c r="F26" s="22" t="n">
         <v>46302</v>
       </c>
-      <c r="G26" s="17" t="n">
+      <c r="G26" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="H26" s="15" t="inlineStr">
@@ -1912,18 +1933,18 @@
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="12" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>4. MOYENS DE PAIEMENT — ce qui remplace les codes journaux</t>
         </is>
       </c>
-      <c r="B28" s="13" t="n"/>
-      <c r="C28" s="13" t="n"/>
-      <c r="D28" s="13" t="n"/>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="13" t="n"/>
-      <c r="G28" s="13" t="n"/>
-      <c r="H28" s="13" t="n"/>
+      <c r="B28" s="21" t="n"/>
+      <c r="C28" s="21" t="n"/>
+      <c r="D28" s="21" t="n"/>
+      <c r="E28" s="21" t="n"/>
+      <c r="F28" s="21" t="n"/>
+      <c r="G28" s="21" t="n"/>
+      <c r="H28" s="21" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
@@ -1951,10 +1972,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F29" s="17" t="n">
+      <c r="F29" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G29" s="17" t="n">
+      <c r="G29" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H29" s="15" t="inlineStr">
@@ -1989,10 +2010,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F30" s="17" t="n">
+      <c r="F30" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G30" s="17" t="n">
+      <c r="G30" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H30" s="15" t="inlineStr">
@@ -2027,10 +2048,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F31" s="17" t="n">
+      <c r="F31" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G31" s="17" t="n">
+      <c r="G31" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H31" s="15" t="inlineStr">
@@ -2065,10 +2086,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F32" s="17" t="n">
+      <c r="F32" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G32" s="17" t="n">
+      <c r="G32" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H32" s="15" t="inlineStr">
@@ -2078,18 +2099,18 @@
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="12" t="inlineStr">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t>5. LES ÉCRITURES TOURNENT MÊME QUAND LA COMPTABILITÉ EST ÉTEINTE</t>
         </is>
       </c>
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="13" t="n"/>
-      <c r="D34" s="13" t="n"/>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="13" t="n"/>
-      <c r="G34" s="13" t="n"/>
-      <c r="H34" s="13" t="n"/>
+      <c r="B34" s="21" t="n"/>
+      <c r="C34" s="21" t="n"/>
+      <c r="D34" s="21" t="n"/>
+      <c r="E34" s="21" t="n"/>
+      <c r="F34" s="21" t="n"/>
+      <c r="G34" s="21" t="n"/>
+      <c r="H34" s="21" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
@@ -2117,10 +2138,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F35" s="17" t="n">
+      <c r="F35" s="22" t="n">
         <v>46304</v>
       </c>
-      <c r="G35" s="17" t="n">
+      <c r="G35" s="22" t="n">
         <v>46304</v>
       </c>
       <c r="H35" s="15" t="inlineStr">
@@ -2155,10 +2176,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F36" s="17" t="n">
+      <c r="F36" s="22" t="n">
         <v>46304</v>
       </c>
-      <c r="G36" s="17" t="n">
+      <c r="G36" s="22" t="n">
         <v>46304</v>
       </c>
       <c r="H36" s="15" t="inlineStr">
@@ -2168,18 +2189,18 @@
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="12" t="inlineStr">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>6. CONFIGURATION GLOBALE — saisir les comptes une fois, et non par produit</t>
         </is>
       </c>
-      <c r="B38" s="13" t="n"/>
-      <c r="C38" s="13" t="n"/>
-      <c r="D38" s="13" t="n"/>
-      <c r="E38" s="13" t="n"/>
-      <c r="F38" s="13" t="n"/>
-      <c r="G38" s="13" t="n"/>
-      <c r="H38" s="13" t="n"/>
+      <c r="B38" s="21" t="n"/>
+      <c r="C38" s="21" t="n"/>
+      <c r="D38" s="21" t="n"/>
+      <c r="E38" s="21" t="n"/>
+      <c r="F38" s="21" t="n"/>
+      <c r="G38" s="21" t="n"/>
+      <c r="H38" s="21" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
@@ -2207,10 +2228,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F39" s="17" t="n">
+      <c r="F39" s="22" t="n">
         <v>46307</v>
       </c>
-      <c r="G39" s="17" t="n">
+      <c r="G39" s="22" t="n">
         <v>46307</v>
       </c>
       <c r="H39" s="15" t="inlineStr">
@@ -2245,10 +2266,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F40" s="17" t="n">
+      <c r="F40" s="22" t="n">
         <v>46307</v>
       </c>
-      <c r="G40" s="17" t="n">
+      <c r="G40" s="22" t="n">
         <v>46308</v>
       </c>
       <c r="H40" s="15" t="inlineStr">
@@ -2283,10 +2304,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F41" s="17" t="n">
+      <c r="F41" s="22" t="n">
         <v>46308</v>
       </c>
-      <c r="G41" s="17" t="n">
+      <c r="G41" s="22" t="n">
         <v>46308</v>
       </c>
       <c r="H41" s="15" t="inlineStr">
@@ -2321,10 +2342,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F42" s="17" t="n">
+      <c r="F42" s="22" t="n">
         <v>46308</v>
       </c>
-      <c r="G42" s="17" t="n">
+      <c r="G42" s="22" t="n">
         <v>46308</v>
       </c>
       <c r="H42" s="15" t="inlineStr">
@@ -2359,10 +2380,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F43" s="17" t="n">
+      <c r="F43" s="22" t="n">
         <v>46308</v>
       </c>
-      <c r="G43" s="17" t="n">
+      <c r="G43" s="22" t="n">
         <v>46308</v>
       </c>
       <c r="H43" s="15" t="inlineStr">
@@ -2372,18 +2393,18 @@
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
+      <c r="A45" s="23" t="inlineStr">
         <is>
           <t>7. DÉVERSEMENT COMPTAFLOW — les lignes arrivaient déséquilibrées</t>
         </is>
       </c>
-      <c r="B45" s="13" t="n"/>
-      <c r="C45" s="13" t="n"/>
-      <c r="D45" s="13" t="n"/>
-      <c r="E45" s="13" t="n"/>
-      <c r="F45" s="13" t="n"/>
-      <c r="G45" s="13" t="n"/>
-      <c r="H45" s="13" t="n"/>
+      <c r="B45" s="21" t="n"/>
+      <c r="C45" s="21" t="n"/>
+      <c r="D45" s="21" t="n"/>
+      <c r="E45" s="21" t="n"/>
+      <c r="F45" s="21" t="n"/>
+      <c r="G45" s="21" t="n"/>
+      <c r="H45" s="21" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
@@ -2411,10 +2432,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F46" s="17" t="n">
+      <c r="F46" s="22" t="n">
         <v>46309</v>
       </c>
-      <c r="G46" s="17" t="n">
+      <c r="G46" s="22" t="n">
         <v>46309</v>
       </c>
       <c r="H46" s="15" t="inlineStr">
@@ -2449,10 +2470,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F47" s="17" t="n">
+      <c r="F47" s="22" t="n">
         <v>46309</v>
       </c>
-      <c r="G47" s="17" t="n">
+      <c r="G47" s="22" t="n">
         <v>46309</v>
       </c>
       <c r="H47" s="15" t="inlineStr">
@@ -2487,10 +2508,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F48" s="17" t="n">
+      <c r="F48" s="22" t="n">
         <v>46309</v>
       </c>
-      <c r="G48" s="17" t="n">
+      <c r="G48" s="22" t="n">
         <v>46309</v>
       </c>
       <c r="H48" s="15" t="inlineStr">
@@ -2525,10 +2546,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F49" s="17" t="n">
+      <c r="F49" s="22" t="n">
         <v>46310</v>
       </c>
-      <c r="G49" s="17" t="n">
+      <c r="G49" s="22" t="n">
         <v>46310</v>
       </c>
       <c r="H49" s="15" t="inlineStr">
@@ -2563,10 +2584,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F50" s="17" t="n">
+      <c r="F50" s="22" t="n">
         <v>46310</v>
       </c>
-      <c r="G50" s="17" t="n">
+      <c r="G50" s="22" t="n">
         <v>46310</v>
       </c>
       <c r="H50" s="15" t="inlineStr">
@@ -2576,18 +2597,18 @@
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="12" t="inlineStr">
+      <c r="A52" s="23" t="inlineStr">
         <is>
           <t>8. AVOIRS — un avoir ne peut pas dépasser la facture (image 4)</t>
         </is>
       </c>
-      <c r="B52" s="13" t="n"/>
-      <c r="C52" s="13" t="n"/>
-      <c r="D52" s="13" t="n"/>
-      <c r="E52" s="13" t="n"/>
-      <c r="F52" s="13" t="n"/>
-      <c r="G52" s="13" t="n"/>
-      <c r="H52" s="13" t="n"/>
+      <c r="B52" s="21" t="n"/>
+      <c r="C52" s="21" t="n"/>
+      <c r="D52" s="21" t="n"/>
+      <c r="E52" s="21" t="n"/>
+      <c r="F52" s="21" t="n"/>
+      <c r="G52" s="21" t="n"/>
+      <c r="H52" s="21" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
@@ -2615,10 +2636,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F53" s="17" t="n">
+      <c r="F53" s="22" t="n">
         <v>46311</v>
       </c>
-      <c r="G53" s="17" t="n">
+      <c r="G53" s="22" t="n">
         <v>46311</v>
       </c>
       <c r="H53" s="15" t="inlineStr">
@@ -2653,10 +2674,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F54" s="17" t="n">
+      <c r="F54" s="22" t="n">
         <v>46311</v>
       </c>
-      <c r="G54" s="17" t="n">
+      <c r="G54" s="22" t="n">
         <v>46311</v>
       </c>
       <c r="H54" s="15" t="inlineStr">
@@ -2691,10 +2712,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F55" s="17" t="n">
+      <c r="F55" s="22" t="n">
         <v>46311</v>
       </c>
-      <c r="G55" s="17" t="n">
+      <c r="G55" s="22" t="n">
         <v>46311</v>
       </c>
       <c r="H55" s="15" t="inlineStr">
@@ -2729,10 +2750,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F56" s="17" t="n">
+      <c r="F56" s="22" t="n">
         <v>46311</v>
       </c>
-      <c r="G56" s="17" t="n">
+      <c r="G56" s="22" t="n">
         <v>46311</v>
       </c>
       <c r="H56" s="15" t="inlineStr">
@@ -2742,18 +2763,18 @@
       </c>
     </row>
     <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="12" t="inlineStr">
+      <c r="A58" s="23" t="inlineStr">
         <is>
           <t>9. ÉCRANS D'ENTRÉE — inscription, point de vente, visite guidée</t>
         </is>
       </c>
-      <c r="B58" s="13" t="n"/>
-      <c r="C58" s="13" t="n"/>
-      <c r="D58" s="13" t="n"/>
-      <c r="E58" s="13" t="n"/>
-      <c r="F58" s="13" t="n"/>
-      <c r="G58" s="13" t="n"/>
-      <c r="H58" s="13" t="n"/>
+      <c r="B58" s="21" t="n"/>
+      <c r="C58" s="21" t="n"/>
+      <c r="D58" s="21" t="n"/>
+      <c r="E58" s="21" t="n"/>
+      <c r="F58" s="21" t="n"/>
+      <c r="G58" s="21" t="n"/>
+      <c r="H58" s="21" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="14" t="inlineStr">
@@ -2781,10 +2802,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F59" s="17" t="n">
+      <c r="F59" s="22" t="n">
         <v>46314</v>
       </c>
-      <c r="G59" s="17" t="n">
+      <c r="G59" s="22" t="n">
         <v>46314</v>
       </c>
       <c r="H59" s="15" t="inlineStr">
@@ -2819,10 +2840,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F60" s="17" t="n">
+      <c r="F60" s="22" t="n">
         <v>46314</v>
       </c>
-      <c r="G60" s="17" t="n">
+      <c r="G60" s="22" t="n">
         <v>46314</v>
       </c>
       <c r="H60" s="15" t="inlineStr">
@@ -2857,10 +2878,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F61" s="17" t="n">
+      <c r="F61" s="22" t="n">
         <v>46314</v>
       </c>
-      <c r="G61" s="17" t="n">
+      <c r="G61" s="22" t="n">
         <v>46314</v>
       </c>
       <c r="H61" s="15" t="inlineStr">
@@ -2895,10 +2916,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F62" s="17" t="n">
+      <c r="F62" s="22" t="n">
         <v>46315</v>
       </c>
-      <c r="G62" s="17" t="n">
+      <c r="G62" s="22" t="n">
         <v>46315</v>
       </c>
       <c r="H62" s="15" t="inlineStr">
@@ -2908,18 +2929,18 @@
       </c>
     </row>
     <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="12" t="inlineStr">
+      <c r="A64" s="23" t="inlineStr">
         <is>
           <t>10. PARAMÈTRES — le compte sur la plateforme FNE</t>
         </is>
       </c>
-      <c r="B64" s="13" t="n"/>
-      <c r="C64" s="13" t="n"/>
-      <c r="D64" s="13" t="n"/>
-      <c r="E64" s="13" t="n"/>
-      <c r="F64" s="13" t="n"/>
-      <c r="G64" s="13" t="n"/>
-      <c r="H64" s="13" t="n"/>
+      <c r="B64" s="21" t="n"/>
+      <c r="C64" s="21" t="n"/>
+      <c r="D64" s="21" t="n"/>
+      <c r="E64" s="21" t="n"/>
+      <c r="F64" s="21" t="n"/>
+      <c r="G64" s="21" t="n"/>
+      <c r="H64" s="21" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="14" t="inlineStr">
@@ -2947,10 +2968,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F65" s="17" t="n">
+      <c r="F65" s="22" t="n">
         <v>46316</v>
       </c>
-      <c r="G65" s="17" t="n">
+      <c r="G65" s="22" t="n">
         <v>46316</v>
       </c>
       <c r="H65" s="15" t="inlineStr">
@@ -2985,10 +3006,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F66" s="17" t="n">
+      <c r="F66" s="22" t="n">
         <v>46316</v>
       </c>
-      <c r="G66" s="17" t="n">
+      <c r="G66" s="22" t="n">
         <v>46316</v>
       </c>
       <c r="H66" s="15" t="inlineStr">
@@ -3023,10 +3044,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F67" s="17" t="n">
+      <c r="F67" s="22" t="n">
         <v>46316</v>
       </c>
-      <c r="G67" s="17" t="n">
+      <c r="G67" s="22" t="n">
         <v>46316</v>
       </c>
       <c r="H67" s="15" t="inlineStr">
@@ -3061,10 +3082,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F68" s="17" t="n">
+      <c r="F68" s="22" t="n">
         <v>46316</v>
       </c>
-      <c r="G68" s="17" t="n">
+      <c r="G68" s="22" t="n">
         <v>46317</v>
       </c>
       <c r="H68" s="15" t="inlineStr">
@@ -3099,10 +3120,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F69" s="17" t="n">
+      <c r="F69" s="22" t="n">
         <v>46317</v>
       </c>
-      <c r="G69" s="17" t="n">
+      <c r="G69" s="22" t="n">
         <v>46317</v>
       </c>
       <c r="H69" s="15" t="inlineStr">
@@ -3137,10 +3158,10 @@
           <t>Sans objet</t>
         </is>
       </c>
-      <c r="F70" s="17" t="n">
+      <c r="F70" s="22" t="n">
         <v>46317</v>
       </c>
-      <c r="G70" s="17" t="n">
+      <c r="G70" s="22" t="n">
         <v>46317</v>
       </c>
       <c r="H70" s="15" t="inlineStr">
@@ -3150,18 +3171,18 @@
       </c>
     </row>
     <row r="72" ht="20" customHeight="1">
-      <c r="A72" s="12" t="inlineStr">
+      <c r="A72" s="23" t="inlineStr">
         <is>
           <t>11. MODÈLES D'IMPORT — refléter exactement les champs de la plateforme</t>
         </is>
       </c>
-      <c r="B72" s="13" t="n"/>
-      <c r="C72" s="13" t="n"/>
-      <c r="D72" s="13" t="n"/>
-      <c r="E72" s="13" t="n"/>
-      <c r="F72" s="13" t="n"/>
-      <c r="G72" s="13" t="n"/>
-      <c r="H72" s="13" t="n"/>
+      <c r="B72" s="21" t="n"/>
+      <c r="C72" s="21" t="n"/>
+      <c r="D72" s="21" t="n"/>
+      <c r="E72" s="21" t="n"/>
+      <c r="F72" s="21" t="n"/>
+      <c r="G72" s="21" t="n"/>
+      <c r="H72" s="21" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="14" t="inlineStr">
@@ -3189,10 +3210,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F73" s="17" t="n">
+      <c r="F73" s="22" t="n">
         <v>46318</v>
       </c>
-      <c r="G73" s="17" t="n">
+      <c r="G73" s="22" t="n">
         <v>46318</v>
       </c>
       <c r="H73" s="15" t="inlineStr">
@@ -3227,10 +3248,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F74" s="17" t="n">
+      <c r="F74" s="22" t="n">
         <v>46318</v>
       </c>
-      <c r="G74" s="17" t="n">
+      <c r="G74" s="22" t="n">
         <v>46318</v>
       </c>
       <c r="H74" s="15" t="inlineStr">
@@ -3265,10 +3286,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F75" s="17" t="n">
+      <c r="F75" s="22" t="n">
         <v>46318</v>
       </c>
-      <c r="G75" s="17" t="n">
+      <c r="G75" s="22" t="n">
         <v>46318</v>
       </c>
       <c r="H75" s="15" t="inlineStr">
@@ -3303,10 +3324,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F76" s="17" t="n">
+      <c r="F76" s="22" t="n">
         <v>46318</v>
       </c>
-      <c r="G76" s="17" t="n">
+      <c r="G76" s="22" t="n">
         <v>46318</v>
       </c>
       <c r="H76" s="15" t="inlineStr">
@@ -3316,18 +3337,18 @@
       </c>
     </row>
     <row r="78" ht="20" customHeight="1">
-      <c r="A78" s="12" t="inlineStr">
+      <c r="A78" s="23" t="inlineStr">
         <is>
           <t>12. PERFORMANCE — l'application est lente</t>
         </is>
       </c>
-      <c r="B78" s="13" t="n"/>
-      <c r="C78" s="13" t="n"/>
-      <c r="D78" s="13" t="n"/>
-      <c r="E78" s="13" t="n"/>
-      <c r="F78" s="13" t="n"/>
-      <c r="G78" s="13" t="n"/>
-      <c r="H78" s="13" t="n"/>
+      <c r="B78" s="21" t="n"/>
+      <c r="C78" s="21" t="n"/>
+      <c r="D78" s="21" t="n"/>
+      <c r="E78" s="21" t="n"/>
+      <c r="F78" s="21" t="n"/>
+      <c r="G78" s="21" t="n"/>
+      <c r="H78" s="21" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="14" t="inlineStr">
@@ -3355,10 +3376,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F79" s="17" t="n">
+      <c r="F79" s="22" t="n">
         <v>46321</v>
       </c>
-      <c r="G79" s="17" t="n">
+      <c r="G79" s="22" t="n">
         <v>46321</v>
       </c>
       <c r="H79" s="15" t="inlineStr">
@@ -3393,10 +3414,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F80" s="17" t="n">
+      <c r="F80" s="22" t="n">
         <v>46321</v>
       </c>
-      <c r="G80" s="17" t="n">
+      <c r="G80" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="H80" s="15" t="inlineStr">
@@ -3431,10 +3452,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F81" s="17" t="n">
+      <c r="F81" s="22" t="n">
         <v>46322</v>
       </c>
-      <c r="G81" s="17" t="n">
+      <c r="G81" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="H81" s="15" t="inlineStr">
@@ -3469,10 +3490,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F82" s="17" t="n">
+      <c r="F82" s="22" t="n">
         <v>46322</v>
       </c>
-      <c r="G82" s="17" t="n">
+      <c r="G82" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="H82" s="15" t="inlineStr">
@@ -3482,18 +3503,18 @@
       </c>
     </row>
     <row r="84" ht="20" customHeight="1">
-      <c r="A84" s="12" t="inlineStr">
+      <c r="A84" s="23" t="inlineStr">
         <is>
           <t>13. CONDUITE DU CHANTIER</t>
         </is>
       </c>
-      <c r="B84" s="13" t="n"/>
-      <c r="C84" s="13" t="n"/>
-      <c r="D84" s="13" t="n"/>
-      <c r="E84" s="13" t="n"/>
-      <c r="F84" s="13" t="n"/>
-      <c r="G84" s="13" t="n"/>
-      <c r="H84" s="13" t="n"/>
+      <c r="B84" s="21" t="n"/>
+      <c r="C84" s="21" t="n"/>
+      <c r="D84" s="21" t="n"/>
+      <c r="E84" s="21" t="n"/>
+      <c r="F84" s="21" t="n"/>
+      <c r="G84" s="21" t="n"/>
+      <c r="H84" s="21" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="14" t="inlineStr">
@@ -3521,10 +3542,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F85" s="17" t="n">
+      <c r="F85" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G85" s="17" t="n">
+      <c r="G85" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="H85" s="15" t="inlineStr">
@@ -3559,10 +3580,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F86" s="17" t="n">
+      <c r="F86" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G86" s="17" t="n">
+      <c r="G86" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="H86" s="15" t="inlineStr">
@@ -3597,10 +3618,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F87" s="17" t="n">
+      <c r="F87" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G87" s="17" t="n">
+      <c r="G87" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="H87" s="15" t="inlineStr">
@@ -3635,10 +3656,10 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="F88" s="17" t="n">
+      <c r="F88" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G88" s="17" t="n">
+      <c r="G88" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H88" s="15" t="inlineStr">
@@ -3648,18 +3669,18 @@
       </c>
     </row>
     <row r="89" ht="20" customHeight="1">
-      <c r="A89" s="12" t="inlineStr">
+      <c r="A89" s="23" t="inlineStr">
         <is>
           <t>14. TROUVÉ EN CHEMIN — relevé pendant le chantier 1, le 02/10/2026</t>
         </is>
       </c>
-      <c r="B89" s="13" t="n"/>
-      <c r="C89" s="13" t="n"/>
-      <c r="D89" s="13" t="n"/>
-      <c r="E89" s="13" t="n"/>
-      <c r="F89" s="13" t="n"/>
-      <c r="G89" s="13" t="n"/>
-      <c r="H89" s="13" t="n"/>
+      <c r="B89" s="21" t="n"/>
+      <c r="C89" s="21" t="n"/>
+      <c r="D89" s="21" t="n"/>
+      <c r="E89" s="21" t="n"/>
+      <c r="F89" s="21" t="n"/>
+      <c r="G89" s="21" t="n"/>
+      <c r="H89" s="21" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
@@ -3687,10 +3708,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F90" s="17" t="n">
+      <c r="F90" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G90" s="17" t="n">
+      <c r="G90" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H90" s="15" t="inlineStr">
@@ -3725,10 +3746,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F91" s="17" t="n">
+      <c r="F91" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G91" s="17" t="n">
+      <c r="G91" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H91" s="15" t="inlineStr">
@@ -3763,10 +3784,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F92" s="17" t="n">
+      <c r="F92" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G92" s="17" t="n">
+      <c r="G92" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H92" s="15" t="inlineStr">
@@ -3801,10 +3822,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F93" s="17" t="n">
+      <c r="F93" s="22" t="n">
         <v>46297</v>
       </c>
-      <c r="G93" s="17" t="n">
+      <c r="G93" s="22" t="n">
         <v>46297</v>
       </c>
       <c r="H93" s="15" t="inlineStr">
@@ -3814,18 +3835,18 @@
       </c>
     </row>
     <row r="94" ht="20" customHeight="1">
-      <c r="A94" s="12" t="inlineStr">
+      <c r="A94" s="23" t="inlineStr">
         <is>
           <t>15. LA LIVRAISON — relevé le 05/10/2026</t>
         </is>
       </c>
-      <c r="B94" s="13" t="n"/>
-      <c r="C94" s="13" t="n"/>
-      <c r="D94" s="13" t="n"/>
-      <c r="E94" s="13" t="n"/>
-      <c r="F94" s="13" t="n"/>
-      <c r="G94" s="13" t="n"/>
-      <c r="H94" s="13" t="n"/>
+      <c r="B94" s="21" t="n"/>
+      <c r="C94" s="21" t="n"/>
+      <c r="D94" s="21" t="n"/>
+      <c r="E94" s="21" t="n"/>
+      <c r="F94" s="21" t="n"/>
+      <c r="G94" s="21" t="n"/>
+      <c r="H94" s="21" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="14" t="inlineStr">
@@ -3853,10 +3874,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F95" s="17" t="n">
+      <c r="F95" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G95" s="17" t="n">
+      <c r="G95" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H95" s="15" t="inlineStr">
@@ -3891,10 +3912,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F96" s="17" t="n">
+      <c r="F96" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G96" s="17" t="n">
+      <c r="G96" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H96" s="15" t="inlineStr">
@@ -3929,10 +3950,10 @@
           <t>À trancher</t>
         </is>
       </c>
-      <c r="F97" s="17" t="n">
+      <c r="F97" s="22" t="n">
         <v>46301</v>
       </c>
-      <c r="G97" s="17" t="n">
+      <c r="G97" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="H97" s="15" t="inlineStr">
@@ -3967,10 +3988,10 @@
           <t>Terminé</t>
         </is>
       </c>
-      <c r="F98" s="17" t="n">
+      <c r="F98" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G98" s="17" t="n">
+      <c r="G98" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H98" s="15" t="inlineStr">
@@ -3980,18 +4001,18 @@
       </c>
     </row>
     <row r="100" ht="20" customHeight="1">
-      <c r="A100" s="12" t="inlineStr">
+      <c r="A100" s="23" t="inlineStr">
         <is>
           <t>16. LES ÉCRITURES D'ACHAT VENUES DE LA DGI — règles en vigueur</t>
         </is>
       </c>
-      <c r="B100" s="13" t="n"/>
-      <c r="C100" s="13" t="n"/>
-      <c r="D100" s="13" t="n"/>
-      <c r="E100" s="13" t="n"/>
-      <c r="F100" s="13" t="n"/>
-      <c r="G100" s="13" t="n"/>
-      <c r="H100" s="13" t="n"/>
+      <c r="B100" s="21" t="n"/>
+      <c r="C100" s="21" t="n"/>
+      <c r="D100" s="21" t="n"/>
+      <c r="E100" s="21" t="n"/>
+      <c r="F100" s="21" t="n"/>
+      <c r="G100" s="21" t="n"/>
+      <c r="H100" s="21" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="14" t="inlineStr">
@@ -4019,10 +4040,10 @@
           <t>Sans objet</t>
         </is>
       </c>
-      <c r="F101" s="17" t="n">
+      <c r="F101" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G101" s="17" t="n">
+      <c r="G101" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H101" s="15" t="inlineStr">
@@ -4057,10 +4078,10 @@
           <t>Sans objet</t>
         </is>
       </c>
-      <c r="F102" s="17" t="n">
+      <c r="F102" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G102" s="17" t="n">
+      <c r="G102" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H102" s="15" t="inlineStr">
@@ -4095,10 +4116,10 @@
           <t>Sans objet</t>
         </is>
       </c>
-      <c r="F103" s="17" t="n">
+      <c r="F103" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G103" s="17" t="n">
+      <c r="G103" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H103" s="15" t="inlineStr">
@@ -4133,10 +4154,10 @@
           <t>Sans objet</t>
         </is>
       </c>
-      <c r="F104" s="17" t="n">
+      <c r="F104" s="22" t="n">
         <v>46300</v>
       </c>
-      <c r="G104" s="17" t="n">
+      <c r="G104" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="H104" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Lot 42 : les comptes se saisissent une fois, et non par produit
Sections 3.3, 3.6, 5 et 6 du plan.

- ImputationService porte l'ordre de priorite unique : exception de
  l'article (case cochee) > type > categorie > configuration generale >
  defaut ; et les tiers (411000 / 401000), lus jusqu'ici a dix endroits.
- Nouvelle page Configuration comptable (generale, par categorie, par
  type, stock et variations), derriere le garde-fou comptabilite ; chaque
  compte est relu au plan et a la classe.
- Fiche produit : plus aucun compte comptabilite fermee ; ouverte,
  "herite de la configuration globale" et une case d'exception.
- Migration : la reprise de l'existant ne coche que ce qui differe du
  defaut et de la categorie ; rien n'est efface.
- Les immobilisations passent derriere le garde-fou comptabilite.

Suite : 1 479 epreuves, 1 474 passantes, 5 sautees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -735,10 +735,10 @@
         <v>6</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E7" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F7" s="15" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -795,10 +795,10 @@
         <v>2</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F9" s="15" t="n">
         <v>0</v>
@@ -808,7 +808,7 @@
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -825,10 +825,10 @@
         <v>5</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F10" s="15" t="n">
         <v>0</v>
@@ -838,7 +838,7 @@
       </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -1152,10 +1152,10 @@
         <v>71</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="F22" s="10" t="n">
         <v>1</v>
@@ -1410,6 +1410,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="23" t="inlineStr">
         <is>
@@ -1690,6 +1691,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="23" t="inlineStr">
         <is>
@@ -1798,12 +1800,12 @@
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>Deux menus obligatoires sur la création, la modification en ligne et la fiche. Ils disparaissent quand la comptabilité est éteinte ; le serveur pose 701000 et 601000. Quand elle est allumée, ils ne reviennent pas tels quels : voir le chantier 6 (configuration globale).</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Deux menus obligatoires sur la création, la modification en ligne et la fiche. Ils disparaissent quand la comptabilité est éteinte ; le serveur pose 701000 et 601000. Quand elle est allumée, ils ne reviennent pas tels quels : voir le chantier 6 (configuration globale). FAIT au lot 42 avec la section 6 : fermée, rien n'est demandé ni accepté ; ouverte, l'article hérite et une case en fait une exception.</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F23" s="22" t="n">
@@ -1912,12 +1914,12 @@
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>Comptabilité éteinte = aucun écran, aucun champ, aucun lien comptable. Une épreuve parcourt les routes et les vues pour l'établir, plutôt qu'une relecture à l'œil.</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Comptabilité éteinte = aucun écran, aucun champ, aucun lien comptable. Une épreuve parcourt les routes et les vues pour l'établir, plutôt qu'une relecture à l'œil. FAIT au lot 42 : ConfigurationComptableTest cherche douze marques comptables sur clients, fournisseurs, catalogue et fiche. TROUVÉ : les immobilisations restaient ouvertes à tous ; elles passent derrière le garde-fou.</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F26" s="22" t="n">
@@ -1932,6 +1934,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="23" t="inlineStr">
         <is>
@@ -2098,6 +2101,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="23" t="inlineStr">
         <is>
@@ -2130,19 +2134,19 @@
       </c>
       <c r="D35" s="14" t="inlineStr">
         <is>
-          <t>Vente, achat, avoir, règlement : chaque événement continue de produire son écriture et de l'enregistrer, comptabilité activée ou non. C'est ce qui permet d'allumer la comptabilité six mois plus tard et d'avoir les livres complets — et c'est ce que Comptaflow reçoit. La page « Opération &amp; écriture globale » reste alimentée ; elle est seulement masquée.</t>
-        </is>
-      </c>
-      <c r="E35" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Vente, achat, avoir, règlement : chaque événement continue de produire son écriture et de l'enregistrer, comptabilité activée ou non. C'est ce qui permet d'allumer la comptabilité six mois plus tard et d'avoir les livres complets — et c'est ce que Comptaflow reçoit. La page « Opération &amp; écriture globale » reste alimentée ; elle est seulement masquée. FAIT : la suite des écritures tourne déjà sur des entreprises à comptabilité fermée (défaut depuis le lot 39).</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F35" s="22" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="G35" s="22" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="H35" s="15" t="inlineStr">
         <is>
@@ -2168,19 +2172,19 @@
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
-          <t>Quand l'utilisateur ne voit aucun champ de compte, le serveur doit en choisir un qui tienne. ORDRE DE PRIORITÉ, écrit une fois dans un service et non recopié sur chaque écran : (1) exception portée par le produit ; (2) configuration globale (chantier 6) ; (3) compte de la famille ; (4) défaut 701000 à la vente, 601000 à l'achat. ET LES TIERS, ajoutés le 05/10/2026 à la demande du propriétaire : le client porte 411000, le fournisseur 401000 — le compte collectif de sa nature. Les oublier laisserait chaque écriture de vente ou d'achat sans contrepartie de tiers, et c'est précisément ce que le numéro de tiers sert à subdiviser chez Comptaflow.</t>
-        </is>
-      </c>
-      <c r="E36" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Quand l'utilisateur ne voit aucun champ de compte, le serveur doit en choisir un qui tienne. ORDRE DE PRIORITÉ, écrit une fois dans un service et non recopié sur chaque écran : (1) exception portée par le produit ; (2) configuration globale (chantier 6) ; (3) compte de la famille ; (4) défaut 701000 à la vente, 601000 à l'achat. ET LES TIERS, ajoutés le 05/10/2026 à la demande du propriétaire : le client porte 411000, le fournisseur 401000 — le compte collectif de sa nature. Les oublier laisserait chaque écriture de vente ou d'achat sans contrepartie de tiers, et c'est précisément ce que le numéro de tiers sert à subdiviser chez Comptaflow. FAIT au lot 42 : ImputationService — exception (case cochée) &gt; type &gt; catégorie (famille) &gt; générale &gt; défaut ; compteClient / compteFournisseur remplacent dix lectures dispersées. Écart assumé : la configuration générale passe APRÈS la catégorie, qui porte la famille — voir journal 42.1.</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F36" s="22" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="G36" s="22" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="H36" s="15" t="inlineStr">
         <is>
@@ -2188,6 +2192,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="23" t="inlineStr">
         <is>
@@ -2223,16 +2228,16 @@
           <t>Une page unique qui remplace la saisie d'un compte sur chaque fiche produit. Deux sections : configuration vente, configuration achat.</t>
         </is>
       </c>
-      <c r="E39" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F39" s="22" t="n">
-        <v>46307</v>
+        <v>46302</v>
       </c>
       <c r="G39" s="22" t="n">
-        <v>46307</v>
+        <v>46302</v>
       </c>
       <c r="H39" s="15" t="inlineStr">
         <is>
@@ -2261,16 +2266,16 @@
           <t>(1) Configuration générale — deux champs : le compte de vente de tous les produits, le compte d'achat de tous les produits. (2) Configuration par catégorie — un couple de champs par catégorie. (3) Configuration par type — un couple par type (stockable, service, …). Le plus précis l'emporte : type, puis catégorie, puis général.</t>
         </is>
       </c>
-      <c r="E40" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F40" s="22" t="n">
-        <v>46307</v>
+        <v>46302</v>
       </c>
       <c r="G40" s="22" t="n">
-        <v>46308</v>
+        <v>46302</v>
       </c>
       <c r="H40" s="15" t="inlineStr">
         <is>
@@ -2299,16 +2304,16 @@
           <t>Les comptes de variation (6031/6032/6033, 736) et de stock (31/32/33/36) sont posés par le système. Une section les affiche : ce qui est fait, avec quels comptes, et permet de les changer. Rien n'est demandé — c'est une lecture qui accepte une correction.</t>
         </is>
       </c>
-      <c r="E41" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="E41" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F41" s="22" t="n">
-        <v>46308</v>
+        <v>46302</v>
       </c>
       <c r="G41" s="22" t="n">
-        <v>46308</v>
+        <v>46302</v>
       </c>
       <c r="H41" s="15" t="inlineStr">
         <is>
@@ -2337,16 +2342,16 @@
           <t>Dès que la configuration globale est renseignée, la fiche produit n'affiche plus de champ de compte mais la mention « hérite de la configuration globale », avec les comptes qui s'appliquent. Une case à cocher ouvre deux champs (vente, achat) : cochée, elle PRIME sur la configuration globale, parce qu'elle est portée par le produit lui-même. Décochée, le produit revient à l'héritage — et ne garde pas en silence l'ancienne valeur.</t>
         </is>
       </c>
-      <c r="E42" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F42" s="22" t="n">
-        <v>46308</v>
+        <v>46302</v>
       </c>
       <c r="G42" s="22" t="n">
-        <v>46308</v>
+        <v>46302</v>
       </c>
       <c r="H42" s="15" t="inlineStr">
         <is>
@@ -2372,19 +2377,19 @@
       </c>
       <c r="D43" s="14" t="inlineStr">
         <is>
-          <t>Les produits portent déjà des comptes. Ceux qui diffèrent du défaut (701000 / 601000) sont réputés voulus : ils basculent en exception cochée. Les autres passent en héritage. Sans cette règle, l'arrivée de la configuration globale réécrirait des imputations choisies.</t>
-        </is>
-      </c>
-      <c r="E43" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Les produits portent déjà des comptes. Ceux qui diffèrent du défaut (701000 / 601000) sont réputés voulus : ils basculent en exception cochée. Les autres passent en héritage. Sans cette règle, l'arrivée de la configuration globale réécrirait des imputations choisies. FAIT au lot 42 : défaut lu au pluriel (701000/701100, 601000/601100) ; un compte égal à celui de la catégorie n'est pas une exception ; rien n'est effacé.</t>
+        </is>
+      </c>
+      <c r="E43" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F43" s="22" t="n">
-        <v>46308</v>
+        <v>46302</v>
       </c>
       <c r="G43" s="22" t="n">
-        <v>46308</v>
+        <v>46302</v>
       </c>
       <c r="H43" s="15" t="inlineStr">
         <is>
@@ -2392,6 +2397,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="23" t="inlineStr">
         <is>
@@ -2596,6 +2602,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="23" t="inlineStr">
         <is>
@@ -2762,6 +2769,7 @@
         </is>
       </c>
     </row>
+    <row r="57"/>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="23" t="inlineStr">
         <is>
@@ -2928,6 +2936,7 @@
         </is>
       </c>
     </row>
+    <row r="63"/>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="23" t="inlineStr">
         <is>
@@ -3170,6 +3179,7 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="23" t="inlineStr">
         <is>
@@ -3336,6 +3346,7 @@
         </is>
       </c>
     </row>
+    <row r="77"/>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="23" t="inlineStr">
         <is>
@@ -3502,6 +3513,7 @@
         </is>
       </c>
     </row>
+    <row r="83"/>
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="23" t="inlineStr">
         <is>
@@ -4000,6 +4012,7 @@
         </is>
       </c>
     </row>
+    <row r="99"/>
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="23" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Lot 43 : le deversement Comptaflow, une operation une saisie
Section 7 du plan (7.1 a 7.4). Le pendant chez Comptaflow est la revision
b40b9bd de guysergekouassi/COMPTAFLOW.

- Diagnostic corrige : chaque ecriture Selflow porte deja un seul compte ;
  le defaut etait a la reception, ou n_saisie valait la cle_selflow de la
  ligne. Comptaflow numerote desormais une saisie par operation.
- L'operation repart entiere, lignes deja recues comprises ; un echec ne
  degrade plus ce qui etait confirme.
- Controle avant envoi : un compte par ligne, montant du bon cote,
  equilibre ; ce qui ne tombe pas reste chez nous en statut anomalie, et
  l'ecran de liaison le dit.
- selflow:sync-ecritures --all parcourt tout l'historique au lieu des
  cinquante memes premieres operations.

Suite : 1 484 epreuves, 1 479 passantes, 5 sautees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -855,10 +855,10 @@
         <v>5</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F11" s="15" t="n">
         <v>0</v>
@@ -868,7 +868,7 @@
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>4/5</t>
         </is>
       </c>
     </row>
@@ -1152,10 +1152,10 @@
         <v>71</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F22" s="10" t="n">
         <v>1</v>
@@ -2430,19 +2430,19 @@
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>DIAGNOSTIC POSÉ : `DeverserOperationComptaflow::ligne()` envoie `compte_debit`, `compte_credit`, `debit` et `credit` sur UNE SEULE ligne. C'est le modèle interne de Selflow ; Comptaflow attend une ligne par mouvement de compte. D'où la ligne unique par numéro de saisie et la balance qui ne tombe pas. PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : ce n'est PAS un simple dédoublement. Une vente avec TVA, timbre et remise fait plus de deux lignes, un règlement partiel aussi. Le déversement doit porter l'opération ENTIÈRE, et ses lignes doivent se retrouver groupées par leur référence — le numéro de saisie. C'est lui qui fait le couple, pas la position dans la liste.</t>
-        </is>
-      </c>
-      <c r="E46" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>DIAGNOSTIC POSÉ : `DeverserOperationComptaflow::ligne()` envoie `compte_debit`, `compte_credit`, `debit` et `credit` sur UNE SEULE ligne. C'est le modèle interne de Selflow ; Comptaflow attend une ligne par mouvement de compte. D'où la ligne unique par numéro de saisie et la balance qui ne tombe pas. PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : ce n'est PAS un simple dédoublement. Une vente avec TVA, timbre et remise fait plus de deux lignes, un règlement partiel aussi. Le déversement doit porter l'opération ENTIÈRE, et ses lignes doivent se retrouver groupées par leur référence — le numéro de saisie. C'est lui qui fait le couple, pas la position dans la liste. FAIT au lot 43 — DIAGNOSTIC CORRIGÉ : les lignes Selflow portent déjà un compte chacune ; le défaut était chez Comptaflow, qui écrivait n_saisie = cle_selflow (unique par ligne). Comptaflow b40b9bd attribue désormais un numéro de saisie par opération.</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F46" s="22" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="G46" s="22" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="H46" s="15" t="inlineStr">
         <is>
@@ -2468,19 +2468,19 @@
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>Relire ce que Comptaflow attend — nom des champs, sens du montant, journal, date, pièce, numéro de tiers, exercice — et s'y conformer sans rien lui dicter. Selflow envoie ; Comptaflow décide.</t>
-        </is>
-      </c>
-      <c r="E47" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Relire ce que Comptaflow attend — nom des champs, sens du montant, journal, date, pièce, numéro de tiers, exercice — et s'y conformer sans rien lui dicter. Selflow envoie ; Comptaflow décide. FAIT au lot 43 : contrat relu, tableau au journal ; Selflow renvoie l'opération entière, lignes déjà reçues comprises.</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F47" s="22" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="G47" s="22" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="H47" s="15" t="inlineStr">
         <is>
@@ -2506,19 +2506,19 @@
       </c>
       <c r="D48" s="14" t="inlineStr">
         <is>
-          <t>Somme des débits = somme des crédits, vérifiée avant l'envoi. Une opération qui ne tombe pas n'est pas envoyée : elle est signalée. Déverser un déséquilibre oblige à le chercher dans l'autre application, où l'on n'a pas la pièce d'origine.</t>
-        </is>
-      </c>
-      <c r="E48" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Somme des débits = somme des crédits, vérifiée avant l'envoi. Une opération qui ne tombe pas n'est pas envoyée : elle est signalée. Déverser un déséquilibre oblige à le chercher dans l'autre application, où l'on n'a pas la pièce d'origine. FAIT au lot 43 : DeverserOperationComptaflow::anomalie() — un compte par ligne, montant du bon côté, équilibre ; statut « anomalie » affiché à l'écran de liaison. Comptaflow refait le contrôle.</t>
+        </is>
+      </c>
+      <c r="E48" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F48" s="22" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="G48" s="22" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="H48" s="15" t="inlineStr">
         <is>
@@ -2544,19 +2544,19 @@
       </c>
       <c r="D49" s="14" t="inlineStr">
         <is>
-          <t>Les opérations déjà déversées sous l'ancienne forme sont à rejouer. Vérifier que le déversement est idempotent côté Comptaflow AVANT de rejouer quoi que ce soit — sinon la balance double.</t>
-        </is>
-      </c>
-      <c r="E49" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Les opérations déjà déversées sous l'ancienne forme sont à rejouer. Vérifier que le déversement est idempotent côté Comptaflow AVANT de rejouer quoi que ce soit — sinon la balance double. FAIT au lot 43 : idempotence vérifiée côté Comptaflow (DeversementEcrituresTest) ; les lignes de l'ancienne forme se regroupent au renvoi ; --all parcourt tout l'historique. Ordre de déploiement : Comptaflow, Selflow, puis selflow:sync-ecritures --all.</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F49" s="22" t="n">
-        <v>46310</v>
+        <v>46302</v>
       </c>
       <c r="G49" s="22" t="n">
-        <v>46310</v>
+        <v>46302</v>
       </c>
       <c r="H49" s="15" t="inlineStr">
         <is>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>Une vente, un achat, un avoir, un règlement — puis relire la balance chez Comptaflow. La vérification se fait sur la plateforme, pas seulement sur les épreuves.</t>
+          <t>Une vente, un achat, un avoir, un règlement — puis relire la balance chez Comptaflow. La vérification se fait sur la plateforme, pas seulement sur les épreuves. NON FAIT — demande les plateformes déployées, inaccessibles depuis la session du 07/10/2026.</t>
         </is>
       </c>
       <c r="E50" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Lot 44 : un avoir ne rend pas plus que la facture
Section 8 du plan (8.1 a 8.3 ; 8.4 a trancher).

- Plafond en montant au serveur, dans la transaction et sur la facture
  relue verrouillee : le plafond en quantite laissait passer un prix
  releve a la main et les lignes ajoutees a l'avoir.
- L'avoir total refuse une facture qui porte deja un avoir.
- Le compteur des quantites deja creditees ignorait les avoirs d'une
  autre periode (filtre global de Vente).
- Les factures entierement avoirees sortent de la liste et de la
  recherche ; les autres annoncent leur reste.
- L'avoir de BAPA reste ferme (DGI, perimetre FNE gele) : question posee
  au proprietaire, consignee au journal.

Suite : 1 491 epreuves, 1 486 passantes, 5 sautees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -885,20 +885,20 @@
         <v>4</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>3/4</t>
         </is>
       </c>
     </row>
@@ -1152,13 +1152,13 @@
         <v>71</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" s="10" t="n">
         <v>5</v>
@@ -2635,19 +2635,19 @@
       </c>
       <c r="D53" s="14" t="inlineStr">
         <is>
-          <t>RÉPONSE À VOTRE QUESTION : non, un avoir ne doit pas pouvoir dépasser la valeur de la pièce d'origine — cela reviendrait à rendre plus que ce qui a été facturé, et la TVA collectée deviendrait négative sur la pièce. Contrôle au serveur, pas seulement à l'écran : somme des avoirs déjà établis + avoir en cours ≤ total de la facture. VALIDÉ par le propriétaire le 2 octobre 2026.</t>
-        </is>
-      </c>
-      <c r="E53" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>RÉPONSE À VOTRE QUESTION : non, un avoir ne doit pas pouvoir dépasser la valeur de la pièce d'origine — cela reviendrait à rendre plus que ce qui a été facturé, et la TVA collectée deviendrait négative sur la pièce. Contrôle au serveur, pas seulement à l'écran : somme des avoirs déjà établis + avoir en cours ≤ total de la facture. VALIDÉ par le propriétaire le 2 octobre 2026. FAIT au lot 44 : plafond en MONTANT dans la transaction, facture relue verrouillée ; l'avoir total refuse une facture déjà avoirée. TROUVÉ : le compteur des quantités déjà créditées passait par le filtre de période.</t>
+        </is>
+      </c>
+      <c r="E53" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F53" s="22" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="G53" s="22" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="H53" s="15" t="inlineStr">
         <is>
@@ -2673,19 +2673,19 @@
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
-          <t>Une facture entièrement avoirée n'a plus rien à rendre : elle sort de la liste déroulante et du champ de recherche. La proposer mène à un refus qu'on ne comprend qu'après coup.</t>
-        </is>
-      </c>
-      <c r="E54" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Une facture entièrement avoirée n'a plus rien à rendre : elle sort de la liste déroulante et du champ de recherche. La proposer mène à un refus qu'on ne comprend qu'après coup. FAIT au lot 44 : Vente::scopeEncoreAvoirables(), liste et recherche.</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F54" s="22" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="G54" s="22" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="H54" s="15" t="inlineStr">
         <is>
@@ -2711,19 +2711,19 @@
       </c>
       <c r="D55" s="14" t="inlineStr">
         <is>
-          <t>Celles qui portent déjà un avoir sans atteindre le total restent proposées, avec la mention du reste à avoirer — « reste 45 000 F sur 120 000 F ». Sans cette mention, on saisit un montant au jugé et on se fait refuser.</t>
-        </is>
-      </c>
-      <c r="E55" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Celles qui portent déjà un avoir sans atteindre le total restent proposées, avec la mention du reste à avoirer — « reste 45 000 F sur 120 000 F ». Sans cette mention, on saisit un montant au jugé et on se fait refuser. FAIT au lot 44 : « reste 88 500 F sur 118 000 F » dans la liste, la recherche et la fenêtre d'avoir.</t>
+        </is>
+      </c>
+      <c r="E55" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F55" s="22" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="G55" s="22" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="H55" s="15" t="inlineStr">
         <is>
@@ -2749,16 +2749,16 @@
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : l'avoir fournisseur ne concerne QUE les BAPA — les bordereaux d'achat auprès d'un particulier, que Selflow émet et que la DGI certifie. Un achat ordinaire est une pièce du fournisseur, pas de nous : on ne l'avoire pas, on demande au fournisseur son propre avoir. Le contrôle de dépassement s'applique donc au BAPA, et l'écran ne doit pas proposer d'avoir sur les autres achats.</t>
-        </is>
-      </c>
-      <c r="E56" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : l'avoir fournisseur ne concerne QUE les BAPA — les bordereaux d'achat auprès d'un particulier, que Selflow émet et que la DGI certifie. Un achat ordinaire est une pièce du fournisseur, pas de nous : on ne l'avoire pas, on demande au fournisseur son propre avoir. Le contrôle de dépassement s'applique donc au BAPA, et l'écran ne doit pas proposer d'avoir sur les autres achats. À TRANCHER (07/10/2026) : aucun écran ne propose d'avoir sur un achat ordinaire (retiré le 25/09). Mais l'avoir de BAPA est fermé depuis le lot 23 parce que la DGI ne le normalise pas ; l'ouvrir toucherait FneService (gelé). Question au propriétaire : la plateforme l'accepte-t-elle désormais ?</t>
+        </is>
+      </c>
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>À trancher</t>
         </is>
       </c>
       <c r="F56" s="22" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="G56" s="22" t="n">
         <v>46311</v>

</xml_diff>

<commit_message>
Lot 45 : les ecrans d'entree
Section 9 du plan.

- Les six pages publiques chargeaient Tabler Icons en version flottante :
  carre vide a la place des fleches de l'inscription. Font Awesome 6.5.0
  epingle, comme le reste de l'application.
- Un oeil sur la confirmation du mot de passe, et les deux basculent
  ensemble.
- Creation d'un point de vente : 3 001 requetes pour 1 500 articles (un
  firstOrCreate par article), desormais 5. Le bouton s'annonce.
- La visite guidee ouvre la section repliee ou la barre du telephone qui
  cache sa cible, puis la referme ; elle ne promet plus de plan comptable
  quand la comptabilite est fermee.

Suite : 1 498 epreuves, 1 493 passantes, 5 sautees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -915,10 +915,10 @@
         <v>4</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F13" s="15" t="n">
         <v>0</v>
@@ -928,7 +928,7 @@
       </c>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -1152,10 +1152,10 @@
         <v>71</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F22" s="10" t="n">
         <v>2</v>
@@ -2802,19 +2802,19 @@
       </c>
       <c r="D59" s="14" t="inlineStr">
         <is>
-          <t>Les boutons « Retour », « Suivant » et « Terminer sans remplir la suite » montrent un carré vide à la place de leur icône : la police d'icônes n'est pas chargée sur la page publique, ou le glyphe n'existe pas dans la version servie. À corriger à la source — une icône absente sur la toute première page donne le ton du reste.</t>
-        </is>
-      </c>
-      <c r="E59" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Les boutons « Retour », « Suivant » et « Terminer sans remplir la suite » montrent un carré vide à la place de leur icône : la police d'icônes n'est pas chargée sur la page publique, ou le glyphe n'existe pas dans la version servie. À corriger à la source — une icône absente sur la toute première page donne le ton du reste. FAIT au lot 45 : les six pages publiques chargeaient Tabler Icons en version flottante ; Font Awesome 6.5.0 épinglé (cdnjs), comme le reste de l'application.</t>
+        </is>
+      </c>
+      <c r="E59" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F59" s="22" t="n">
-        <v>46314</v>
+        <v>46302</v>
       </c>
       <c r="G59" s="22" t="n">
-        <v>46314</v>
+        <v>46302</v>
       </c>
       <c r="H59" s="15" t="inlineStr">
         <is>
@@ -2840,19 +2840,19 @@
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
-          <t>Le champ « Mot de passe » porte un œil, « Confirmer le mot de passe » n'en a pas. Les deux doivent en porter un, et les deux doivent basculer ensemble : on compare deux saisies, on ne peut pas les comparer si une seule est lisible.</t>
-        </is>
-      </c>
-      <c r="E60" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Le champ « Mot de passe » porte un œil, « Confirmer le mot de passe » n'en a pas. Les deux doivent en porter un, et les deux doivent basculer ensemble : on compare deux saisies, on ne peut pas les comparer si une seule est lisible. FAIT au lot 45.</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F60" s="22" t="n">
-        <v>46314</v>
+        <v>46302</v>
       </c>
       <c r="G60" s="22" t="n">
-        <v>46314</v>
+        <v>46302</v>
       </c>
       <c r="H60" s="15" t="inlineStr">
         <is>
@@ -2878,19 +2878,19 @@
       </c>
       <c r="D61" s="14" t="inlineStr">
         <is>
-          <t>Entre le clic sur « Créer » et la réponse, l'écran reste figé sans rien dire. Chercher la cause avant d'ajouter un sablier : création du stock d'ouverture pour tout le catalogue à chaque nouveau site, appel réseau synchrone, ou index manquant. Ce qui peut attendre part en file ; le bouton se désactive et annonce ce qui se passe.</t>
-        </is>
-      </c>
-      <c r="E61" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Entre le clic sur « Créer » et la réponse, l'écran reste figé sans rien dire. Chercher la cause avant d'ajouter un sablier : création du stock d'ouverture pour tout le catalogue à chaque nouveau site, appel réseau synchrone, ou index manquant. Ce qui peut attendre part en file ; le bouton se désactive et annonce ce qui se passe. FAIT au lot 45 — MESURÉ : 3 001 requêtes pour 1 500 articles (un firstOrCreate par article) ; désormais 5 requêtes, 37 ms. Bouton désactivé et annoncé.</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F61" s="22" t="n">
-        <v>46314</v>
+        <v>46302</v>
       </c>
       <c r="G61" s="22" t="n">
-        <v>46314</v>
+        <v>46302</v>
       </c>
       <c r="H61" s="15" t="inlineStr">
         <is>
@@ -2916,19 +2916,19 @@
       </c>
       <c r="D62" s="14" t="inlineStr">
         <is>
-          <t>L'étape 3 sur 7 parle du catalogue alors que la section n'est pas à l'écran. La visite doit lire la barre latérale réelle — modules actifs, habilitations, comptabilité activée — et sauter ce qui n'existe pas pour cet utilisateur. À reprendre APRÈS le chantier 1 (dépliage) et le chantier 2 (masquage), qui changent tous deux ce qui est visible.</t>
-        </is>
-      </c>
-      <c r="E62" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>L'étape 3 sur 7 parle du catalogue alors que la section n'est pas à l'écran. La visite doit lire la barre latérale réelle — modules actifs, habilitations, comptabilité activée — et sauter ce qui n'existe pas pour cet utilisateur. À reprendre APRÈS le chantier 1 (dépliage) et le chantier 2 (masquage), qui changent tous deux ce qui est visible. FAIT au lot 45 : la visite ouvre la section repliée ou la barre du téléphone qui cache sa cible, puis la referme ; ne promet plus de plan comptable quand la comptabilité est fermée.</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F62" s="22" t="n">
-        <v>46315</v>
+        <v>46302</v>
       </c>
       <c r="G62" s="22" t="n">
-        <v>46315</v>
+        <v>46302</v>
       </c>
       <c r="H62" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Lot 47 : les modeles d'import refletent les ecrans
Section 11 du plan.

- Clients et fournisseurs : numero_tiers retire et ignore ; le compte
  collectif ne figure au modele, et n'est lu, que comptabilite ouverte.
- Articles : les quatre comptes retires et ignores ; l'article importe
  herite de la configuration comptable globale.
- Immobilisations : pas de modele sans comptabilite.
- ModelesDImportTest compare chaque colonne aux champs des ecrans. Il a
  trouve que le prix de consignation et le delai de retour ne se
  saisissaient nulle part : ils rejoignent la fiche produit.

Suite : 1 512 epreuves, 1 507 passantes, 5 sautees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -975,10 +975,10 @@
         <v>4</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>0</v>
@@ -988,7 +988,7 @@
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -1152,10 +1152,10 @@
         <v>71</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F22" s="10" t="n">
         <v>2</v>
@@ -3212,19 +3212,19 @@
       </c>
       <c r="D73" s="14" t="inlineStr">
         <is>
-          <t>Reprendre les sept modèles (points de vente, clients, fournisseurs, utilisateurs, articles, stock initial, immobilisations) et les confronter aux formulaires. Toute colonne qui ne correspond à aucun champ saisissable disparaît : un modèle qui promet une colonne que rien ne lit fait saisir pour rien, et laisse croire que la donnée est entrée.</t>
-        </is>
-      </c>
-      <c r="E73" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Reprendre les sept modèles (points de vente, clients, fournisseurs, utilisateurs, articles, stock initial, immobilisations) et les confronter aux formulaires. Toute colonne qui ne correspond à aucun champ saisissable disparaît : un modèle qui promet une colonne que rien ne lit fait saisir pour rien, et laisse croire que la donnée est entrée. FAIT au lot 47. TROUVÉ : prix de consignation et délai de retour ne se saisissaient nulle part (l'import était la seule porte) ; ajoutés à la fiche produit.</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F73" s="22" t="n">
-        <v>46318</v>
+        <v>46302</v>
       </c>
       <c r="G73" s="22" t="n">
-        <v>46318</v>
+        <v>46302</v>
       </c>
       <c r="H73" s="15" t="inlineStr">
         <is>
@@ -3250,19 +3250,19 @@
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>Conséquence des chantiers 3.1 et 3.2 : le modèle ne doit pas demander un compte qui n'est plus proposé à l'écran, ni un numéro de tiers devenu automatique.</t>
-        </is>
-      </c>
-      <c r="E74" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Conséquence des chantiers 3.1 et 3.2 : le modèle ne doit pas demander un compte qui n'est plus proposé à l'écran, ni un numéro de tiers devenu automatique. FAIT au lot 47 : numero_tiers retiré et ignoré ; compte_comptable seulement comptabilité ouverte.</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F74" s="22" t="n">
-        <v>46318</v>
+        <v>46302</v>
       </c>
       <c r="G74" s="22" t="n">
-        <v>46318</v>
+        <v>46302</v>
       </c>
       <c r="H74" s="15" t="inlineStr">
         <is>
@@ -3288,19 +3288,19 @@
       </c>
       <c r="D75" s="14" t="inlineStr">
         <is>
-          <t>Même raison : ils viennent de la configuration globale (chantier 6), plus d'une saisie par ligne de classeur.</t>
-        </is>
-      </c>
-      <c r="E75" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Même raison : ils viennent de la configuration globale (chantier 6), plus d'une saisie par ligne de classeur. FAIT au lot 47 : les quatre comptes retirés et ignorés ; l'article importé hérite de la configuration globale.</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F75" s="22" t="n">
-        <v>46318</v>
+        <v>46302</v>
       </c>
       <c r="G75" s="22" t="n">
-        <v>46318</v>
+        <v>46302</v>
       </c>
       <c r="H75" s="15" t="inlineStr">
         <is>
@@ -3326,19 +3326,19 @@
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>Une épreuve qui compare les colonnes annoncées aux champs acceptés, pour que le prochain champ retiré d'un écran ne reste pas dans un modèle.</t>
-        </is>
-      </c>
-      <c r="E76" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Une épreuve qui compare les colonnes annoncées aux champs acceptés, pour que le prochain champ retiré d'un écran ne reste pas dans un modèle. FAIT au lot 47 : ModelesDImportTest compare chaque colonne aux champs des écrans, comptabilité fermée puis ouverte.</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F76" s="22" t="n">
-        <v>46318</v>
+        <v>46302</v>
       </c>
       <c r="G76" s="22" t="n">
-        <v>46318</v>
+        <v>46302</v>
       </c>
       <c r="H76" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Lot 53 : le transport d'une livraison
Chantier 15.3, tranche par le proprietaire le 07/10/2026 : tout est
obligatoire, et le bon imprime le porte.

- Au depart : adresse, livreur (personnel choisi dans l'entreprise, ou
  prestataire nomme), vehicule, heure. A l'arrivee : heure, receptionnaire,
  signature tracee a l'ecran, observations. TransportLivraisonService porte
  les deux jeux de regles pour les deux chemins qui expedient.
- La file Livraisons du stock sortait la marchandise sans etablir de bon :
  elle en etablit un desormais.
- Les quantites du bon etaient des entiers ; elles passent en decimal(15,3)
  par une nouvelle migration.
- Le bon imprime porte un bloc Transport ; le bloc de certification FNE
  n'est pas touche.

Suite : 1 501 epreuves, 1 496 passantes, 5 sautees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -1095,20 +1095,20 @@
         <v>4</v>
       </c>
       <c r="D19" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E19" s="15" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -1212,13 +1212,13 @@
         <v>81</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E23" s="10" t="n">
         <v>4</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G23" s="10" t="n">
         <v>8</v>
@@ -1262,7 +1262,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1306,7 +1305,7 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>1. NAVIGATION — à traiter en premier</t>
         </is>
@@ -1473,7 +1472,7 @@
     </row>
     <row r="10"/>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>2. COMPTABILITÉ — le principe : Selflow facture, Comptaflow tient les livres</t>
         </is>
@@ -1754,7 +1753,7 @@
     </row>
     <row r="19"/>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>3. COMPTABILITÉ ÉTEINTE — ce qui disparaît des écrans courants</t>
         </is>
@@ -1997,7 +1996,7 @@
     </row>
     <row r="27"/>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="12" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>4. MOYENS DE PAIEMENT — ce qui remplace les codes journaux</t>
         </is>
@@ -2164,7 +2163,7 @@
     </row>
     <row r="33"/>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="12" t="inlineStr">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t>5. LES ÉCRITURES TOURNENT MÊME QUAND LA COMPTABILITÉ EST ÉTEINTE</t>
         </is>
@@ -2255,7 +2254,7 @@
     </row>
     <row r="37"/>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="12" t="inlineStr">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>6. CONFIGURATION GLOBALE — saisir les comptes une fois, et non par produit</t>
         </is>
@@ -2460,7 +2459,7 @@
     </row>
     <row r="44"/>
     <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
+      <c r="A45" s="23" t="inlineStr">
         <is>
           <t>7. DÉVERSEMENT COMPTAFLOW — les lignes arrivaient déséquilibrées</t>
         </is>
@@ -2665,7 +2664,7 @@
     </row>
     <row r="51"/>
     <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="12" t="inlineStr">
+      <c r="A52" s="23" t="inlineStr">
         <is>
           <t>8. AVOIRS — un avoir ne peut pas dépasser la facture (image 4)</t>
         </is>
@@ -2832,7 +2831,7 @@
     </row>
     <row r="57"/>
     <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="12" t="inlineStr">
+      <c r="A58" s="23" t="inlineStr">
         <is>
           <t>9. ÉCRANS D'ENTRÉE — inscription, point de vente, visite guidée</t>
         </is>
@@ -2999,7 +2998,7 @@
     </row>
     <row r="63"/>
     <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="12" t="inlineStr">
+      <c r="A64" s="23" t="inlineStr">
         <is>
           <t>10. PARAMÈTRES — le compte sur la plateforme FNE</t>
         </is>
@@ -3242,7 +3241,7 @@
     </row>
     <row r="71"/>
     <row r="72" ht="20" customHeight="1">
-      <c r="A72" s="12" t="inlineStr">
+      <c r="A72" s="23" t="inlineStr">
         <is>
           <t>11. MODÈLES D'IMPORT — refléter exactement les champs de la plateforme</t>
         </is>
@@ -3409,7 +3408,7 @@
     </row>
     <row r="77"/>
     <row r="78" ht="20" customHeight="1">
-      <c r="A78" s="12" t="inlineStr">
+      <c r="A78" s="23" t="inlineStr">
         <is>
           <t>12. PERFORMANCE — l'application est lente</t>
         </is>
@@ -3576,7 +3575,7 @@
     </row>
     <row r="83"/>
     <row r="84" ht="20" customHeight="1">
-      <c r="A84" s="12" t="inlineStr">
+      <c r="A84" s="23" t="inlineStr">
         <is>
           <t>13. CONDUITE DU CHANTIER</t>
         </is>
@@ -3742,7 +3741,7 @@
       </c>
     </row>
     <row r="89" ht="20" customHeight="1">
-      <c r="A89" s="12" t="inlineStr">
+      <c r="A89" s="23" t="inlineStr">
         <is>
           <t>14. TROUVÉ EN CHEMIN — relevé pendant le chantier 1, le 02/10/2026</t>
         </is>
@@ -3908,7 +3907,7 @@
       </c>
     </row>
     <row r="94" ht="20" customHeight="1">
-      <c r="A94" s="12" t="inlineStr">
+      <c r="A94" s="23" t="inlineStr">
         <is>
           <t>15. LA LIVRAISON — relevé le 05/10/2026</t>
         </is>
@@ -4015,16 +4014,16 @@
       </c>
       <c r="D97" s="14" t="inlineStr">
         <is>
-          <t>Demandé par le propriétaire le 05/10/2026. L'écran ne porte que la quantité à expédier : aucune information sur la DESTINATION, sur QUI se charge de la livraison, ni sur les HEURES — départ et arrivée. À ajouter, avec tout ce qui accompagne le suivi d'une livraison : adresse de livraison, livreur (personnel ou prestataire), véhicule ou immatriculation, heure de départ, heure d'arrivée, nom et signature du réceptionnaire, observations. À TRANCHER avec le propriétaire : lesquels sont obligatoires, et si le bon de livraison imprimé doit les porter.</t>
-        </is>
-      </c>
-      <c r="E97" s="20" t="inlineStr">
-        <is>
-          <t>À trancher</t>
+          <t>Demandé par le propriétaire le 05/10/2026. L'écran ne porte que la quantité à expédier : aucune information sur la DESTINATION, sur QUI se charge de la livraison, ni sur les HEURES — départ et arrivée. À ajouter, avec tout ce qui accompagne le suivi d'une livraison : adresse de livraison, livreur (personnel ou prestataire), véhicule ou immatriculation, heure de départ, heure d'arrivée, nom et signature du réceptionnaire, observations. À TRANCHER avec le propriétaire : lesquels sont obligatoires, et si le bon de livraison imprimé doit les porter. TRANCHÉ PAR LE PROPRIÉTAIRE LE 07/10 : tout obligatoire, imprimé sur le bon. FAIT au lot 53 : départ (adresse, livreur, véhicule, heure) à la création, arrivée (heure, réceptionnaire, signature tracée, observations) à « marquer livré ». TROUVÉ : la file Livraisons du stock n'établissait aucun bon, et les quantités du bon étaient des entiers.</t>
+        </is>
+      </c>
+      <c r="E97" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F97" s="22" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="G97" s="22" t="n">
         <v>46302</v>
@@ -4075,7 +4074,7 @@
     </row>
     <row r="99"/>
     <row r="100" ht="20" customHeight="1">
-      <c r="A100" s="12" t="inlineStr">
+      <c r="A100" s="23" t="inlineStr">
         <is>
           <t>16. LES ÉCRITURES D'ACHAT VENUES DE LA DGI — règles en vigueur</t>
         </is>

</xml_diff>

<commit_message>
Lot 54 : l'avoir interne d'un BAPA
Chantier 8.4. La DGI ne normalise toujours pas l'avoir d'un BAPA
(confirme par le proprietaire le 07/10/2026) : l'avoir est interne, non
certifie, et ne vaut que pour la comptabilite et le stock.

- Deux tables a part (avoirs_bapa, avoir_bapa_lignes) : une ligne achats
  sur un vendeur sans NCC serait prise pour un BAPA par quatre chemins qui
  parlent a la DGI.
- Plafond en quantite et en montant, au serveur, sous verrou ; prix du
  bordereau, non saisissable ; seul un BAPA finalise s'avoire.
- Ecriture sans TVA (fournisseur debite, charge recreditee), retour stock
  au choix, document qui se dit non certifie.

Suite : 1 506 epreuves, 1 501 passantes, 5 sautees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -885,20 +885,20 @@
         <v>4</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E12" s="15" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>Terminée</t>
         </is>
       </c>
     </row>
@@ -1212,13 +1212,13 @@
         <v>81</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E23" s="10" t="n">
         <v>4</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" s="10" t="n">
         <v>8</v>
@@ -2809,19 +2809,19 @@
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : l'avoir fournisseur ne concerne QUE les BAPA — les bordereaux d'achat auprès d'un particulier, que Selflow émet et que la DGI certifie. Un achat ordinaire est une pièce du fournisseur, pas de nous : on ne l'avoire pas, on demande au fournisseur son propre avoir. Le contrôle de dépassement s'applique donc au BAPA, et l'écran ne doit pas proposer d'avoir sur les autres achats. À TRANCHER, relevé le 06/10/2026 : l'avoir fournisseur a été retiré le 25/09 sur TOUS les achats, et aucun n'est proposé sur un achat ordinaire — la seconde moitié du chantier est donc acquise. Mais le BAPA porte une interdiction écrite (`Achat::estBapa()`, AVOIR_BAPA_INTERDIT) : « la DGI ne normalise pas l'avoir d'un BAPA ». Le rétablir supposerait de certifier cet avoir, donc de toucher FneService — périmètre gelé. Il faut votre décision : (a) la DGI le permet désormais — exception 1 ou 3 de CLAUDE.md, et je l'ouvre avec le plafond ; (b) un avoir de BAPA interne, non certifié, qui ne vaudrait que pour la comptabilité.</t>
-        </is>
-      </c>
-      <c r="E56" s="20" t="inlineStr">
-        <is>
-          <t>À trancher</t>
+          <t>PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : l'avoir fournisseur ne concerne QUE les BAPA — les bordereaux d'achat auprès d'un particulier, que Selflow émet et que la DGI certifie. Un achat ordinaire est une pièce du fournisseur, pas de nous : on ne l'avoire pas, on demande au fournisseur son propre avoir. Le contrôle de dépassement s'applique donc au BAPA, et l'écran ne doit pas proposer d'avoir sur les autres achats. À TRANCHER, relevé le 06/10/2026 : l'avoir fournisseur a été retiré le 25/09 sur TOUS les achats, et aucun n'est proposé sur un achat ordinaire — la seconde moitié du chantier est donc acquise. Mais le BAPA porte une interdiction écrite (`Achat::estBapa()`, AVOIR_BAPA_INTERDIT) : « la DGI ne normalise pas l'avoir d'un BAPA ». Le rétablir supposerait de certifier cet avoir, donc de toucher FneService — périmètre gelé. Il faut votre décision : (a) la DGI le permet désormais — exception 1 ou 3 de CLAUDE.md, et je l'ouvre avec le plafond ; (b) un avoir de BAPA interne, non certifié, qui ne vaudrait que pour la comptabilité. TRANCHÉ LE 07/10 : la DGI ne normalise toujours pas l'avoir de BAPA. FAIT au lot 54, option (b) : avoir INTERNE non certifié, tables à part (avoirs_bapa) que rien de ce qui parle à la DGI ne lit ; plafond en quantité et en montant sous verrou ; écriture sans TVA ; retour stock au choix.</t>
+        </is>
+      </c>
+      <c r="E56" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F56" s="22" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="G56" s="22" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="H56" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Lot 55 : ce que la session parallele avait trouve
Deux sessions ont refait le meme plan en parallele depuis 9c2edeb. La
branche des lots 41 a 52 fait foi ; ce que l'autre avait trouve et que
celle-ci ne couvrait pas est reporte (section 19 du plan) :

- le plafond des avoirs passait par le filtre de periode global ;
- les fiches creees par l'API, le B2B ou un BAPA naissaient sans numero de
  tiers ni compte collectif ;
- les immobilisations restaient ouvertes comptabilite fermee ;
- une ligne a deux comptes partait chez Comptaflow ;
- la consignation ne se saisissait nulle part ;
- la visite guidee n'ouvrait pas la barre d'un telephone.

Suite : 1 512 epreuves, 1 507 passantes, 5 sautees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1203,24 +1203,54 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>19. REPORTÉ DE LA SESSION PARALLÈLE — 07/10/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n">
+        <v>118</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>Terminée</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C23" s="10" t="n">
-        <v>81</v>
-      </c>
-      <c r="D23" s="10" t="n">
-        <v>69</v>
-      </c>
-      <c r="E23" s="10" t="n">
+      <c r="C24" s="10" t="n">
+        <v>87</v>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>75</v>
+      </c>
+      <c r="E24" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="10" t="n">
+      <c r="F24" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="10" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1235,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4641,25 +4671,269 @@
         </is>
       </c>
     </row>
+    <row r="117"/>
+    <row r="118" ht="20" customHeight="1">
+      <c r="A118" s="23" t="inlineStr">
+        <is>
+          <t>19. REPORTÉ DE LA SESSION PARALLÈLE — 07/10/2026</t>
+        </is>
+      </c>
+      <c r="B118" s="21" t="n"/>
+      <c r="C118" s="21" t="n"/>
+      <c r="D118" s="21" t="n"/>
+      <c r="E118" s="21" t="n"/>
+      <c r="F118" s="21" t="n"/>
+      <c r="G118" s="21" t="n"/>
+      <c r="H118" s="21" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="14" t="inlineStr">
+        <is>
+          <t>Avoirs de vente</t>
+        </is>
+      </c>
+      <c r="B119" s="15" t="inlineStr">
+        <is>
+          <t>19.1</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>Le plafond voyait à travers le filtre de période</t>
+        </is>
+      </c>
+      <c r="D119" s="14" t="inlineStr">
+        <is>
+          <t>Vente::resteAAvoirer() et le compteur des quantités déjà créditées passaient par le filtre de période global : un avoir d'une autre période échappait au plafond, et la même somme pouvait être rendue deux fois. Lus hors période.</t>
+        </is>
+      </c>
+      <c r="E119" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F119" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="G119" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H119" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="14" t="inlineStr">
+        <is>
+          <t>Tiers</t>
+        </is>
+      </c>
+      <c r="B120" s="15" t="inlineStr">
+        <is>
+          <t>19.2</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>Le numéro de tiers posé par toutes les portes</t>
+        </is>
+      </c>
+      <c r="D120" s="14" t="inlineStr">
+        <is>
+          <t>L'API mobile, le parcours B2B et le tiers d'un BAPA créaient des fiches sans numéro de tiers ni compte collectif ; leurs écritures retombaient en vrac sur le collectif chez Comptaflow. Posés à la création du modèle.</t>
+        </is>
+      </c>
+      <c r="E120" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F120" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="G120" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H120" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="14" t="inlineStr">
+        <is>
+          <t>Immobilisations</t>
+        </is>
+      </c>
+      <c r="B121" s="15" t="inlineStr">
+        <is>
+          <t>19.3</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>Derrière le garde-fou de la comptabilité</t>
+        </is>
+      </c>
+      <c r="D121" s="14" t="inlineStr">
+        <is>
+          <t>Comptes d'immobilisation, dotations, clôture d'exercice : de la tenue de livres, restée ouverte à toute entreprise par son adresse. 404 (Not Found — introuvable) quand la comptabilité est fermée.</t>
+        </is>
+      </c>
+      <c r="E121" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F121" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="G121" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H121" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="14" t="inlineStr">
+        <is>
+          <t>Déversement</t>
+        </is>
+      </c>
+      <c r="B122" s="15" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>Une ligne à deux comptes ne part pas</t>
+        </is>
+      </c>
+      <c r="D122" s="14" t="inlineStr">
+        <is>
+          <t>Comptaflow ne lit qu'un compte par ligne ; l'équilibre recompté ne voyait pas une ligne à deux comptes ou au montant du mauvais côté. Contrôle ajouté avant l'envoi.</t>
+        </is>
+      </c>
+      <c r="E122" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F122" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="G122" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H122" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="14" t="inlineStr">
+        <is>
+          <t>Fiche produit</t>
+        </is>
+      </c>
+      <c r="B123" s="15" t="inlineStr">
+        <is>
+          <t>19.5</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>La consignation se saisit enfin</t>
+        </is>
+      </c>
+      <c r="D123" s="14" t="inlineStr">
+        <is>
+          <t>Prix de consignation et délai de retour ne se saisissaient nulle part : l'import était la seule porte vers les consignations. Ajoutés à la fiche.</t>
+        </is>
+      </c>
+      <c r="E123" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F123" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="G123" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H123" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="14" t="inlineStr">
+        <is>
+          <t>Visite guidée</t>
+        </is>
+      </c>
+      <c r="B124" s="15" t="inlineStr">
+        <is>
+          <t>19.6</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>Sur téléphone, la barre s'ouvre</t>
+        </is>
+      </c>
+      <c r="D124" s="14" t="inlineStr">
+        <is>
+          <t>La barre latérale d'un téléphone est hors écran : la visite l'ouvre pour désigner une entrée du menu, attend la fin du glissement, puis la referme.</t>
+        </is>
+      </c>
+      <c r="E124" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F124" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="G124" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H124" s="15" t="inlineStr">
+        <is>
+          <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:H116"/>
-  <mergeCells count="18">
+  <mergeCells count="19">
+    <mergeCell ref="A64:H64"/>
+    <mergeCell ref="A11:H11"/>
     <mergeCell ref="A45:H45"/>
     <mergeCell ref="A94:H94"/>
+    <mergeCell ref="A78:H78"/>
+    <mergeCell ref="A118:H118"/>
+    <mergeCell ref="A84:H84"/>
+    <mergeCell ref="A89:H89"/>
+    <mergeCell ref="A105:H105"/>
+    <mergeCell ref="A5:H5"/>
     <mergeCell ref="A100:H100"/>
-    <mergeCell ref="A78:H78"/>
-    <mergeCell ref="A105:H105"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A38:H38"/>
     <mergeCell ref="A72:H72"/>
     <mergeCell ref="A52:H52"/>
-    <mergeCell ref="A64:H64"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="A112:H112"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A84:H84"/>
-    <mergeCell ref="A89:H89"/>
     <mergeCell ref="A58:H58"/>
     <mergeCell ref="A34:H34"/>
   </mergeCells>

</xml_diff>

<commit_message>
Retrait du lot 54 : pas d'avoir sur un BAPA, pas d'avoir tout court
Le proprietaire a refuse l'avoir interne non certifie le 07/10/2026 :
aucun avoir sur un achat, BAPA compris. Tables, ecrans, routes, ecriture
et epreuve du lot 54 sont retires avant tout deploiement (la migration n'a
jamais tourne en production). Journal, plan (8.4) et passation a jour.

Suite : 1 507 epreuves, 1 502 passantes, 5 sautees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -2834,12 +2834,12 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Même contrôle sur l'avoir de BAPA — et lui seul</t>
+          <t>Pas d'avoir sur un achat, BAPA compris</t>
         </is>
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : l'avoir fournisseur ne concerne QUE les BAPA — les bordereaux d'achat auprès d'un particulier, que Selflow émet et que la DGI certifie. Un achat ordinaire est une pièce du fournisseur, pas de nous : on ne l'avoire pas, on demande au fournisseur son propre avoir. Le contrôle de dépassement s'applique donc au BAPA, et l'écran ne doit pas proposer d'avoir sur les autres achats. À TRANCHER, relevé le 06/10/2026 : l'avoir fournisseur a été retiré le 25/09 sur TOUS les achats, et aucun n'est proposé sur un achat ordinaire — la seconde moitié du chantier est donc acquise. Mais le BAPA porte une interdiction écrite (`Achat::estBapa()`, AVOIR_BAPA_INTERDIT) : « la DGI ne normalise pas l'avoir d'un BAPA ». Le rétablir supposerait de certifier cet avoir, donc de toucher FneService — périmètre gelé. Il faut votre décision : (a) la DGI le permet désormais — exception 1 ou 3 de CLAUDE.md, et je l'ouvre avec le plafond ; (b) un avoir de BAPA interne, non certifié, qui ne vaudrait que pour la comptabilité. TRANCHÉ LE 07/10 : la DGI ne normalise toujours pas l'avoir de BAPA. FAIT au lot 54, option (b) : avoir INTERNE non certifié, tables à part (avoirs_bapa) que rien de ce qui parle à la DGI ne lit ; plafond en quantité et en montant sous verrou ; écriture sans TVA ; retour stock au choix.</t>
+          <t>PRÉCISÉ PAR LE PROPRIÉTAIRE le 05/10/2026 : l'avoir fournisseur ne concerne QUE les BAPA — les bordereaux d'achat auprès d'un particulier, que Selflow émet et que la DGI certifie. Un achat ordinaire est une pièce du fournisseur, pas de nous : on ne l'avoire pas, on demande au fournisseur son propre avoir. Le contrôle de dépassement s'applique donc au BAPA, et l'écran ne doit pas proposer d'avoir sur les autres achats. À TRANCHER, relevé le 06/10/2026 : l'avoir fournisseur a été retiré le 25/09 sur TOUS les achats, et aucun n'est proposé sur un achat ordinaire — la seconde moitié du chantier est donc acquise. Mais le BAPA porte une interdiction écrite (`Achat::estBapa()`, AVOIR_BAPA_INTERDIT) : « la DGI ne normalise pas l'avoir d'un BAPA ». Le rétablir supposerait de certifier cet avoir, donc de toucher FneService — périmètre gelé. Il faut votre décision : (a) la DGI le permet désormais — exception 1 ou 3 de CLAUDE.md, et je l'ouvre avec le plafond ; (b) un avoir de BAPA interne, non certifié, qui ne vaudrait que pour la comptabilité. TRANCHÉ PAR LE PROPRIÉTAIRE LE 07/10/2026 : AUCUN AVOIR sur un achat, BAPA compris — ni certifié, ni interne. Un avoir interne établi au lot 54 a été retiré le jour même. Aucun écran d'achat n'en propose (AvoirDeBapaTest).</t>
         </is>
       </c>
       <c r="E56" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Lot 56 : la suite Comptaflow au vert, chantier 18.3 termine
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -1185,10 +1185,10 @@
         <v>4</v>
       </c>
       <c r="D22" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="H22" s="18" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>3/4</t>
         </is>
       </c>
     </row>
@@ -1242,10 +1242,10 @@
         <v>87</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F24" s="10" t="n">
         <v>0</v>
@@ -4615,18 +4615,20 @@
       </c>
       <c r="D115" s="14" t="inlineStr">
         <is>
-          <t>Relevé en lançant sa suite le 06/10/2026 : 19 échecs présents AVANT ce lot (identiques avec et sans). Une vingtième — la recopie au 28 février, qui prenait sa ligne sans ordre — tombait selon l'index choisi par SQLite : corrigée. Les 19 reviennent au mainteneur de Comptaflow.</t>
-        </is>
-      </c>
-      <c r="E115" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Relevé en lançant sa suite le 06/10/2026 : 19 échecs présents AVANT ce lot (identiques avec et sans). Une vingtième — la recopie au 28 février, qui prenait sa ligne sans ordre — tombait selon l'index choisi par SQLite : corrigée. Les 19 reviennent au mainteneur de Comptaflow. FAIT LE 07/10/2026 : les 19 tombaient toutes en 500 sur le même défaut — le manifeste Vite (public/build) absent hors compilation. withoutVite() dans tests/TestCase.php de Comptaflow : 301/301 vertes. Fusionné dans main sur guysergekouassi/COMPTAFLOW et IT-dcknowing/COMPTAFLOW (f776d31).</t>
+        </is>
+      </c>
+      <c r="E115" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F115" s="22" t="n">
         <v>46301</v>
       </c>
-      <c r="G115" s="22" t="n"/>
+      <c r="G115" s="22" t="n">
+        <v>46302</v>
+      </c>
       <c r="H115" s="15" t="inlineStr">
         <is>
           <t>Comptaflow</t>

</xml_diff>

<commit_message>
Plan (section 20), journal (lot 62) et passation du 08/10/2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1233,24 +1233,54 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>20. RETOURS DU PROPRIÉTAIRE — 08/10/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>126</v>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>13/17</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C24" s="10" t="n">
-        <v>87</v>
-      </c>
-      <c r="D24" s="10" t="n">
-        <v>76</v>
-      </c>
-      <c r="E24" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="F24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="10" t="n">
+      <c r="C25" s="10" t="n">
+        <v>104</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>89</v>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="10" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1265,7 +1295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H124"/>
+  <dimension ref="A1:H143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4913,6 +4943,659 @@
       <c r="H124" s="15" t="inlineStr">
         <is>
           <t>Jour 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="125"/>
+    <row r="126">
+      <c r="A126" s="23" t="inlineStr">
+        <is>
+          <t>20. RETOURS DU PROPRIÉTAIRE — 08/10/2026</t>
+        </is>
+      </c>
+      <c r="B126" s="21" t="n"/>
+      <c r="C126" s="21" t="n"/>
+      <c r="D126" s="21" t="n"/>
+      <c r="E126" s="21" t="n"/>
+      <c r="F126" s="21" t="n"/>
+      <c r="G126" s="21" t="n"/>
+      <c r="H126" s="21" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="14" t="inlineStr">
+        <is>
+          <t>Ventes / achats</t>
+        </is>
+      </c>
+      <c r="B127" s="15" t="inlineStr">
+        <is>
+          <t>20.1</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>Le cycle devis → commande → livraison → facture, et le cycle achat, corrigés</t>
+        </is>
+      </c>
+      <c r="D127" s="14" t="inlineStr">
+        <is>
+          <t>25 défauts de la recette du 08/10 corrigés (lot 60) : stock sorti ou entré deux fois, commandes refacturées, fausse facture de la file du stock, avoir sur devis, remise et encaissement d'un BL, numérotation, boutons. 36 épreuves permanentes.</t>
+        </is>
+      </c>
+      <c r="E127" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F127" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G127" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H127" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="14" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="B128" s="15" t="inlineStr">
+        <is>
+          <t>20.2</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>Le module Production corrigé</t>
+        </is>
+      </c>
+      <c r="D128" s="14" t="inlineStr">
+        <is>
+          <t>15 défauts (lot 59) : unités converties, annulation, erreurs 500, arrondis, recette figée dans l'ordre, détail et bon de fabrication imprimable.</t>
+        </is>
+      </c>
+      <c r="E128" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F128" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G128" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H128" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="14" t="inlineStr">
+        <is>
+          <t>Recette de zéro</t>
+        </is>
+      </c>
+      <c r="B129" s="15" t="inlineStr">
+        <is>
+          <t>20.3</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>Une entreprise créée de zéro, par l'interface</t>
+        </is>
+      </c>
+      <c r="D129" s="14" t="inlineStr">
+        <is>
+          <t>Inscription, souscription, paramètres, personnel, catalogue, import, stock, ventes, achats, demandes (lot 61) : 15 corrections. Devis enregistré en espèces : plus encaissé d'office.</t>
+        </is>
+      </c>
+      <c r="E129" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F129" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G129" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H129" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="14" t="inlineStr">
+        <is>
+          <t>Identité</t>
+        </is>
+      </c>
+      <c r="B130" s="15" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>Logo officiel et icône du navigateur</t>
+        </is>
+      </c>
+      <c r="D130" s="14" t="inlineStr">
+        <is>
+          <t>Barre latérale, pages d'entrée, vitrine, favicon (lot 58). Bouton « Créer un compte » de la vitrine lisible.</t>
+        </is>
+      </c>
+      <c r="E130" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F130" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G130" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H130" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="14" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B131" s="15" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>Barre latérale, modèle A</t>
+        </is>
+      </c>
+      <c r="D131" s="14" t="inlineStr">
+        <is>
+          <t>Familles Pilotage, Commerce, Opérations, Finance &amp; fiscalité, Entreprise. Affichage seulement : les habilitations ne changent pas.</t>
+        </is>
+      </c>
+      <c r="E131" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F131" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G131" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H131" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="14" t="inlineStr">
+        <is>
+          <t>Connexion</t>
+        </is>
+      </c>
+      <c r="B132" s="15" t="inlineStr">
+        <is>
+          <t>20.6</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>Page de connexion, proposition 1</t>
+        </is>
+      </c>
+      <c r="D132" s="14" t="inlineStr">
+        <is>
+          <t>Refaite fidèlement à la proposition 1 (tuile 3D, fond quadrillé). La branche « connexion » n'est pas fusionnée.</t>
+        </is>
+      </c>
+      <c r="E132" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F132" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G132" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H132" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="14" t="inlineStr">
+        <is>
+          <t>Compte FNE</t>
+        </is>
+      </c>
+      <c r="B133" s="15" t="inlineStr">
+        <is>
+          <t>20.7</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>États de connexion, champs repris du portail, accès vus par le superadmin</t>
+        </is>
+      </c>
+      <c r="D133" s="14" t="inlineStr">
+        <is>
+          <t>Connexion en cours / en test / établie, création en cours. Champs grisés seulement après un relevé. Accès inscrits pour le scraper, relevé demandé et lancé. « Voir les accès FNE » derrière le mot de passe du superadmin.</t>
+        </is>
+      </c>
+      <c r="E133" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F133" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G133" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H133" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="14" t="inlineStr">
+        <is>
+          <t>Timbre / BAPA</t>
+        </is>
+      </c>
+      <c r="B134" s="15" t="inlineStr">
+        <is>
+          <t>20.8</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>Timbre, BAPA et seuil suivent l'espace FNE dans les deux sens</t>
+        </is>
+      </c>
+      <c r="D134" s="14" t="inlineStr">
+        <is>
+          <t>Coché → coché, décoché → décoché. Timbre décoché : pas de barème en caisse, message dans les paramètres. BAPA décoché : rien du bordereau dans l'application (archives consultables).</t>
+        </is>
+      </c>
+      <c r="E134" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F134" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G134" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H134" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="14" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="B135" s="15" t="inlineStr">
+        <is>
+          <t>20.9</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>Socle par défaut et attributions du superadmin</t>
+        </is>
+      </c>
+      <c r="D135" s="14" t="inlineStr">
+        <is>
+          <t>Case cochée : solde &amp; journal, codes journaux, créances &amp; règlements, plan comptable, configuration des comptes. Encaissements, décaissements, opérations globales, grand livre, lettrage, balance : accordés par le superadmin. Caissier : garde sa caisse.</t>
+        </is>
+      </c>
+      <c r="E135" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F135" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G135" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H135" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="14" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="B136" s="15" t="inlineStr">
+        <is>
+          <t>20.10</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>Exercices antérieurs</t>
+        </is>
+      </c>
+      <c r="D136" s="14" t="inlineStr">
+        <is>
+          <t>L'entreprise demande, le superadmin accorde une sélection d'années ; seuls l'exercice en cours et les années accordées partent chez Comptaflow.</t>
+        </is>
+      </c>
+      <c r="E136" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F136" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G136" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H136" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="14" t="inlineStr">
+        <is>
+          <t>Factures</t>
+        </is>
+      </c>
+      <c r="B137" s="15" t="inlineStr">
+        <is>
+          <t>20.11</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>Colonnes HT et TTC réel dans la liste</t>
+        </is>
+      </c>
+      <c r="D137" s="14" t="inlineStr">
+        <is>
+          <t>TTC = net à payer (timbre et autres taxes compris), comme sur la facture.</t>
+        </is>
+      </c>
+      <c r="E137" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F137" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G137" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H137" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="14" t="inlineStr">
+        <is>
+          <t>FNE</t>
+        </is>
+      </c>
+      <c r="B138" s="15" t="inlineStr">
+        <is>
+          <t>20.12</t>
+        </is>
+      </c>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>Relevé des avoirs du portail (branche du collaborateur)</t>
+        </is>
+      </c>
+      <c r="D138" s="14" t="inlineStr">
+        <is>
+          <t>Intégré. Défaut corrigé : un avoir ÉMIS à un client passait pour un avoir fournisseur et partait au journal des achats.</t>
+        </is>
+      </c>
+      <c r="E138" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F138" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G138" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H138" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="14" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="B139" s="15" t="inlineStr">
+        <is>
+          <t>20.13</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>Lenteur signalée le 08/10</t>
+        </is>
+      </c>
+      <c r="D139" s="14" t="inlineStr">
+        <is>
+          <t>Écrans mesurés : mêmes requêtes et temps qu'au 07/10. Les relevés achats et avoirs ouvraient deux navigateurs à la même minute toutes les 5 min : décalés.</t>
+        </is>
+      </c>
+      <c r="E139" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F139" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G139" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H139" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="14" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B140" s="15" t="inlineStr">
+        <is>
+          <t>20.14</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>Réapprovisionner sans achat saisi</t>
+        </is>
+      </c>
+      <c r="D140" s="14" t="inlineStr">
+        <is>
+          <t>Proposition : une page « Entrée de stock » (article, quantité, coût unitaire, motif) qui fait entrer le stock au coût réel. À valider par le propriétaire.</t>
+        </is>
+      </c>
+      <c r="E140" s="16" t="inlineStr">
+        <is>
+          <t>À trancher</t>
+        </is>
+      </c>
+      <c r="F140" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G140" s="22" t="n"/>
+      <c r="H140" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="14" t="inlineStr">
+        <is>
+          <t>Comptaflow</t>
+        </is>
+      </c>
+      <c r="B141" s="15" t="inlineStr">
+        <is>
+          <t>20.15</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>Liaison réelle et déversement à vérifier</t>
+        </is>
+      </c>
+      <c r="D141" s="14" t="inlineStr">
+        <is>
+          <t>Le test de liaison a été interrompu par une limite d'usage. À reprendre avec 7.5.</t>
+        </is>
+      </c>
+      <c r="E141" s="18" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F141" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G141" s="22" t="n"/>
+      <c r="H141" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="14" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="B142" s="15" t="inlineStr">
+        <is>
+          <t>20.16</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>Résumé de toute la logique de Selflow</t>
+        </is>
+      </c>
+      <c r="D142" s="14" t="inlineStr">
+        <is>
+          <t>Rédaction interrompue par une limite d'usage. À reprendre.</t>
+        </is>
+      </c>
+      <c r="E142" s="18" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F142" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G142" s="22" t="n"/>
+      <c r="H142" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="14" t="inlineStr">
+        <is>
+          <t>Recette de zéro</t>
+        </is>
+      </c>
+      <c r="B143" s="15" t="inlineStr">
+        <is>
+          <t>20.17</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>Défauts restants non corrigés</t>
+        </is>
+      </c>
+      <c r="D143" s="14" t="inlineStr">
+        <is>
+          <t>Catégorie créée sans compte (écritures de stock manquantes), régimes des tiers faux, NCC d'un client B2G effacé, même numéro BC vente/achat, achat antidaté (écriture de stock du jour), libellés FNE incohérents.</t>
+        </is>
+      </c>
+      <c r="E143" s="18" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F143" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G143" s="22" t="n"/>
+      <c r="H143" s="15" t="inlineStr">
+        <is>
+          <t>Jour 3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan (20.14, 20.17), journal (lot 63) et passation du 09/10/2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -1322,6 +1322,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1811,7 +1812,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="23" t="inlineStr">
         <is>
@@ -2054,7 +2054,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="23" t="inlineStr">
         <is>
@@ -2221,7 +2220,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="23" t="inlineStr">
         <is>
@@ -2312,7 +2310,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="23" t="inlineStr">
         <is>
@@ -2517,7 +2514,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="23" t="inlineStr">
         <is>
@@ -2722,7 +2718,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="23" t="inlineStr">
         <is>
@@ -2889,7 +2884,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="23" t="inlineStr">
         <is>
@@ -3056,7 +3050,6 @@
         </is>
       </c>
     </row>
-    <row r="63"/>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="23" t="inlineStr">
         <is>
@@ -3299,7 +3292,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="23" t="inlineStr">
         <is>
@@ -3466,7 +3458,6 @@
         </is>
       </c>
     </row>
-    <row r="77"/>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="23" t="inlineStr">
         <is>
@@ -3633,7 +3624,6 @@
         </is>
       </c>
     </row>
-    <row r="83"/>
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="23" t="inlineStr">
         <is>
@@ -4132,7 +4122,6 @@
         </is>
       </c>
     </row>
-    <row r="99"/>
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="23" t="inlineStr">
         <is>
@@ -4703,7 +4692,6 @@
         </is>
       </c>
     </row>
-    <row r="117"/>
     <row r="118" ht="20" customHeight="1">
       <c r="A118" s="23" t="inlineStr">
         <is>
@@ -4946,7 +4934,6 @@
         </is>
       </c>
     </row>
-    <row r="125"/>
     <row r="126">
       <c r="A126" s="23" t="inlineStr">
         <is>
@@ -5473,18 +5460,20 @@
       </c>
       <c r="D140" s="14" t="inlineStr">
         <is>
-          <t>Proposition : une page « Entrée de stock » (article, quantité, coût unitaire, motif) qui fait entrer le stock au coût réel. À valider par le propriétaire.</t>
+          <t>Page « Entrée de stock » faite (lot 63) : article, quantité, coût réel, raison (achat sans facture, retour, don, autre). CUMP recalculé, écriture 3x/603x avec la raison. 7 épreuves.</t>
         </is>
       </c>
       <c r="E140" s="16" t="inlineStr">
         <is>
-          <t>À trancher</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F140" s="22" t="n">
         <v>46303</v>
       </c>
-      <c r="G140" s="22" t="n"/>
+      <c r="G140" s="22" t="n">
+        <v>46304</v>
+      </c>
       <c r="H140" s="15" t="inlineStr">
         <is>
           <t>Jour 3</t>
@@ -5581,18 +5570,20 @@
       </c>
       <c r="D143" s="14" t="inlineStr">
         <is>
-          <t>Catégorie créée sans compte (écritures de stock manquantes), régimes des tiers faux, NCC d'un client B2G effacé, même numéro BC vente/achat, achat antidaté (écriture de stock du jour), libellés FNE incohérents.</t>
-        </is>
-      </c>
-      <c r="E143" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Corrigé (lot 63) : catégorie sans compte (comptes du type d'article), régimes des tiers (liste de l'entreprise, validation, migration), NCC B2G gardé, BC fournisseur en BCF-, achat antidaté (écriture de stock à la date de l'achat). Reste : libellés FNE incohérents (périmètre gelé, à lister).</t>
+        </is>
+      </c>
+      <c r="E143" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F143" s="22" t="n">
         <v>46303</v>
       </c>
-      <c r="G143" s="22" t="n"/>
+      <c r="G143" s="22" t="n">
+        <v>46304</v>
+      </c>
       <c r="H143" s="15" t="inlineStr">
         <is>
           <t>Jour 3</t>

</xml_diff>

<commit_message>
Plan (20.18 a 20.20), journal et passation : reponses du 09/10/2026
RNE (regime) garde ; NCC du client B2G sur la facture certifiee explique ;
NCC du fournisseur B2G et taux du portail (export, TOB, taxe touristique)
a trancher.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoWtgafwsFvW7Pyzkwtia8
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -1242,16 +1242,16 @@
         <v>126</v>
       </c>
       <c r="C24" s="15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D24" s="15" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G24" s="15" t="n">
         <v>0</v>
@@ -1269,16 +1269,16 @@
         </is>
       </c>
       <c r="C25" s="10" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E25" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G25" s="10" t="n">
         <v>8</v>
@@ -1295,7 +1295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H143"/>
+  <dimension ref="A1:H146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1322,7 +1322,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1531,7 +1530,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="23" t="inlineStr">
         <is>
@@ -5587,6 +5585,116 @@
       <c r="H143" s="15" t="inlineStr">
         <is>
           <t>Jour 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="14" t="inlineStr">
+        <is>
+          <t>FNE</t>
+        </is>
+      </c>
+      <c r="B144" s="15" t="inlineStr">
+        <is>
+          <t>20.18</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="inlineStr">
+        <is>
+          <t>Taux du portail absents de Selflow</t>
+        </is>
+      </c>
+      <c r="D144" s="14" t="inlineStr">
+        <is>
+          <t>Le portail propose « TVA exo export », la Taxe sur les Opérations Bancaires 5 % et 10 % et la Taxe pour le Développement Touristique. Selflow a les quatre codes TVA (A, B, C, D) ; TOB et TDT se saisissent en « autres taxes » (nom et taux). L'export n'a pas de code dans la procédure d'interfaçage : il faut la nouvelle version du référentiel ou une pièce certifiée (périmètre gelé).</t>
+        </is>
+      </c>
+      <c r="E144" s="18" t="inlineStr">
+        <is>
+          <t>À trancher</t>
+        </is>
+      </c>
+      <c r="F144" s="22" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G144" s="22" t="n"/>
+      <c r="H144" s="15" t="inlineStr">
+        <is>
+          <t>Jour 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="14" t="inlineStr">
+        <is>
+          <t>Tiers</t>
+        </is>
+      </c>
+      <c r="B145" s="15" t="inlineStr">
+        <is>
+          <t>20.19</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>NCC du fournisseur B2G</t>
+        </is>
+      </c>
+      <c r="D145" s="14" t="inlineStr">
+        <is>
+          <t>Effacé à l'enregistrement (règle recopiée des clients). Un achat à un fournisseur sans NCC part en bordereau BAPA ; le garder ferait passer ses achats en factures reçues. Recommandé : le garder (une administration est immatriculée, le BAPA vise les producteurs non immatriculés). Accord du propriétaire attendu.</t>
+        </is>
+      </c>
+      <c r="E145" s="18" t="inlineStr">
+        <is>
+          <t>À trancher</t>
+        </is>
+      </c>
+      <c r="F145" s="22" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G145" s="22" t="n"/>
+      <c r="H145" s="15" t="inlineStr">
+        <is>
+          <t>Jour 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="14" t="inlineStr">
+        <is>
+          <t>Tiers</t>
+        </is>
+      </c>
+      <c r="B146" s="15" t="inlineStr">
+        <is>
+          <t>20.20</t>
+        </is>
+      </c>
+      <c r="C146" s="5" t="inlineStr">
+        <is>
+          <t>Régime RNE de l'entreprise</t>
+        </is>
+      </c>
+      <c r="D146" s="14" t="inlineStr">
+        <is>
+          <t>Le propriétaire confirme le 09/10 : le régime RNE et le reçu normalisé RNE sont deux choses distinctes. Le régime reste dans la liste.</t>
+        </is>
+      </c>
+      <c r="E146" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F146" s="22" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G146" s="22" t="n">
+        <v>46304</v>
+      </c>
+      <c r="H146" s="15" t="inlineStr">
+        <is>
+          <t>Jour 4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan, journal et passation : retours de la mise en production du 14/10/2026
Avancement des lots 64 a 69, etude de faisabilite de la communication B2B
(lot 70, a valider), section 21 du classeur, passation et deploiement
(configuration du courriel).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -620,6 +620,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1263,24 +1264,54 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>21. RETOURS DE LA MISE EN PRODUCTION — 14/10/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>148</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
+          <t>9/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C25" s="10" t="n">
-        <v>107</v>
-      </c>
-      <c r="D25" s="10" t="n">
-        <v>92</v>
-      </c>
-      <c r="E25" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="F25" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="G25" s="10" t="n">
+      <c r="C26" s="10" t="n">
+        <v>119</v>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>101</v>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="10" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1295,7 +1326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H146"/>
+  <dimension ref="A1:H160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5698,9 +5729,474 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" s="23" t="inlineStr">
+        <is>
+          <t>21. RETOURS DE LA MISE EN PRODUCTION — 14/10/2026</t>
+        </is>
+      </c>
+      <c r="B148" s="21" t="n"/>
+      <c r="C148" s="21" t="n"/>
+      <c r="D148" s="21" t="n"/>
+      <c r="E148" s="21" t="n"/>
+      <c r="F148" s="21" t="n"/>
+      <c r="G148" s="21" t="n"/>
+      <c r="H148" s="21" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="14" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="B149" s="15" t="inlineStr">
+        <is>
+          <t>21.1</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>Mot de passe oublié : le lien ne s'affiche plus, le courriel part</t>
+        </is>
+      </c>
+      <c r="D149" s="14" t="inlineStr">
+        <is>
+          <t>Faille : le lien de réinitialisation s'affichait à l'écran de quiconque tapait une adresse. Il ne part plus que par courriel ; serveur sans transport signalé ; jeton vérifié ; même réponse pour une adresse inconnue. Commande selflow:verifier-courriel (lot 64).</t>
+        </is>
+      </c>
+      <c r="E149" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F149" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G149" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H149" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="14" t="inlineStr">
+        <is>
+          <t>Courriels</t>
+        </is>
+      </c>
+      <c r="B150" s="15" t="inlineStr">
+        <is>
+          <t>21.2</t>
+        </is>
+      </c>
+      <c r="C150" s="5" t="inlineStr">
+        <is>
+          <t>Avis d'ouverture de compte</t>
+        </is>
+      </c>
+      <c r="D150" s="14" t="inlineStr">
+        <is>
+          <t>Inscription, employé, responsable créé par le superadmin, admin interne : le titulaire est prévenu, sans mot de passe (lot 64).</t>
+        </is>
+      </c>
+      <c r="E150" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F150" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G150" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H150" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="14" t="inlineStr">
+        <is>
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="B151" s="15" t="inlineStr">
+        <is>
+          <t>21.3</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>La facture « ne passe pas », sans message</t>
+        </is>
+      </c>
+      <c r="D151" s="14" t="inlineStr">
+        <is>
+          <t>Refus de stock et de lot périmé perdus sous la clé error : affichés. Message de 3 s nommant la pièce, panier vidé (lot 65).</t>
+        </is>
+      </c>
+      <c r="E151" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F151" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G151" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H151" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="14" t="inlineStr">
+        <is>
+          <t>Écrans</t>
+        </is>
+      </c>
+      <c r="B152" s="15" t="inlineStr">
+        <is>
+          <t>21.4</t>
+        </is>
+      </c>
+      <c r="C152" s="5" t="inlineStr">
+        <is>
+          <t>Recherche du catalogue, avatar, fusée, domaine en un clic</t>
+        </is>
+      </c>
+      <c r="D152" s="14" t="inlineStr">
+        <is>
+          <t>Recherche sur tout le catalogue ; initiales si la photo manque ; fusée retirée ; le clic sur le domaine mène à l'étape suivante (lot 65).</t>
+        </is>
+      </c>
+      <c r="E152" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F152" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G152" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H152" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="14" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="B153" s="15" t="inlineStr">
+        <is>
+          <t>21.5</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>L'avoir, écriture d'origine en négatif</t>
+        </is>
+      </c>
+      <c r="D153" s="14" t="inlineStr">
+        <is>
+          <t>Taxes parafiscales contre-passées, remboursement en espèces écrit (411/caisse), retour au coût de sortie. Le timbre reste dû (lot 67).</t>
+        </is>
+      </c>
+      <c r="E153" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F153" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G153" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H153" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="14" t="inlineStr">
+        <is>
+          <t>Achats</t>
+        </is>
+      </c>
+      <c r="B154" s="15" t="inlineStr">
+        <is>
+          <t>21.6</t>
+        </is>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t>Un geste par étape, actions dans la liste</t>
+        </is>
+      </c>
+      <c r="D154" s="14" t="inlineStr">
+        <is>
+          <t>DP : confirmer la commande ; BC : bon de réception et facturer. Achat B2B « Bon de commande » (lot 66).</t>
+        </is>
+      </c>
+      <c r="E154" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F154" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G154" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H154" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="14" t="inlineStr">
+        <is>
+          <t>Achats</t>
+        </is>
+      </c>
+      <c r="B155" s="15" t="inlineStr">
+        <is>
+          <t>21.7</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>Facture déclarée par le fournisseur</t>
+        </is>
+      </c>
+      <c r="D155" s="14" t="inlineStr">
+        <is>
+          <t>Question à la facturation : oui → saisie informative, la facture reçue de la DGI porte l'écriture ; non → écriture comme avant (lot 66).</t>
+        </is>
+      </c>
+      <c r="E155" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F155" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G155" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H155" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="14" t="inlineStr">
+        <is>
+          <t>Stickers</t>
+        </is>
+      </c>
+      <c r="B156" s="15" t="inlineStr">
+        <is>
+          <t>21.8</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>Achat des stickers confié à DC-Knowing</t>
+        </is>
+      </c>
+      <c r="D156" s="14" t="inlineStr">
+        <is>
+          <t>Demande (quantité, site, urgence) gardée, courriel à DC-Knowing et accusé au demandeur, page superadmin avec statut (lot 68).</t>
+        </is>
+      </c>
+      <c r="E156" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F156" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G156" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H156" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="14" t="inlineStr">
+        <is>
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="B157" s="15" t="inlineStr">
+        <is>
+          <t>21.9</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>Vente pas à pas</t>
+        </is>
+      </c>
+      <c r="D157" s="14" t="inlineStr">
+        <is>
+          <t>Bascule Caisse / Pas à pas : articles, client et document, règlement, valider et facturer. Même formulaire (lot 69). Vérifiée dans Chromium.</t>
+        </is>
+      </c>
+      <c r="E157" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F157" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G157" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H157" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="14" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="B158" s="15" t="inlineStr">
+        <is>
+          <t>21.10</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>Le timbre d'une facture annulée est-il remboursé au client ?</t>
+        </is>
+      </c>
+      <c r="D158" s="14" t="inlineStr">
+        <is>
+          <t>Aujourd'hui non : il reste dû à l'État (la plateforme ne le porte sur aucun avoir). Si l'entreprise le rend, il devient une charge (646).</t>
+        </is>
+      </c>
+      <c r="E158" s="18" t="inlineStr">
+        <is>
+          <t>À trancher</t>
+        </is>
+      </c>
+      <c r="F158" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G158" s="22" t="n"/>
+      <c r="H158" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="14" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="B159" s="15" t="inlineStr">
+        <is>
+          <t>21.11</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>Communication B2B approfondie</t>
+        </is>
+      </c>
+      <c r="D159" s="14" t="inlineStr">
+        <is>
+          <t>Faisable sans toucher au périmètre gelé : 70a fil de discussion, 70b commander et confirmer (BC confirmé — en attente de livraison), 70c livrer, facturer, réceptionner, 70d notifications. Défauts de l'existant relevés. À valider.</t>
+        </is>
+      </c>
+      <c r="E159" s="18" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F159" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G159" s="22" t="n"/>
+      <c r="H159" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="14" t="inlineStr">
+        <is>
+          <t>Retours</t>
+        </is>
+      </c>
+      <c r="B160" s="15" t="inlineStr">
+        <is>
+          <t>21.12</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>« Des corrections à revoir pour Selflow.docx »</t>
+        </is>
+      </c>
+      <c r="D160" s="14" t="inlineStr">
+        <is>
+          <t>Document annoncé, non parvenu dans la session du 14/10. À traiter à réception.</t>
+        </is>
+      </c>
+      <c r="E160" s="18" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F160" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G160" s="22" t="n"/>
+      <c r="H160" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:H116"/>
-  <mergeCells count="19">
+  <mergeCells count="20">
+    <mergeCell ref="A148:H148"/>
     <mergeCell ref="A64:H64"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A45:H45"/>

</xml_diff>

<commit_message>
Vitrine : menu court, liens des applications, contraste ; plan et passation a jour
Le menu reprenait le titre entier des sections et s'empilait sur trois
lignes. Selflow et Comptaflow menent a leur site. Pastille et bouton du haut
de page lisibles. Plan, journal, classeur et passation : lots 71 a 73, et les
reponses du proprietaire (timbre non rembourse, commande B2B directe).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -1273,10 +1273,10 @@
         <v>148</v>
       </c>
       <c r="C25" s="15" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D25" s="15" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E25" s="15" t="n">
         <v>2</v>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="H25" s="18" t="inlineStr">
         <is>
-          <t>9/12</t>
+          <t>15/18</t>
         </is>
       </c>
     </row>
@@ -1300,10 +1300,10 @@
         </is>
       </c>
       <c r="C26" s="10" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="E26" s="10" t="n">
         <v>7</v>
@@ -1326,7 +1326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6103,18 +6103,20 @@
       </c>
       <c r="D158" s="14" t="inlineStr">
         <is>
-          <t>Aujourd'hui non : il reste dû à l'État (la plateforme ne le porte sur aucun avoir). Si l'entreprise le rend, il devient une charge (646).</t>
-        </is>
-      </c>
-      <c r="E158" s="18" t="inlineStr">
-        <is>
-          <t>À trancher</t>
+          <t>Tranché le 14/10 : non. Le timbre reste dû à l'État (la plateforme ne le porte sur aucun avoir).</t>
+        </is>
+      </c>
+      <c r="E158" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F158" s="22" t="n">
         <v>46309</v>
       </c>
-      <c r="G158" s="22" t="n"/>
+      <c r="G158" s="22" t="n">
+        <v>46309</v>
+      </c>
       <c r="H158" s="15" t="inlineStr">
         <is>
           <t>Jour 5</t>
@@ -6139,7 +6141,7 @@
       </c>
       <c r="D159" s="14" t="inlineStr">
         <is>
-          <t>Faisable sans toucher au périmètre gelé : 70a fil de discussion, 70b commander et confirmer (BC confirmé — en attente de livraison), 70c livrer, facturer, réceptionner, 70d notifications. Défauts de l'existant relevés. À valider.</t>
+          <t>Faisable sans toucher au périmètre gelé : 70a fil de discussion, 70b commander et confirmer (BC confirmé — en attente de livraison), 70c livrer, facturer, réceptionner, 70d notifications. Défauts de l'existant relevés. Validé le 14/10 ; commande directe sans demande de prix autorisée. À programmer.</t>
         </is>
       </c>
       <c r="E159" s="18" t="inlineStr">
@@ -6175,19 +6177,245 @@
       </c>
       <c r="D160" s="14" t="inlineStr">
         <is>
-          <t>Document annoncé, non parvenu dans la session du 14/10. À traiter à réception.</t>
-        </is>
-      </c>
-      <c r="E160" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
+          <t>Reçu le 14/10 (dix images) : traité aux lots 71 à 73 (voir 21.13 à 21.18).</t>
+        </is>
+      </c>
+      <c r="E160" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F160" s="22" t="n">
         <v>46309</v>
       </c>
-      <c r="G160" s="22" t="n"/>
+      <c r="G160" s="22" t="n">
+        <v>46309</v>
+      </c>
       <c r="H160" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="14" t="inlineStr">
+        <is>
+          <t>Articles</t>
+        </is>
+      </c>
+      <c r="B161" s="15" t="inlineStr">
+        <is>
+          <t>21.13</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>Erreur 500 en ligne à la création d'un article</t>
+        </is>
+      </c>
+      <c r="D161" s="14" t="inlineStr">
+        <is>
+          <t>Catégorie « nouvelle » sans nom : la chaîne partait en base, MySQL la refusait. Catégorie et sous-catégorie validées (lot 71).</t>
+        </is>
+      </c>
+      <c r="E161" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F161" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G161" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H161" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="14" t="inlineStr">
+        <is>
+          <t>Connexion</t>
+        </is>
+      </c>
+      <c r="B162" s="15" t="inlineStr">
+        <is>
+          <t>21.14</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>Mot de passe : page 429, règles de saisie</t>
+        </is>
+      </c>
+      <c r="D162" s="14" t="inlineStr">
+        <is>
+          <t>Borne par adresse saisie, page lisible ; liste des règles cochée en direct (lot 71).</t>
+        </is>
+      </c>
+      <c r="E162" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F162" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G162" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H162" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="14" t="inlineStr">
+        <is>
+          <t>Écrans</t>
+        </is>
+      </c>
+      <c r="B163" s="15" t="inlineStr">
+        <is>
+          <t>21.15</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>Recherches et import du stock d'ouverture</t>
+        </is>
+      </c>
+      <c r="D163" s="14" t="inlineStr">
+        <is>
+          <t>Plus de rechargement à chaque frappe (dix écrans) ; modèle d'inventaire rempli des articles de l'entreprise (lot 71).</t>
+        </is>
+      </c>
+      <c r="E163" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F163" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G163" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H163" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="14" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="B164" s="15" t="inlineStr">
+        <is>
+          <t>21.16</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Modifier et supprimer les comptes créés</t>
+        </is>
+      </c>
+      <c r="D164" s="14" t="inlineStr">
+        <is>
+          <t>Seulement les comptes créés par l'entreprise ; un compte employé garde son numéro et ne se supprime pas (lot 72).</t>
+        </is>
+      </c>
+      <c r="E164" s="16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F164" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G164" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H164" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="14" t="inlineStr">
+        <is>
+          <t>FNE</t>
+        </is>
+      </c>
+      <c r="B165" s="15" t="inlineStr">
+        <is>
+          <t>21.17</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>Gestion FNE : d'où viennent les chiffres</t>
+        </is>
+      </c>
+      <c r="D165" s="14" t="inlineStr">
+        <is>
+          <t>Timbre, solde et stickers ne viennent que des certifications : la page le dit ; proformas « non transmis ». Défaut d'affichage des sous-modules à préciser (lot 72).</t>
+        </is>
+      </c>
+      <c r="E165" s="18" t="inlineStr">
+        <is>
+          <t>À trancher</t>
+        </is>
+      </c>
+      <c r="F165" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G165" s="22" t="n"/>
+      <c r="H165" s="15" t="inlineStr">
+        <is>
+          <t>Jour 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="14" t="inlineStr">
+        <is>
+          <t>Vitrine</t>
+        </is>
+      </c>
+      <c r="B166" s="15" t="inlineStr">
+        <is>
+          <t>21.18</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>Page d'accueil</t>
+        </is>
+      </c>
+      <c r="D166" s="14" t="inlineStr">
+        <is>
+          <t>Menu court, liens Selflow et Comptaflow, contraste du haut de page (lot 73). Attendus : textes et adresses de RHFlow, LegalFlow, Agent-AI, CGA-Connect ; section « Le cabinet » à compléter ou masquer.</t>
+        </is>
+      </c>
+      <c r="E166" s="18" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F166" s="22" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G166" s="22" t="n"/>
+      <c r="H166" s="15" t="inlineStr">
         <is>
           <t>Jour 5</t>
         </is>

</xml_diff>

<commit_message>
Pas a pas : l'etape 1 en liste avec une barre en bas ; retour arriere du parcours ; plan des retours a part
Etape 1 refaite : une ligne par article avec compteur, plus de panier lateral,
barre fixe (articles, net a payer, suite). Le bouton Retour du navigateur
restaurait le drapeau 'deja envoye' du parcours : efface a l'affichage.
PLAN-RETOURS-PRODUCTION.xlsx, meme modele que le plan de correction, qui
retrouve son etat du 09/10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016FDQ3AChyqrpZ6HWR6zrEi
</commit_message>
<xml_diff>
--- a/PLAN-CORRECTION-SELFLOW.xlsx
+++ b/PLAN-CORRECTION-SELFLOW.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -620,7 +620,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1264,54 +1263,24 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>21. RETOURS DE LA MISE EN PRODUCTION — 14/10/2026</t>
-        </is>
-      </c>
-      <c r="B25" s="15" t="n">
-        <v>148</v>
-      </c>
-      <c r="C25" s="15" t="n">
-        <v>18</v>
-      </c>
-      <c r="D25" s="15" t="n">
-        <v>15</v>
-      </c>
-      <c r="E25" s="15" t="n">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>107</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F25" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="18" t="inlineStr">
-        <is>
-          <t>15/18</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="n">
-        <v>125</v>
-      </c>
-      <c r="D26" s="10" t="n">
-        <v>107</v>
-      </c>
-      <c r="E26" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="F26" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="G26" s="10" t="n">
+      <c r="G25" s="10" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1326,7 +1295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H166"/>
+  <dimension ref="A1:H146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5729,702 +5698,9 @@
         </is>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" s="23" t="inlineStr">
-        <is>
-          <t>21. RETOURS DE LA MISE EN PRODUCTION — 14/10/2026</t>
-        </is>
-      </c>
-      <c r="B148" s="21" t="n"/>
-      <c r="C148" s="21" t="n"/>
-      <c r="D148" s="21" t="n"/>
-      <c r="E148" s="21" t="n"/>
-      <c r="F148" s="21" t="n"/>
-      <c r="G148" s="21" t="n"/>
-      <c r="H148" s="21" t="n"/>
-    </row>
-    <row r="149">
-      <c r="A149" s="14" t="inlineStr">
-        <is>
-          <t>Sécurité</t>
-        </is>
-      </c>
-      <c r="B149" s="15" t="inlineStr">
-        <is>
-          <t>21.1</t>
-        </is>
-      </c>
-      <c r="C149" s="5" t="inlineStr">
-        <is>
-          <t>Mot de passe oublié : le lien ne s'affiche plus, le courriel part</t>
-        </is>
-      </c>
-      <c r="D149" s="14" t="inlineStr">
-        <is>
-          <t>Faille : le lien de réinitialisation s'affichait à l'écran de quiconque tapait une adresse. Il ne part plus que par courriel ; serveur sans transport signalé ; jeton vérifié ; même réponse pour une adresse inconnue. Commande selflow:verifier-courriel (lot 64).</t>
-        </is>
-      </c>
-      <c r="E149" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F149" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G149" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H149" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="14" t="inlineStr">
-        <is>
-          <t>Courriels</t>
-        </is>
-      </c>
-      <c r="B150" s="15" t="inlineStr">
-        <is>
-          <t>21.2</t>
-        </is>
-      </c>
-      <c r="C150" s="5" t="inlineStr">
-        <is>
-          <t>Avis d'ouverture de compte</t>
-        </is>
-      </c>
-      <c r="D150" s="14" t="inlineStr">
-        <is>
-          <t>Inscription, employé, responsable créé par le superadmin, admin interne : le titulaire est prévenu, sans mot de passe (lot 64).</t>
-        </is>
-      </c>
-      <c r="E150" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F150" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G150" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H150" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="14" t="inlineStr">
-        <is>
-          <t>Ventes</t>
-        </is>
-      </c>
-      <c r="B151" s="15" t="inlineStr">
-        <is>
-          <t>21.3</t>
-        </is>
-      </c>
-      <c r="C151" s="5" t="inlineStr">
-        <is>
-          <t>La facture « ne passe pas », sans message</t>
-        </is>
-      </c>
-      <c r="D151" s="14" t="inlineStr">
-        <is>
-          <t>Refus de stock et de lot périmé perdus sous la clé error : affichés. Message de 3 s nommant la pièce, panier vidé (lot 65).</t>
-        </is>
-      </c>
-      <c r="E151" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F151" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G151" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H151" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="14" t="inlineStr">
-        <is>
-          <t>Écrans</t>
-        </is>
-      </c>
-      <c r="B152" s="15" t="inlineStr">
-        <is>
-          <t>21.4</t>
-        </is>
-      </c>
-      <c r="C152" s="5" t="inlineStr">
-        <is>
-          <t>Recherche du catalogue, avatar, fusée, domaine en un clic</t>
-        </is>
-      </c>
-      <c r="D152" s="14" t="inlineStr">
-        <is>
-          <t>Recherche sur tout le catalogue ; initiales si la photo manque ; fusée retirée ; le clic sur le domaine mène à l'étape suivante (lot 65).</t>
-        </is>
-      </c>
-      <c r="E152" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F152" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G152" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H152" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="14" t="inlineStr">
-        <is>
-          <t>Comptabilité</t>
-        </is>
-      </c>
-      <c r="B153" s="15" t="inlineStr">
-        <is>
-          <t>21.5</t>
-        </is>
-      </c>
-      <c r="C153" s="5" t="inlineStr">
-        <is>
-          <t>L'avoir, écriture d'origine en négatif</t>
-        </is>
-      </c>
-      <c r="D153" s="14" t="inlineStr">
-        <is>
-          <t>Taxes parafiscales contre-passées, remboursement en espèces écrit (411/caisse), retour au coût de sortie. Le timbre reste dû (lot 67).</t>
-        </is>
-      </c>
-      <c r="E153" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F153" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G153" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H153" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="14" t="inlineStr">
-        <is>
-          <t>Achats</t>
-        </is>
-      </c>
-      <c r="B154" s="15" t="inlineStr">
-        <is>
-          <t>21.6</t>
-        </is>
-      </c>
-      <c r="C154" s="5" t="inlineStr">
-        <is>
-          <t>Un geste par étape, actions dans la liste</t>
-        </is>
-      </c>
-      <c r="D154" s="14" t="inlineStr">
-        <is>
-          <t>DP : confirmer la commande ; BC : bon de réception et facturer. Achat B2B « Bon de commande » (lot 66).</t>
-        </is>
-      </c>
-      <c r="E154" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F154" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G154" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H154" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="14" t="inlineStr">
-        <is>
-          <t>Achats</t>
-        </is>
-      </c>
-      <c r="B155" s="15" t="inlineStr">
-        <is>
-          <t>21.7</t>
-        </is>
-      </c>
-      <c r="C155" s="5" t="inlineStr">
-        <is>
-          <t>Facture déclarée par le fournisseur</t>
-        </is>
-      </c>
-      <c r="D155" s="14" t="inlineStr">
-        <is>
-          <t>Question à la facturation : oui → saisie informative, la facture reçue de la DGI porte l'écriture ; non → écriture comme avant (lot 66).</t>
-        </is>
-      </c>
-      <c r="E155" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F155" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G155" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H155" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="14" t="inlineStr">
-        <is>
-          <t>Stickers</t>
-        </is>
-      </c>
-      <c r="B156" s="15" t="inlineStr">
-        <is>
-          <t>21.8</t>
-        </is>
-      </c>
-      <c r="C156" s="5" t="inlineStr">
-        <is>
-          <t>Achat des stickers confié à DC-Knowing</t>
-        </is>
-      </c>
-      <c r="D156" s="14" t="inlineStr">
-        <is>
-          <t>Demande (quantité, site, urgence) gardée, courriel à DC-Knowing et accusé au demandeur, page superadmin avec statut (lot 68).</t>
-        </is>
-      </c>
-      <c r="E156" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F156" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G156" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H156" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="14" t="inlineStr">
-        <is>
-          <t>Ventes</t>
-        </is>
-      </c>
-      <c r="B157" s="15" t="inlineStr">
-        <is>
-          <t>21.9</t>
-        </is>
-      </c>
-      <c r="C157" s="5" t="inlineStr">
-        <is>
-          <t>Vente pas à pas</t>
-        </is>
-      </c>
-      <c r="D157" s="14" t="inlineStr">
-        <is>
-          <t>Bascule Caisse / Pas à pas : articles, client et document, règlement, valider et facturer. Même formulaire (lot 69). Vérifiée dans Chromium.</t>
-        </is>
-      </c>
-      <c r="E157" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F157" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G157" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H157" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="14" t="inlineStr">
-        <is>
-          <t>Comptabilité</t>
-        </is>
-      </c>
-      <c r="B158" s="15" t="inlineStr">
-        <is>
-          <t>21.10</t>
-        </is>
-      </c>
-      <c r="C158" s="5" t="inlineStr">
-        <is>
-          <t>Le timbre d'une facture annulée est-il remboursé au client ?</t>
-        </is>
-      </c>
-      <c r="D158" s="14" t="inlineStr">
-        <is>
-          <t>Tranché le 14/10 : non. Le timbre reste dû à l'État (la plateforme ne le porte sur aucun avoir).</t>
-        </is>
-      </c>
-      <c r="E158" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F158" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G158" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H158" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="14" t="inlineStr">
-        <is>
-          <t>B2B</t>
-        </is>
-      </c>
-      <c r="B159" s="15" t="inlineStr">
-        <is>
-          <t>21.11</t>
-        </is>
-      </c>
-      <c r="C159" s="5" t="inlineStr">
-        <is>
-          <t>Communication B2B approfondie</t>
-        </is>
-      </c>
-      <c r="D159" s="14" t="inlineStr">
-        <is>
-          <t>Faisable sans toucher au périmètre gelé : 70a fil de discussion, 70b commander et confirmer (BC confirmé — en attente de livraison), 70c livrer, facturer, réceptionner, 70d notifications. Défauts de l'existant relevés. Validé le 14/10 ; commande directe sans demande de prix autorisée. À programmer.</t>
-        </is>
-      </c>
-      <c r="E159" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F159" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G159" s="22" t="n"/>
-      <c r="H159" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="14" t="inlineStr">
-        <is>
-          <t>Retours</t>
-        </is>
-      </c>
-      <c r="B160" s="15" t="inlineStr">
-        <is>
-          <t>21.12</t>
-        </is>
-      </c>
-      <c r="C160" s="5" t="inlineStr">
-        <is>
-          <t>« Des corrections à revoir pour Selflow.docx »</t>
-        </is>
-      </c>
-      <c r="D160" s="14" t="inlineStr">
-        <is>
-          <t>Reçu le 14/10 (dix images) : traité aux lots 71 à 73 (voir 21.13 à 21.18).</t>
-        </is>
-      </c>
-      <c r="E160" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F160" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G160" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H160" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="14" t="inlineStr">
-        <is>
-          <t>Articles</t>
-        </is>
-      </c>
-      <c r="B161" s="15" t="inlineStr">
-        <is>
-          <t>21.13</t>
-        </is>
-      </c>
-      <c r="C161" s="5" t="inlineStr">
-        <is>
-          <t>Erreur 500 en ligne à la création d'un article</t>
-        </is>
-      </c>
-      <c r="D161" s="14" t="inlineStr">
-        <is>
-          <t>Catégorie « nouvelle » sans nom : la chaîne partait en base, MySQL la refusait. Catégorie et sous-catégorie validées (lot 71).</t>
-        </is>
-      </c>
-      <c r="E161" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F161" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G161" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H161" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="14" t="inlineStr">
-        <is>
-          <t>Connexion</t>
-        </is>
-      </c>
-      <c r="B162" s="15" t="inlineStr">
-        <is>
-          <t>21.14</t>
-        </is>
-      </c>
-      <c r="C162" s="5" t="inlineStr">
-        <is>
-          <t>Mot de passe : page 429, règles de saisie</t>
-        </is>
-      </c>
-      <c r="D162" s="14" t="inlineStr">
-        <is>
-          <t>Borne par adresse saisie, page lisible ; liste des règles cochée en direct (lot 71).</t>
-        </is>
-      </c>
-      <c r="E162" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F162" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G162" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H162" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="14" t="inlineStr">
-        <is>
-          <t>Écrans</t>
-        </is>
-      </c>
-      <c r="B163" s="15" t="inlineStr">
-        <is>
-          <t>21.15</t>
-        </is>
-      </c>
-      <c r="C163" s="5" t="inlineStr">
-        <is>
-          <t>Recherches et import du stock d'ouverture</t>
-        </is>
-      </c>
-      <c r="D163" s="14" t="inlineStr">
-        <is>
-          <t>Plus de rechargement à chaque frappe (dix écrans) ; modèle d'inventaire rempli des articles de l'entreprise (lot 71).</t>
-        </is>
-      </c>
-      <c r="E163" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F163" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G163" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H163" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="14" t="inlineStr">
-        <is>
-          <t>Comptabilité</t>
-        </is>
-      </c>
-      <c r="B164" s="15" t="inlineStr">
-        <is>
-          <t>21.16</t>
-        </is>
-      </c>
-      <c r="C164" s="5" t="inlineStr">
-        <is>
-          <t>Modifier et supprimer les comptes créés</t>
-        </is>
-      </c>
-      <c r="D164" s="14" t="inlineStr">
-        <is>
-          <t>Seulement les comptes créés par l'entreprise ; un compte employé garde son numéro et ne se supprime pas (lot 72).</t>
-        </is>
-      </c>
-      <c r="E164" s="16" t="inlineStr">
-        <is>
-          <t>Terminé</t>
-        </is>
-      </c>
-      <c r="F164" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G164" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="H164" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="14" t="inlineStr">
-        <is>
-          <t>FNE</t>
-        </is>
-      </c>
-      <c r="B165" s="15" t="inlineStr">
-        <is>
-          <t>21.17</t>
-        </is>
-      </c>
-      <c r="C165" s="5" t="inlineStr">
-        <is>
-          <t>Gestion FNE : d'où viennent les chiffres</t>
-        </is>
-      </c>
-      <c r="D165" s="14" t="inlineStr">
-        <is>
-          <t>Timbre, solde et stickers ne viennent que des certifications : la page le dit ; proformas « non transmis ». Défaut d'affichage des sous-modules à préciser (lot 72).</t>
-        </is>
-      </c>
-      <c r="E165" s="18" t="inlineStr">
-        <is>
-          <t>À trancher</t>
-        </is>
-      </c>
-      <c r="F165" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G165" s="22" t="n"/>
-      <c r="H165" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="14" t="inlineStr">
-        <is>
-          <t>Vitrine</t>
-        </is>
-      </c>
-      <c r="B166" s="15" t="inlineStr">
-        <is>
-          <t>21.18</t>
-        </is>
-      </c>
-      <c r="C166" s="5" t="inlineStr">
-        <is>
-          <t>Page d'accueil</t>
-        </is>
-      </c>
-      <c r="D166" s="14" t="inlineStr">
-        <is>
-          <t>Menu court, liens Selflow et Comptaflow, contraste du haut de page (lot 73). Attendus : textes et adresses de RHFlow, LegalFlow, Agent-AI, CGA-Connect ; section « Le cabinet » à compléter ou masquer.</t>
-        </is>
-      </c>
-      <c r="E166" s="18" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="F166" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G166" s="22" t="n"/>
-      <c r="H166" s="15" t="inlineStr">
-        <is>
-          <t>Jour 5</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A4:H116"/>
-  <mergeCells count="20">
-    <mergeCell ref="A148:H148"/>
+  <mergeCells count="19">
     <mergeCell ref="A64:H64"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A45:H45"/>

</xml_diff>